<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-26 18:20 UTC
</commit_message>
<xml_diff>
--- a/data/50001545 - XEMORTIZ MINERA FRISCO.xlsx
+++ b/data/50001545 - XEMORTIZ MINERA FRISCO.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1608" uniqueCount="373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1608" uniqueCount="374">
   <si>
     <t>50001545 - XEMORTIZ MINERA FRISCO</t>
   </si>
@@ -613,6 +613,9 @@
   </si>
   <si>
     <t>check planos,Ingenieria y diseñoo:</t>
+  </si>
+  <si>
+    <t>Tarea en curso</t>
   </si>
   <si>
     <t>1214596734094526</t>
@@ -3338,7 +3341,7 @@
       </c>
       <c r="C29" s="10"/>
       <c r="D29" s="9">
-        <v>46197.20554309028</v>
+        <v>46199.75288726852</v>
       </c>
       <c r="E29" s="10" t="s">
         <v>116</v>
@@ -3399,9 +3402,11 @@
       <c r="B30" s="5">
         <v>46149.168830532406</v>
       </c>
-      <c r="C30" s="6"/>
+      <c r="C30" s="5">
+        <v>46199.752829537036</v>
+      </c>
       <c r="D30" s="5">
-        <v>46198.80594373842</v>
+        <v>46199.75283171296</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>119</v>
@@ -3460,7 +3465,7 @@
       </c>
       <c r="C31" s="10"/>
       <c r="D31" s="9">
-        <v>46196.16862795139</v>
+        <v>46199.752836423606</v>
       </c>
       <c r="E31" s="10" t="s">
         <v>122</v>
@@ -3517,9 +3522,11 @@
       <c r="B32" s="5">
         <v>46149.16884</v>
       </c>
-      <c r="C32" s="6"/>
+      <c r="C32" s="5">
+        <v>46199.75287768518</v>
+      </c>
       <c r="D32" s="5">
-        <v>46185.52448216435</v>
+        <v>46199.752879155094</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>125</v>
@@ -4431,7 +4438,7 @@
       </c>
       <c r="C48" s="6"/>
       <c r="D48" s="5">
-        <v>46197.71372509259</v>
+        <v>46199.752894212965</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>178</v>
@@ -4481,13 +4488,13 @@
       <c r="T48" s="6">
         <v>0</v>
       </c>
-      <c r="U48" s="11" t="s">
-        <v>81</v>
+      <c r="U48" s="12" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" s="8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B49" s="9">
         <v>46149.16897216435</v>
@@ -4503,10 +4510,10 @@
         <v>26</v>
       </c>
       <c r="G49" s="10" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="H49" s="10" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="I49" s="10"/>
       <c r="J49" s="9">
@@ -4528,7 +4535,7 @@
         <v>178</v>
       </c>
       <c r="P49" s="10" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="Q49" s="9">
         <v>46184</v>
@@ -4548,7 +4555,7 @@
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B50" s="5">
         <v>46149.16898688657</v>
@@ -4558,16 +4565,16 @@
         <v>46155.59844700231</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F50" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G50" s="6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="I50" s="5">
         <v>46241</v>
@@ -4588,7 +4595,7 @@
         <v>170</v>
       </c>
       <c r="O50" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="P50" s="6" t="s">
         <v>26</v>
@@ -4611,7 +4618,7 @@
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" s="8" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B51" s="9">
         <v>46149.168991412036</v>
@@ -4621,7 +4628,7 @@
         <v>46155.59855652778</v>
       </c>
       <c r="E51" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F51" s="10" t="s">
         <v>26</v>
@@ -4646,13 +4653,13 @@
         <v>26</v>
       </c>
       <c r="N51" s="10" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="O51" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P51" s="10" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="Q51" s="10"/>
       <c r="R51" s="10"/>
@@ -4662,7 +4669,7 @@
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B52" s="5">
         <v>46149.16900017361</v>
@@ -4672,7 +4679,7 @@
         <v>46155.59855292824</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F52" s="6" t="s">
         <v>26</v>
@@ -4697,13 +4704,13 @@
         <v>26</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="O52" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P52" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="Q52" s="6"/>
       <c r="R52" s="6"/>
@@ -4713,7 +4720,7 @@
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B53" s="9">
         <v>46155.577817384255</v>
@@ -4723,7 +4730,7 @@
         <v>46155.59854846065</v>
       </c>
       <c r="E53" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F53" s="10" t="s">
         <v>26</v>
@@ -4748,13 +4755,13 @@
         <v>26</v>
       </c>
       <c r="N53" s="10" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="O53" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P53" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="Q53" s="10"/>
       <c r="R53" s="10"/>
@@ -4764,7 +4771,7 @@
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B54" s="5">
         <v>46155.577829050926</v>
@@ -4774,7 +4781,7 @@
         <v>46155.59854489584</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F54" s="6" t="s">
         <v>26</v>
@@ -4799,13 +4806,13 @@
         <v>26</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="O54" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P54" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="Q54" s="6"/>
       <c r="R54" s="6"/>
@@ -4815,7 +4822,7 @@
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" s="8" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B55" s="9">
         <v>46149.1690050926</v>
@@ -4825,7 +4832,7 @@
         <v>46155.55893427083</v>
       </c>
       <c r="E55" s="10" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F55" s="10" t="s">
         <v>25</v>
@@ -4849,7 +4856,7 @@
         <v>26</v>
       </c>
       <c r="O55" s="10" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="P55" s="10" t="s">
         <v>26</v>
@@ -4862,7 +4869,7 @@
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B56" s="5">
         <v>46149.16900940972</v>
@@ -4872,16 +4879,16 @@
         <v>46196.2065696412</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F56" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G56" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I56" s="5">
         <v>46202</v>
@@ -4899,13 +4906,13 @@
         <v>26</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="O56" s="6" t="s">
         <v>137</v>
       </c>
       <c r="P56" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="Q56" s="5">
         <v>46202</v>
@@ -4925,7 +4932,7 @@
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A57" s="8" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B57" s="9">
         <v>46149.16901516204</v>
@@ -4935,7 +4942,7 @@
         <v>46176.17164681713</v>
       </c>
       <c r="E57" s="10" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F57" s="10" t="s">
         <v>26</v>
@@ -4962,13 +4969,13 @@
         <v>26</v>
       </c>
       <c r="N57" s="10" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="O57" s="10" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="P57" s="10" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="Q57" s="9">
         <v>46174</v>
@@ -4988,7 +4995,7 @@
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B58" s="5">
         <v>46149.16902107639</v>
@@ -4998,16 +5005,16 @@
         <v>46196.20656958333</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G58" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I58" s="5">
         <v>46202</v>
@@ -5025,13 +5032,13 @@
         <v>26</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="O58" s="6" t="s">
         <v>145</v>
       </c>
       <c r="P58" s="6" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="Q58" s="5">
         <v>46202</v>
@@ -5051,7 +5058,7 @@
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A59" s="8" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B59" s="9">
         <v>46149.16902621528</v>
@@ -5061,7 +5068,7 @@
         <v>46176.17164685186</v>
       </c>
       <c r="E59" s="10" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F59" s="10" t="s">
         <v>26</v>
@@ -5088,13 +5095,13 @@
         <v>26</v>
       </c>
       <c r="N59" s="10" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="O59" s="10" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="P59" s="10" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="Q59" s="9">
         <v>46174</v>
@@ -5114,7 +5121,7 @@
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B60" s="5">
         <v>46149.1690303588</v>
@@ -5124,16 +5131,16 @@
         <v>46155.59866159722</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F60" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G60" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I60" s="5">
         <v>46211</v>
@@ -5151,13 +5158,13 @@
         <v>26</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="O60" s="6" t="s">
         <v>167</v>
       </c>
       <c r="P60" s="6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="Q60" s="5">
         <v>46211</v>
@@ -5177,7 +5184,7 @@
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A61" s="8" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B61" s="9">
         <v>46149.16903488426</v>
@@ -5187,7 +5194,7 @@
         <v>46155.5990459375</v>
       </c>
       <c r="E61" s="10" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F61" s="10" t="s">
         <v>26</v>
@@ -5214,13 +5221,13 @@
         <v>26</v>
       </c>
       <c r="N61" s="10" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="O61" s="10" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="P61" s="10" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="Q61" s="9">
         <v>46213</v>
@@ -5240,7 +5247,7 @@
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B62" s="5">
         <v>46149.1690391088</v>
@@ -5250,7 +5257,7 @@
         <v>46155.56887822917</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F62" s="6" t="s">
         <v>25</v>
@@ -5274,7 +5281,7 @@
         <v>26</v>
       </c>
       <c r="O62" s="6" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="P62" s="6" t="s">
         <v>26</v>
@@ -5287,7 +5294,7 @@
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A63" s="8" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B63" s="9">
         <v>46149.169042442125</v>
@@ -5297,16 +5304,16 @@
         <v>46161.57724337963</v>
       </c>
       <c r="E63" s="10" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="F63" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G63" s="10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H63" s="10" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="I63" s="9">
         <v>46217</v>
@@ -5324,13 +5331,13 @@
         <v>26</v>
       </c>
       <c r="N63" s="10" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="O63" s="10" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="P63" s="10" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="Q63" s="9">
         <v>46217</v>
@@ -5350,7 +5357,7 @@
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B64" s="5">
         <v>46149.169049375</v>
@@ -5360,16 +5367,16 @@
         <v>46155.59925321759</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F64" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G64" s="6" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="I64" s="5">
         <v>46217</v>
@@ -5387,13 +5394,13 @@
         <v>26</v>
       </c>
       <c r="N64" s="6" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="O64" s="6" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="P64" s="6" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="Q64" s="6"/>
       <c r="R64" s="6"/>
@@ -5403,7 +5410,7 @@
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A65" s="8" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B65" s="9">
         <v>46149.16905616898</v>
@@ -5413,16 +5420,16 @@
         <v>46155.59924960649</v>
       </c>
       <c r="E65" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F65" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G65" s="10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H65" s="10" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="I65" s="9">
         <v>46217</v>
@@ -5440,13 +5447,13 @@
         <v>26</v>
       </c>
       <c r="N65" s="10" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="O65" s="10" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="P65" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="Q65" s="10"/>
       <c r="R65" s="10"/>
@@ -5456,7 +5463,7 @@
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B66" s="5">
         <v>46155.562074166664</v>
@@ -5466,16 +5473,16 @@
         <v>46155.59924675926</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F66" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G66" s="6" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H66" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="I66" s="5">
         <v>46217</v>
@@ -5493,13 +5500,13 @@
         <v>26</v>
       </c>
       <c r="N66" s="6" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="O66" s="6" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="P66" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="Q66" s="6"/>
       <c r="R66" s="6"/>
@@ -5509,7 +5516,7 @@
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A67" s="8" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B67" s="9">
         <v>46155.562095416666</v>
@@ -5519,16 +5526,16 @@
         <v>46155.59924362268</v>
       </c>
       <c r="E67" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F67" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G67" s="10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H67" s="10" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="I67" s="9">
         <v>46217</v>
@@ -5546,13 +5553,13 @@
         <v>26</v>
       </c>
       <c r="N67" s="10" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="O67" s="10" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="P67" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="Q67" s="10"/>
       <c r="R67" s="10"/>
@@ -5562,7 +5569,7 @@
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B68" s="5">
         <v>46149.169104699075</v>
@@ -5572,16 +5579,16 @@
         <v>46155.59934020833</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="F68" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G68" s="6" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="I68" s="5">
         <v>46220</v>
@@ -5599,13 +5606,13 @@
         <v>26</v>
       </c>
       <c r="N68" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="O68" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="P68" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="Q68" s="5">
         <v>46220</v>
@@ -5625,7 +5632,7 @@
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A69" s="8" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B69" s="9">
         <v>46149.1691096412</v>
@@ -5635,16 +5642,16 @@
         <v>46155.59950737268</v>
       </c>
       <c r="E69" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F69" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G69" s="10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H69" s="10" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="I69" s="9">
         <v>46220</v>
@@ -5662,13 +5669,13 @@
         <v>26</v>
       </c>
       <c r="N69" s="10" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="O69" s="10" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="P69" s="10" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="Q69" s="10"/>
       <c r="R69" s="10"/>
@@ -5678,7 +5685,7 @@
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B70" s="5">
         <v>46149.16911491899</v>
@@ -5688,16 +5695,16 @@
         <v>46155.59950449074</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F70" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G70" s="6" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H70" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="I70" s="5">
         <v>46220</v>
@@ -5715,13 +5722,13 @@
         <v>26</v>
       </c>
       <c r="N70" s="6" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="O70" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="P70" s="6" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="Q70" s="6"/>
       <c r="R70" s="6"/>
@@ -5731,7 +5738,7 @@
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71" s="8" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B71" s="9">
         <v>46155.562225625</v>
@@ -5741,16 +5748,16 @@
         <v>46155.5995016088</v>
       </c>
       <c r="E71" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F71" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G71" s="10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H71" s="10" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="I71" s="9">
         <v>46220</v>
@@ -5768,13 +5775,13 @@
         <v>26</v>
       </c>
       <c r="N71" s="10" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="O71" s="10" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="P71" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="Q71" s="10"/>
       <c r="R71" s="10"/>
@@ -5784,7 +5791,7 @@
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B72" s="5">
         <v>46155.56224557871</v>
@@ -5794,16 +5801,16 @@
         <v>46155.59949699074</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F72" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G72" s="6" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="I72" s="5">
         <v>46220</v>
@@ -5821,13 +5828,13 @@
         <v>26</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="O72" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="P72" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="Q72" s="6"/>
       <c r="R72" s="6"/>
@@ -5837,7 +5844,7 @@
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A73" s="8" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B73" s="9">
         <v>46149.169119768514</v>
@@ -5847,7 +5854,7 @@
         <v>46155.59937984953</v>
       </c>
       <c r="E73" s="10" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="F73" s="10" t="s">
         <v>26</v>
@@ -5874,13 +5881,13 @@
         <v>26</v>
       </c>
       <c r="N73" s="10" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="O73" s="10" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="P73" s="10" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="Q73" s="9">
         <v>46227</v>
@@ -5900,7 +5907,7 @@
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B74" s="5">
         <v>46149.16912365741</v>
@@ -5910,7 +5917,7 @@
         <v>46155.59963545139</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F74" s="6" t="s">
         <v>26</v>
@@ -5937,13 +5944,13 @@
         <v>26</v>
       </c>
       <c r="N74" s="6" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="O74" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="P74" s="6" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="Q74" s="6"/>
       <c r="R74" s="6"/>
@@ -5953,7 +5960,7 @@
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A75" s="8" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B75" s="9">
         <v>46149.16912908565</v>
@@ -5963,7 +5970,7 @@
         <v>46155.59963275463</v>
       </c>
       <c r="E75" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F75" s="10" t="s">
         <v>26</v>
@@ -5990,13 +5997,13 @@
         <v>26</v>
       </c>
       <c r="N75" s="10" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="O75" s="10" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="P75" s="10" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="Q75" s="10"/>
       <c r="R75" s="10"/>
@@ -6006,7 +6013,7 @@
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B76" s="5">
         <v>46155.56233189815</v>
@@ -6016,7 +6023,7 @@
         <v>46155.59962995371</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F76" s="6" t="s">
         <v>26</v>
@@ -6043,13 +6050,13 @@
         <v>26</v>
       </c>
       <c r="N76" s="6" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="O76" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="P76" s="6" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="Q76" s="6"/>
       <c r="R76" s="6"/>
@@ -6059,7 +6066,7 @@
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77" s="8" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B77" s="9">
         <v>46155.562344351856</v>
@@ -6069,7 +6076,7 @@
         <v>46155.599625891206</v>
       </c>
       <c r="E77" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F77" s="10" t="s">
         <v>26</v>
@@ -6096,13 +6103,13 @@
         <v>26</v>
       </c>
       <c r="N77" s="10" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="O77" s="10" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="P77" s="10" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="Q77" s="10"/>
       <c r="R77" s="10"/>
@@ -6112,7 +6119,7 @@
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B78" s="5">
         <v>46149.16913412037</v>
@@ -6122,7 +6129,7 @@
         <v>46155.57120092593</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F78" s="6" t="s">
         <v>25</v>
@@ -6146,7 +6153,7 @@
         <v>26</v>
       </c>
       <c r="O78" s="6" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="P78" s="6" t="s">
         <v>26</v>
@@ -6159,7 +6166,7 @@
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" s="8" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B79" s="9">
         <v>46149.16913708333</v>
@@ -6169,16 +6176,16 @@
         <v>46182.17098876157</v>
       </c>
       <c r="E79" s="10" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F79" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G79" s="10" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H79" s="10" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I79" s="10"/>
       <c r="J79" s="9">
@@ -6194,13 +6201,13 @@
         <v>26</v>
       </c>
       <c r="N79" s="10" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="O79" s="10" t="s">
         <v>113</v>
       </c>
       <c r="P79" s="10" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="Q79" s="9">
         <v>46181</v>
@@ -6220,7 +6227,7 @@
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B80" s="5">
         <v>46149.16914224537</v>
@@ -6230,16 +6237,16 @@
         <v>46165.180999432865</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F80" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G80" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H80" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I80" s="5">
         <v>46164</v>
@@ -6257,13 +6264,13 @@
         <v>26</v>
       </c>
       <c r="N80" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="O80" s="6" t="s">
         <v>104</v>
       </c>
       <c r="P80" s="6" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="Q80" s="5">
         <v>46164</v>
@@ -6283,7 +6290,7 @@
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81" s="8" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B81" s="9">
         <v>46149.16914733796</v>
@@ -6293,16 +6300,16 @@
         <v>46198.171336064814</v>
       </c>
       <c r="E81" s="10" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="F81" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G81" s="10" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H81" s="10" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I81" s="9">
         <v>46197</v>
@@ -6320,13 +6327,13 @@
         <v>26</v>
       </c>
       <c r="N81" s="10" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="O81" s="10" t="s">
         <v>122</v>
       </c>
       <c r="P81" s="10" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="Q81" s="9">
         <v>46197</v>
@@ -6346,7 +6353,7 @@
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B82" s="5">
         <v>46149.16915236111</v>
@@ -6356,16 +6363,16 @@
         <v>46155.59985006944</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F82" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G82" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H82" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I82" s="5">
         <v>46231</v>
@@ -6383,13 +6390,13 @@
         <v>26</v>
       </c>
       <c r="N82" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="O82" s="6" t="s">
         <v>155</v>
       </c>
       <c r="P82" s="6" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="Q82" s="5">
         <v>46231</v>
@@ -6409,7 +6416,7 @@
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A83" s="8" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B83" s="9">
         <v>46149.16915732639</v>
@@ -6419,7 +6426,7 @@
         <v>46155.58270766203</v>
       </c>
       <c r="E83" s="10" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="F83" s="10" t="s">
         <v>25</v>
@@ -6443,7 +6450,7 @@
         <v>26</v>
       </c>
       <c r="O83" s="10" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="P83" s="10" t="s">
         <v>26</v>
@@ -6456,7 +6463,7 @@
     </row>
     <row r="84" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A84" s="4" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B84" s="5">
         <v>46149.16916049768</v>
@@ -6466,7 +6473,7 @@
         <v>46155.60047521991</v>
       </c>
       <c r="E84" s="6" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="F84" s="6" t="s">
         <v>26</v>
@@ -6493,13 +6500,13 @@
         <v>26</v>
       </c>
       <c r="N84" s="6" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="O84" s="6" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="P84" s="6" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="Q84" s="5">
         <v>46230</v>
@@ -6519,7 +6526,7 @@
     </row>
     <row r="85" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A85" s="8" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B85" s="9">
         <v>46149.16916685185</v>
@@ -6529,7 +6536,7 @@
         <v>46155.60002515046</v>
       </c>
       <c r="E85" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F85" s="10" t="s">
         <v>26</v>
@@ -6556,10 +6563,10 @@
         <v>26</v>
       </c>
       <c r="N85" s="10" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="O85" s="10" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="P85" s="10" t="s">
         <v>26</v>
@@ -6572,7 +6579,7 @@
     </row>
     <row r="86" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B86" s="5">
         <v>46149.16917037037</v>
@@ -6582,7 +6589,7 @@
         <v>46155.60002232638</v>
       </c>
       <c r="E86" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F86" s="6" t="s">
         <v>26</v>
@@ -6609,10 +6616,10 @@
         <v>26</v>
       </c>
       <c r="N86" s="6" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="O86" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="P86" s="6" t="s">
         <v>26</v>
@@ -6625,7 +6632,7 @@
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A87" s="8" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B87" s="9">
         <v>46155.5624656713</v>
@@ -6635,7 +6642,7 @@
         <v>46155.60026604167</v>
       </c>
       <c r="E87" s="10" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F87" s="10" t="s">
         <v>26</v>
@@ -6662,13 +6669,13 @@
         <v>26</v>
       </c>
       <c r="N87" s="10" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="O87" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P87" s="10" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="Q87" s="10"/>
       <c r="R87" s="10"/>
@@ -6678,7 +6685,7 @@
     </row>
     <row r="88" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B88" s="5">
         <v>46155.562495266204</v>
@@ -6688,7 +6695,7 @@
         <v>46155.600359212964</v>
       </c>
       <c r="E88" s="6" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F88" s="6" t="s">
         <v>26</v>
@@ -6715,13 +6722,13 @@
         <v>26</v>
       </c>
       <c r="N88" s="6" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="O88" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P88" s="6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="Q88" s="6"/>
       <c r="R88" s="6"/>
@@ -6731,7 +6738,7 @@
     </row>
     <row r="89" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A89" s="8" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B89" s="9">
         <v>46149.16917405093</v>
@@ -6741,7 +6748,7 @@
         <v>46155.600641770834</v>
       </c>
       <c r="E89" s="10" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="F89" s="10" t="s">
         <v>26</v>
@@ -6768,13 +6775,13 @@
         <v>26</v>
       </c>
       <c r="N89" s="10" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="O89" s="10" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="P89" s="10" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="Q89" s="9">
         <v>46237</v>
@@ -6794,7 +6801,7 @@
     </row>
     <row r="90" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A90" s="4" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B90" s="5">
         <v>46149.169178321754</v>
@@ -6804,7 +6811,7 @@
         <v>46155.600606238426</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F90" s="6" t="s">
         <v>26</v>
@@ -6829,13 +6836,13 @@
         <v>26</v>
       </c>
       <c r="N90" s="6" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="O90" s="6" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="P90" s="6" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="Q90" s="6"/>
       <c r="R90" s="6"/>
@@ -6845,7 +6852,7 @@
     </row>
     <row r="91" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A91" s="8" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B91" s="9">
         <v>46149.169183148144</v>
@@ -6855,7 +6862,7 @@
         <v>46155.60060333333</v>
       </c>
       <c r="E91" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F91" s="10" t="s">
         <v>26</v>
@@ -6880,13 +6887,13 @@
         <v>26</v>
       </c>
       <c r="N91" s="10" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="O91" s="10" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="P91" s="10" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="Q91" s="10"/>
       <c r="R91" s="10"/>
@@ -6896,7 +6903,7 @@
     </row>
     <row r="92" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A92" s="4" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B92" s="5">
         <v>46155.56256662037</v>
@@ -6906,7 +6913,7 @@
         <v>46155.600600254635</v>
       </c>
       <c r="E92" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F92" s="6" t="s">
         <v>26</v>
@@ -6931,13 +6938,13 @@
         <v>26</v>
       </c>
       <c r="N92" s="6" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="O92" s="6" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="P92" s="6" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="Q92" s="6"/>
       <c r="R92" s="6"/>
@@ -6947,7 +6954,7 @@
     </row>
     <row r="93" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A93" s="8" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B93" s="9">
         <v>46155.56257849537</v>
@@ -6957,7 +6964,7 @@
         <v>46155.60059528935</v>
       </c>
       <c r="E93" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F93" s="10" t="s">
         <v>26</v>
@@ -6982,13 +6989,13 @@
         <v>26</v>
       </c>
       <c r="N93" s="10" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="O93" s="10" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="P93" s="10" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="Q93" s="10"/>
       <c r="R93" s="10"/>
@@ -6998,7 +7005,7 @@
     </row>
     <row r="94" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A94" s="4" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B94" s="5">
         <v>46149.169187962965</v>
@@ -7008,7 +7015,7 @@
         <v>46155.60079344908</v>
       </c>
       <c r="E94" s="6" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F94" s="6" t="s">
         <v>26</v>
@@ -7035,13 +7042,13 @@
         <v>26</v>
       </c>
       <c r="N94" s="6" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="O94" s="6" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="P94" s="6" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="Q94" s="5">
         <v>46238</v>
@@ -7061,7 +7068,7 @@
     </row>
     <row r="95" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A95" s="8" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B95" s="9">
         <v>46149.1691919213</v>
@@ -7071,7 +7078,7 @@
         <v>46155.600763483795</v>
       </c>
       <c r="E95" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F95" s="10" t="s">
         <v>26</v>
@@ -7096,13 +7103,13 @@
         <v>26</v>
       </c>
       <c r="N95" s="10" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="O95" s="10" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="P95" s="10" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="Q95" s="10"/>
       <c r="R95" s="10"/>
@@ -7112,7 +7119,7 @@
     </row>
     <row r="96" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A96" s="4" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B96" s="5">
         <v>46149.16919760416</v>
@@ -7122,7 +7129,7 @@
         <v>46155.60076056713</v>
       </c>
       <c r="E96" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F96" s="6" t="s">
         <v>26</v>
@@ -7147,13 +7154,13 @@
         <v>26</v>
       </c>
       <c r="N96" s="6" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="O96" s="6" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="P96" s="6" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="Q96" s="6"/>
       <c r="R96" s="6"/>
@@ -7163,7 +7170,7 @@
     </row>
     <row r="97" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A97" s="8" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B97" s="9">
         <v>46155.562660428244</v>
@@ -7173,7 +7180,7 @@
         <v>46155.60075752315</v>
       </c>
       <c r="E97" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F97" s="10" t="s">
         <v>26</v>
@@ -7198,13 +7205,13 @@
         <v>26</v>
       </c>
       <c r="N97" s="10" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="O97" s="10" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="P97" s="10" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="Q97" s="10"/>
       <c r="R97" s="10"/>
@@ -7214,7 +7221,7 @@
     </row>
     <row r="98" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A98" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B98" s="5">
         <v>46155.56267193287</v>
@@ -7224,7 +7231,7 @@
         <v>46155.600753645835</v>
       </c>
       <c r="E98" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F98" s="6" t="s">
         <v>26</v>
@@ -7249,13 +7256,13 @@
         <v>26</v>
       </c>
       <c r="N98" s="6" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="O98" s="6" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="P98" s="6" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="Q98" s="6"/>
       <c r="R98" s="6"/>
@@ -7265,7 +7272,7 @@
     </row>
     <row r="99" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A99" s="8" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B99" s="9">
         <v>46149.169203125</v>
@@ -7275,7 +7282,7 @@
         <v>46155.60094263889</v>
       </c>
       <c r="E99" s="10" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="F99" s="10" t="s">
         <v>26</v>
@@ -7302,13 +7309,13 @@
         <v>26</v>
       </c>
       <c r="N99" s="10" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="O99" s="10" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="P99" s="10" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="Q99" s="9">
         <v>46239</v>
@@ -7328,7 +7335,7 @@
     </row>
     <row r="100" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A100" s="4" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B100" s="5">
         <v>46149.16920694444</v>
@@ -7338,7 +7345,7 @@
         <v>46155.600918067124</v>
       </c>
       <c r="E100" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F100" s="6" t="s">
         <v>26</v>
@@ -7363,13 +7370,13 @@
         <v>26</v>
       </c>
       <c r="N100" s="6" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="O100" s="6" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="P100" s="6" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="Q100" s="6"/>
       <c r="R100" s="6"/>
@@ -7379,7 +7386,7 @@
     </row>
     <row r="101" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A101" s="8" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B101" s="9">
         <v>46149.16921202546</v>
@@ -7389,7 +7396,7 @@
         <v>46155.60091518519</v>
       </c>
       <c r="E101" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F101" s="10" t="s">
         <v>26</v>
@@ -7414,13 +7421,13 @@
         <v>26</v>
       </c>
       <c r="N101" s="10" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="O101" s="10" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="P101" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="Q101" s="10"/>
       <c r="R101" s="10"/>
@@ -7430,7 +7437,7 @@
     </row>
     <row r="102" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A102" s="4" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B102" s="5">
         <v>46155.562741851856</v>
@@ -7440,7 +7447,7 @@
         <v>46155.60091216435</v>
       </c>
       <c r="E102" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F102" s="6" t="s">
         <v>26</v>
@@ -7465,13 +7472,13 @@
         <v>26</v>
       </c>
       <c r="N102" s="6" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="O102" s="6" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="P102" s="6" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="Q102" s="6"/>
       <c r="R102" s="6"/>
@@ -7481,7 +7488,7 @@
     </row>
     <row r="103" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A103" s="8" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B103" s="9">
         <v>46155.562755046296</v>
@@ -7491,7 +7498,7 @@
         <v>46155.60090780092</v>
       </c>
       <c r="E103" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F103" s="10" t="s">
         <v>26</v>
@@ -7516,13 +7523,13 @@
         <v>26</v>
       </c>
       <c r="N103" s="10" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="O103" s="10" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="P103" s="10" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="Q103" s="10"/>
       <c r="R103" s="10"/>
@@ -7532,7 +7539,7 @@
     </row>
     <row r="104" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A104" s="4" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B104" s="5">
         <v>46149.16921689815</v>
@@ -7542,7 +7549,7 @@
         <v>46155.60109780093</v>
       </c>
       <c r="E104" s="6" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="F104" s="6" t="s">
         <v>26</v>
@@ -7569,13 +7576,13 @@
         <v>26</v>
       </c>
       <c r="N104" s="6" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="O104" s="6" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="P104" s="6" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="Q104" s="5">
         <v>46240</v>
@@ -7595,7 +7602,7 @@
     </row>
     <row r="105" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A105" s="8" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B105" s="9">
         <v>46149.169220717595</v>
@@ -7605,7 +7612,7 @@
         <v>46155.60106565972</v>
       </c>
       <c r="E105" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F105" s="10" t="s">
         <v>26</v>
@@ -7632,13 +7639,13 @@
         <v>26</v>
       </c>
       <c r="N105" s="10" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="O105" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P105" s="10" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="Q105" s="10"/>
       <c r="R105" s="10"/>
@@ -7648,7 +7655,7 @@
     </row>
     <row r="106" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A106" s="4" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B106" s="5">
         <v>46149.16922577546</v>
@@ -7658,7 +7665,7 @@
         <v>46155.601062546295</v>
       </c>
       <c r="E106" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F106" s="6" t="s">
         <v>26</v>
@@ -7685,13 +7692,13 @@
         <v>26</v>
       </c>
       <c r="N106" s="6" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="O106" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P106" s="6" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="Q106" s="6"/>
       <c r="R106" s="6"/>
@@ -7701,7 +7708,7 @@
     </row>
     <row r="107" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A107" s="8" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B107" s="9">
         <v>46155.56285743056</v>
@@ -7711,7 +7718,7 @@
         <v>46155.60105936343</v>
       </c>
       <c r="E107" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F107" s="10" t="s">
         <v>26</v>
@@ -7738,13 +7745,13 @@
         <v>26</v>
       </c>
       <c r="N107" s="10" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="O107" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P107" s="10" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="Q107" s="10"/>
       <c r="R107" s="10"/>
@@ -7754,7 +7761,7 @@
     </row>
     <row r="108" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A108" s="4" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B108" s="5">
         <v>46155.56284611111</v>
@@ -7764,7 +7771,7 @@
         <v>46155.60105565972</v>
       </c>
       <c r="E108" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F108" s="6" t="s">
         <v>26</v>
@@ -7791,13 +7798,13 @@
         <v>26</v>
       </c>
       <c r="N108" s="6" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="O108" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P108" s="6" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="Q108" s="6"/>
       <c r="R108" s="6"/>
@@ -7807,7 +7814,7 @@
     </row>
     <row r="109" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A109" s="8" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B109" s="9">
         <v>46149.169270370374</v>
@@ -7817,7 +7824,7 @@
         <v>46155.601273506945</v>
       </c>
       <c r="E109" s="10" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="F109" s="10" t="s">
         <v>26</v>
@@ -7844,13 +7851,13 @@
         <v>26</v>
       </c>
       <c r="N109" s="10" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="O109" s="10" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="P109" s="10" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="Q109" s="9">
         <v>46244</v>
@@ -7870,7 +7877,7 @@
     </row>
     <row r="110" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A110" s="4" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B110" s="5">
         <v>46149.16928524306</v>
@@ -7880,7 +7887,7 @@
         <v>46155.60133046296</v>
       </c>
       <c r="E110" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F110" s="6" t="s">
         <v>26</v>
@@ -7905,13 +7912,13 @@
         <v>26</v>
       </c>
       <c r="N110" s="6" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="O110" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P110" s="6" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="Q110" s="6"/>
       <c r="R110" s="6"/>
@@ -7921,7 +7928,7 @@
     </row>
     <row r="111" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A111" s="8" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B111" s="9">
         <v>46149.16929128472</v>
@@ -7931,7 +7938,7 @@
         <v>46155.60132649305</v>
       </c>
       <c r="E111" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F111" s="10" t="s">
         <v>26</v>
@@ -7956,13 +7963,13 @@
         <v>26</v>
       </c>
       <c r="N111" s="10" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="O111" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P111" s="10" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="Q111" s="10"/>
       <c r="R111" s="10"/>
@@ -7972,7 +7979,7 @@
     </row>
     <row r="112" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A112" s="4" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B112" s="5">
         <v>46155.562937361115</v>
@@ -7982,7 +7989,7 @@
         <v>46155.60132342593</v>
       </c>
       <c r="E112" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F112" s="6" t="s">
         <v>26</v>
@@ -8007,13 +8014,13 @@
         <v>26</v>
       </c>
       <c r="N112" s="6" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="O112" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P112" s="6" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="Q112" s="6"/>
       <c r="R112" s="6"/>
@@ -8023,7 +8030,7 @@
     </row>
     <row r="113" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A113" s="8" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B113" s="9">
         <v>46155.56294952546</v>
@@ -8033,7 +8040,7 @@
         <v>46155.60131890046</v>
       </c>
       <c r="E113" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F113" s="10" t="s">
         <v>26</v>
@@ -8058,13 +8065,13 @@
         <v>26</v>
       </c>
       <c r="N113" s="10" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="O113" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P113" s="10" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="Q113" s="10"/>
       <c r="R113" s="10"/>
@@ -8074,7 +8081,7 @@
     </row>
     <row r="114" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A114" s="4" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B114" s="5">
         <v>46149.16929695602</v>
@@ -8084,7 +8091,7 @@
         <v>46155.590775185185</v>
       </c>
       <c r="E114" s="6" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F114" s="6" t="s">
         <v>25</v>
@@ -8108,7 +8115,7 @@
         <v>26</v>
       </c>
       <c r="O114" s="6" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="P114" s="6" t="s">
         <v>26</v>
@@ -8121,7 +8128,7 @@
     </row>
     <row r="115" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A115" s="8" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B115" s="9">
         <v>46149.169301041664</v>
@@ -8131,16 +8138,16 @@
         <v>46155.60146953704</v>
       </c>
       <c r="E115" s="10" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F115" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G115" s="10" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="H115" s="10" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="I115" s="10"/>
       <c r="J115" s="9">
@@ -8156,13 +8163,13 @@
         <v>26</v>
       </c>
       <c r="N115" s="10" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="O115" s="10" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="P115" s="10" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="Q115" s="9">
         <v>46245</v>
@@ -8182,7 +8189,7 @@
     </row>
     <row r="116" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A116" s="4" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B116" s="5">
         <v>46149.1693071412</v>
@@ -8192,16 +8199,16 @@
         <v>46155.60144278935</v>
       </c>
       <c r="E116" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F116" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G116" s="6" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="H116" s="6" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="I116" s="6"/>
       <c r="J116" s="5">
@@ -8217,13 +8224,13 @@
         <v>26</v>
       </c>
       <c r="N116" s="6" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="O116" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P116" s="6" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="Q116" s="6"/>
       <c r="R116" s="6"/>
@@ -8233,7 +8240,7 @@
     </row>
     <row r="117" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A117" s="8" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B117" s="9">
         <v>46149.16931233797</v>
@@ -8243,16 +8250,16 @@
         <v>46155.60143921296</v>
       </c>
       <c r="E117" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F117" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G117" s="10" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="H117" s="10" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="I117" s="10"/>
       <c r="J117" s="9">
@@ -8268,13 +8275,13 @@
         <v>26</v>
       </c>
       <c r="N117" s="10" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="O117" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P117" s="10" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="Q117" s="10"/>
       <c r="R117" s="10"/>
@@ -8284,7 +8291,7 @@
     </row>
     <row r="118" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A118" s="4" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B118" s="5">
         <v>46155.56303070602</v>
@@ -8294,16 +8301,16 @@
         <v>46155.601436296296</v>
       </c>
       <c r="E118" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F118" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G118" s="6" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="H118" s="6" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="I118" s="6"/>
       <c r="J118" s="5">
@@ -8319,13 +8326,13 @@
         <v>26</v>
       </c>
       <c r="N118" s="6" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="O118" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P118" s="6" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="Q118" s="6"/>
       <c r="R118" s="6"/>
@@ -8335,7 +8342,7 @@
     </row>
     <row r="119" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A119" s="8" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B119" s="9">
         <v>46155.56306011574</v>
@@ -8345,16 +8352,16 @@
         <v>46155.60143193287</v>
       </c>
       <c r="E119" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F119" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G119" s="10" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="H119" s="10" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="I119" s="10"/>
       <c r="J119" s="9">
@@ -8370,13 +8377,13 @@
         <v>26</v>
       </c>
       <c r="N119" s="10" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="O119" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P119" s="10" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="Q119" s="10"/>
       <c r="R119" s="10"/>
@@ -8386,7 +8393,7 @@
     </row>
     <row r="120" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A120" s="4" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B120" s="5">
         <v>46149.1693175</v>
@@ -8396,7 +8403,7 @@
         <v>46155.6016600463</v>
       </c>
       <c r="E120" s="6" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="F120" s="6" t="s">
         <v>26</v>
@@ -8423,13 +8430,13 @@
         <v>26</v>
       </c>
       <c r="N120" s="6" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="O120" s="6" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="P120" s="6" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="Q120" s="5">
         <v>46246</v>
@@ -8449,7 +8456,7 @@
     </row>
     <row r="121" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A121" s="8" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B121" s="9">
         <v>46149.16932247685</v>
@@ -8459,7 +8466,7 @@
         <v>46155.601629756944</v>
       </c>
       <c r="E121" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F121" s="10" t="s">
         <v>26</v>
@@ -8486,13 +8493,13 @@
         <v>26</v>
       </c>
       <c r="N121" s="10" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="O121" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P121" s="10" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="Q121" s="10"/>
       <c r="R121" s="10"/>
@@ -8502,7 +8509,7 @@
     </row>
     <row r="122" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A122" s="4" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B122" s="5">
         <v>46149.16932829861</v>
@@ -8512,7 +8519,7 @@
         <v>46155.60162688658</v>
       </c>
       <c r="E122" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F122" s="6" t="s">
         <v>26</v>
@@ -8539,13 +8546,13 @@
         <v>26</v>
       </c>
       <c r="N122" s="6" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="O122" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P122" s="6" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="Q122" s="6"/>
       <c r="R122" s="6"/>
@@ -8555,7 +8562,7 @@
     </row>
     <row r="123" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A123" s="8" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B123" s="9">
         <v>46155.56313421296</v>
@@ -8565,7 +8572,7 @@
         <v>46155.601624421295</v>
       </c>
       <c r="E123" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F123" s="10" t="s">
         <v>26</v>
@@ -8592,13 +8599,13 @@
         <v>26</v>
       </c>
       <c r="N123" s="10" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="O123" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P123" s="10" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="Q123" s="10"/>
       <c r="R123" s="10"/>
@@ -8608,7 +8615,7 @@
     </row>
     <row r="124" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A124" s="4" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B124" s="5">
         <v>46155.5631459375</v>
@@ -8618,7 +8625,7 @@
         <v>46155.601620671296</v>
       </c>
       <c r="E124" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F124" s="6" t="s">
         <v>26</v>
@@ -8645,13 +8652,13 @@
         <v>26</v>
       </c>
       <c r="N124" s="6" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="O124" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P124" s="6" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="Q124" s="6"/>
       <c r="R124" s="6"/>
@@ -8661,7 +8668,7 @@
     </row>
     <row r="125" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A125" s="8" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B125" s="9">
         <v>46149.16933366898</v>
@@ -8671,16 +8678,16 @@
         <v>46155.60192047454</v>
       </c>
       <c r="E125" s="10" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F125" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G125" s="10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H125" s="10" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="I125" s="9">
         <v>46247</v>
@@ -8698,13 +8705,13 @@
         <v>26</v>
       </c>
       <c r="N125" s="10" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="O125" s="10" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="P125" s="10" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="Q125" s="9">
         <v>46247</v>
@@ -8724,7 +8731,7 @@
     </row>
     <row r="126" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A126" s="4" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B126" s="5">
         <v>46149.16933884259</v>
@@ -8734,16 +8741,16 @@
         <v>46155.601853796295</v>
       </c>
       <c r="E126" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F126" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G126" s="6" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H126" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="I126" s="6"/>
       <c r="J126" s="5">
@@ -8759,13 +8766,13 @@
         <v>26</v>
       </c>
       <c r="N126" s="6" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="O126" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P126" s="6" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="Q126" s="6"/>
       <c r="R126" s="6"/>
@@ -8775,7 +8782,7 @@
     </row>
     <row r="127" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A127" s="8" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B127" s="9">
         <v>46149.16934681713</v>
@@ -8785,16 +8792,16 @@
         <v>46155.60185450231</v>
       </c>
       <c r="E127" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F127" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G127" s="10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H127" s="10" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="I127" s="10"/>
       <c r="J127" s="9">
@@ -8810,13 +8817,13 @@
         <v>26</v>
       </c>
       <c r="N127" s="10" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="O127" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P127" s="10" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="Q127" s="10"/>
       <c r="R127" s="10"/>
@@ -8826,7 +8833,7 @@
     </row>
     <row r="128" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A128" s="4" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B128" s="5">
         <v>46155.56323461806</v>
@@ -8836,16 +8843,16 @@
         <v>46155.60185530093</v>
       </c>
       <c r="E128" s="6" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F128" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G128" s="6" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H128" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="I128" s="6"/>
       <c r="J128" s="5">
@@ -8861,13 +8868,13 @@
         <v>26</v>
       </c>
       <c r="N128" s="6" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="O128" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P128" s="6" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="Q128" s="6"/>
       <c r="R128" s="6"/>
@@ -8877,7 +8884,7 @@
     </row>
     <row r="129" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A129" s="8" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B129" s="9">
         <v>46155.563225370366</v>
@@ -8887,16 +8894,16 @@
         <v>46155.60185603009</v>
       </c>
       <c r="E129" s="10" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F129" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G129" s="10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H129" s="10" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="I129" s="10"/>
       <c r="J129" s="9">
@@ -8912,13 +8919,13 @@
         <v>26</v>
       </c>
       <c r="N129" s="10" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="O129" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P129" s="10" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="Q129" s="10"/>
       <c r="R129" s="10"/>
@@ -8928,7 +8935,7 @@
     </row>
     <row r="130" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A130" s="4" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B130" s="5">
         <v>46149.1693534375</v>
@@ -8938,16 +8945,16 @@
         <v>46155.60216496528</v>
       </c>
       <c r="E130" s="6" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="F130" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G130" s="6" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H130" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="I130" s="5">
         <v>46248</v>
@@ -8965,13 +8972,13 @@
         <v>26</v>
       </c>
       <c r="N130" s="6" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="O130" s="6" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="P130" s="6" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="Q130" s="5">
         <v>46248</v>
@@ -8991,7 +8998,7 @@
     </row>
     <row r="131" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A131" s="8" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B131" s="9">
         <v>46149.16935909722</v>
@@ -9001,16 +9008,16 @@
         <v>46155.602132280095</v>
       </c>
       <c r="E131" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F131" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G131" s="10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H131" s="10" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="I131" s="10"/>
       <c r="J131" s="9">
@@ -9026,13 +9033,13 @@
         <v>26</v>
       </c>
       <c r="N131" s="10" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="O131" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P131" s="10" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="Q131" s="10"/>
       <c r="R131" s="10"/>
@@ -9042,7 +9049,7 @@
     </row>
     <row r="132" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A132" s="4" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B132" s="5">
         <v>46149.16936413194</v>
@@ -9052,16 +9059,16 @@
         <v>46155.602128969906</v>
       </c>
       <c r="E132" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F132" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G132" s="6" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H132" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="I132" s="6"/>
       <c r="J132" s="5">
@@ -9077,13 +9084,13 @@
         <v>26</v>
       </c>
       <c r="N132" s="6" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="O132" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P132" s="6" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="Q132" s="6"/>
       <c r="R132" s="6"/>
@@ -9093,7 +9100,7 @@
     </row>
     <row r="133" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A133" s="8" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B133" s="9">
         <v>46155.56332277777</v>
@@ -9103,16 +9110,16 @@
         <v>46155.60212502315</v>
       </c>
       <c r="E133" s="10" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F133" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G133" s="10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H133" s="10" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="I133" s="10"/>
       <c r="J133" s="9">
@@ -9128,13 +9135,13 @@
         <v>26</v>
       </c>
       <c r="N133" s="10" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="O133" s="10" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="P133" s="10" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="Q133" s="10"/>
       <c r="R133" s="10"/>
@@ -9144,7 +9151,7 @@
     </row>
     <row r="134" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A134" s="4" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B134" s="5">
         <v>46155.56333268518</v>
@@ -9154,16 +9161,16 @@
         <v>46155.602120462965</v>
       </c>
       <c r="E134" s="6" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F134" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G134" s="6" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H134" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="I134" s="6"/>
       <c r="J134" s="5">
@@ -9179,13 +9186,13 @@
         <v>26</v>
       </c>
       <c r="N134" s="6" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="O134" s="6" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="P134" s="6" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="Q134" s="6"/>
       <c r="R134" s="6"/>
@@ -9195,7 +9202,7 @@
     </row>
     <row r="135" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A135" s="8" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B135" s="9">
         <v>46149.16936914352</v>
@@ -9205,7 +9212,7 @@
         <v>46155.60238891204</v>
       </c>
       <c r="E135" s="10" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="F135" s="10" t="s">
         <v>25</v>
@@ -9229,7 +9236,7 @@
         <v>26</v>
       </c>
       <c r="O135" s="10" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="P135" s="10" t="s">
         <v>26</v>
@@ -9242,7 +9249,7 @@
     </row>
     <row r="136" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A136" s="4" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B136" s="5">
         <v>46149.169373136574</v>
@@ -9252,16 +9259,16 @@
         <v>46155.602217824075</v>
       </c>
       <c r="E136" s="6" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="F136" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G136" s="6" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="H136" s="6" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="I136" s="5">
         <v>46251</v>
@@ -9279,13 +9286,13 @@
         <v>26</v>
       </c>
       <c r="N136" s="6" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="O136" s="6" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="P136" s="6" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="Q136" s="5">
         <v>46251</v>
@@ -9305,7 +9312,7 @@
     </row>
     <row r="137" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A137" s="8" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B137" s="9">
         <v>46149.169417349534</v>
@@ -9315,7 +9322,7 @@
         <v>46196.86942971065</v>
       </c>
       <c r="E137" s="10" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="F137" s="10" t="s">
         <v>26</v>
@@ -9342,13 +9349,13 @@
         <v>26</v>
       </c>
       <c r="N137" s="10" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="O137" s="10" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="P137" s="10" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="Q137" s="9">
         <v>46251</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-26 19:25 UTC
</commit_message>
<xml_diff>
--- a/data/50001545 - XEMORTIZ MINERA FRISCO.xlsx
+++ b/data/50001545 - XEMORTIZ MINERA FRISCO.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1608" uniqueCount="374">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1609" uniqueCount="374">
   <si>
     <t>50001545 - XEMORTIZ MINERA FRISCO</t>
   </si>
@@ -315,60 +315,63 @@
     <t>Propuesta compras:,Generación OC materiales corte Laser OT 4315</t>
   </si>
   <si>
+    <t>Tarea en curso</t>
+  </si>
+  <si>
+    <t>1214596725443928</t>
+  </si>
+  <si>
+    <t>Propuesta Corte plasma  OT 4315</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generación OC Corte Plasma OT 4315 </t>
+  </si>
+  <si>
+    <t>1214596725443938</t>
+  </si>
+  <si>
+    <t>Propuesta Mecanizado OT 4315</t>
+  </si>
+  <si>
+    <t>Generación OC Mecanizado OT 4315</t>
+  </si>
+  <si>
+    <t>1214596734036201</t>
+  </si>
+  <si>
+    <t>Propuesta Fabricación externa  OT 4315</t>
+  </si>
+  <si>
+    <t>Generacion OC Fabricación Externa OT 4315</t>
+  </si>
+  <si>
+    <t>1214563704105176</t>
+  </si>
+  <si>
+    <t>Compras:</t>
+  </si>
+  <si>
+    <t>Motor OT 4315,Alabe OT 4315,rodete OT 4315,Materiales corte Laser OT 4315</t>
+  </si>
+  <si>
+    <t>1214596734036211</t>
+  </si>
+  <si>
+    <t>Alabe OT 4315</t>
+  </si>
+  <si>
+    <t>Eliana</t>
+  </si>
+  <si>
+    <t>ecarico@zitron.com</t>
+  </si>
+  <si>
+    <t>Generación OC Alabe OT 4315,Fabricación Alabe OT 4315</t>
+  </si>
+  <si>
     <t>Tarea sin iniciar</t>
   </si>
   <si>
-    <t>1214596725443928</t>
-  </si>
-  <si>
-    <t>Propuesta Corte plasma  OT 4315</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generación OC Corte Plasma OT 4315 </t>
-  </si>
-  <si>
-    <t>1214596725443938</t>
-  </si>
-  <si>
-    <t>Propuesta Mecanizado OT 4315</t>
-  </si>
-  <si>
-    <t>Generación OC Mecanizado OT 4315</t>
-  </si>
-  <si>
-    <t>1214596734036201</t>
-  </si>
-  <si>
-    <t>Propuesta Fabricación externa  OT 4315</t>
-  </si>
-  <si>
-    <t>Generacion OC Fabricación Externa OT 4315</t>
-  </si>
-  <si>
-    <t>1214563704105176</t>
-  </si>
-  <si>
-    <t>Compras:</t>
-  </si>
-  <si>
-    <t>Motor OT 4315,Alabe OT 4315,rodete OT 4315,Materiales corte Laser OT 4315</t>
-  </si>
-  <si>
-    <t>1214596734036211</t>
-  </si>
-  <si>
-    <t>Alabe OT 4315</t>
-  </si>
-  <si>
-    <t>Eliana</t>
-  </si>
-  <si>
-    <t>ecarico@zitron.com</t>
-  </si>
-  <si>
-    <t>Generación OC Alabe OT 4315,Fabricación Alabe OT 4315</t>
-  </si>
-  <si>
     <t>1214596734036226</t>
   </si>
   <si>
@@ -613,9 +616,6 @@
   </si>
   <si>
     <t>check planos,Ingenieria y diseñoo:</t>
-  </si>
-  <si>
-    <t>Tarea en curso</t>
   </si>
   <si>
     <t>1214596734094526</t>
@@ -2680,7 +2680,7 @@
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="5">
-        <v>46189.188732361115</v>
+        <v>46199.77909486111</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>76</v>
@@ -2730,7 +2730,7 @@
       <c r="T18" s="6">
         <v>0</v>
       </c>
-      <c r="U18" s="11" t="s">
+      <c r="U18" s="12" t="s">
         <v>81</v>
       </c>
     </row>
@@ -2743,7 +2743,7 @@
       </c>
       <c r="C19" s="10"/>
       <c r="D19" s="9">
-        <v>46189.1887321875</v>
+        <v>46199.779095300924</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>83</v>
@@ -2793,7 +2793,7 @@
       <c r="T19" s="10">
         <v>0</v>
       </c>
-      <c r="U19" s="11" t="s">
+      <c r="U19" s="12" t="s">
         <v>81</v>
       </c>
     </row>
@@ -2806,7 +2806,7 @@
       </c>
       <c r="C20" s="6"/>
       <c r="D20" s="5">
-        <v>46189.18873256944</v>
+        <v>46199.77909486111</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>86</v>
@@ -2856,7 +2856,7 @@
       <c r="T20" s="6">
         <v>0</v>
       </c>
-      <c r="U20" s="11" t="s">
+      <c r="U20" s="12" t="s">
         <v>81</v>
       </c>
     </row>
@@ -2869,7 +2869,7 @@
       </c>
       <c r="C21" s="10"/>
       <c r="D21" s="9">
-        <v>46189.18873219907</v>
+        <v>46199.77909490741</v>
       </c>
       <c r="E21" s="10" t="s">
         <v>89</v>
@@ -2919,7 +2919,7 @@
       <c r="T21" s="10">
         <v>0</v>
       </c>
-      <c r="U21" s="11" t="s">
+      <c r="U21" s="12" t="s">
         <v>81</v>
       </c>
     </row>
@@ -3030,12 +3030,12 @@
         <v>0</v>
       </c>
       <c r="U23" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B24" s="5">
         <v>46149.168804155095</v>
@@ -3045,7 +3045,7 @@
         <v>46196.87158508102</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>26</v>
@@ -3078,23 +3078,23 @@
         <v>69</v>
       </c>
       <c r="P24" s="6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q24" s="6"/>
       <c r="R24" s="6"/>
       <c r="S24" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T24" s="6">
         <v>0</v>
       </c>
       <c r="U24" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B25" s="9">
         <v>46149.16880861111</v>
@@ -3104,7 +3104,7 @@
         <v>46169.86022740741</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F25" s="10" t="s">
         <v>26</v>
@@ -3134,26 +3134,26 @@
         <v>95</v>
       </c>
       <c r="O25" s="10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="P25" s="10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q25" s="10"/>
       <c r="R25" s="10"/>
       <c r="S25" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T25" s="10">
         <v>0</v>
       </c>
       <c r="U25" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B26" s="5">
         <v>46149.16881337963</v>
@@ -3163,7 +3163,7 @@
         <v>46179.17667454861</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>26</v>
@@ -3193,7 +3193,7 @@
         <v>92</v>
       </c>
       <c r="O26" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="P26" s="6" t="s">
         <v>92</v>
@@ -3211,12 +3211,12 @@
         <v>0</v>
       </c>
       <c r="U26" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B27" s="9">
         <v>46149.16881752315</v>
@@ -3226,7 +3226,7 @@
         <v>46197.50269849537</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F27" s="10" t="s">
         <v>26</v>
@@ -3253,29 +3253,29 @@
         <v>26</v>
       </c>
       <c r="N27" s="10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="O27" s="10" t="s">
         <v>72</v>
       </c>
       <c r="P27" s="10" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="Q27" s="10"/>
       <c r="R27" s="10"/>
       <c r="S27" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T27" s="10">
         <v>0</v>
       </c>
       <c r="U27" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B28" s="5">
         <v>46149.168821851854</v>
@@ -3285,7 +3285,7 @@
         <v>46178.170599363424</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F28" s="6" t="s">
         <v>26</v>
@@ -3312,29 +3312,29 @@
         <v>26</v>
       </c>
       <c r="N28" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="O28" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="P28" s="6" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q28" s="6"/>
       <c r="R28" s="6"/>
       <c r="S28" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T28" s="6">
         <v>0</v>
       </c>
       <c r="U28" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B29" s="9">
         <v>46149.1688262963</v>
@@ -3344,7 +3344,7 @@
         <v>46199.75288726852</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F29" s="10" t="s">
         <v>26</v>
@@ -3374,7 +3374,7 @@
         <v>92</v>
       </c>
       <c r="O29" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="P29" s="10" t="s">
         <v>92</v>
@@ -3392,12 +3392,12 @@
         <v>0</v>
       </c>
       <c r="U29" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B30" s="5">
         <v>46149.168830532406</v>
@@ -3409,7 +3409,7 @@
         <v>46199.75283171296</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F30" s="6" t="s">
         <v>26</v>
@@ -3436,29 +3436,29 @@
         <v>26</v>
       </c>
       <c r="N30" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="O30" s="6" t="s">
         <v>66</v>
       </c>
       <c r="P30" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Q30" s="6"/>
       <c r="R30" s="6"/>
       <c r="S30" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T30" s="6">
         <v>0</v>
       </c>
       <c r="U30" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B31" s="9">
         <v>46149.1688349537</v>
@@ -3468,7 +3468,7 @@
         <v>46199.752836423606</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F31" s="10" t="s">
         <v>26</v>
@@ -3495,29 +3495,29 @@
         <v>26</v>
       </c>
       <c r="N31" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="O31" s="10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="P31" s="10" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="Q31" s="10"/>
       <c r="R31" s="10"/>
       <c r="S31" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T31" s="10">
         <v>0</v>
       </c>
       <c r="U31" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B32" s="5">
         <v>46149.16884</v>
@@ -3529,7 +3529,7 @@
         <v>46199.752879155094</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F32" s="6" t="s">
         <v>26</v>
@@ -3556,29 +3556,29 @@
         <v>26</v>
       </c>
       <c r="N32" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="O32" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="P32" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Q32" s="6"/>
       <c r="R32" s="6"/>
       <c r="S32" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T32" s="6">
         <v>0</v>
       </c>
       <c r="U32" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B33" s="9">
         <v>46149.168844375</v>
@@ -3588,16 +3588,16 @@
         <v>46199.16976211805</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F33" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G33" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H33" s="10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I33" s="9">
         <v>46189</v>
@@ -3618,7 +3618,7 @@
         <v>92</v>
       </c>
       <c r="O33" s="10" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="P33" s="10" t="s">
         <v>92</v>
@@ -3630,18 +3630,18 @@
         <v>46199</v>
       </c>
       <c r="S33" s="12" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="T33" s="10">
         <v>0</v>
       </c>
       <c r="U33" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B34" s="5">
         <v>46149.16884893518</v>
@@ -3651,16 +3651,16 @@
         <v>46190.16888383102</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F34" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I34" s="5">
         <v>46189</v>
@@ -3678,29 +3678,29 @@
         <v>26</v>
       </c>
       <c r="N34" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="O34" s="6" t="s">
         <v>76</v>
       </c>
       <c r="P34" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Q34" s="6"/>
       <c r="R34" s="6"/>
       <c r="S34" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T34" s="6">
         <v>0</v>
       </c>
       <c r="U34" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B35" s="9">
         <v>46149.16885364584</v>
@@ -3710,16 +3710,16 @@
         <v>46199.16976567129</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F35" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G35" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H35" s="10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I35" s="9">
         <v>46191</v>
@@ -3737,29 +3737,29 @@
         <v>26</v>
       </c>
       <c r="N35" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="O35" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="P35" s="10" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="Q35" s="10"/>
       <c r="R35" s="10"/>
       <c r="S35" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T35" s="10">
         <v>0</v>
       </c>
       <c r="U35" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B36" s="5">
         <v>46149.1688584375</v>
@@ -3769,16 +3769,16 @@
         <v>46199.169766875</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F36" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I36" s="5">
         <v>46189</v>
@@ -3799,7 +3799,7 @@
         <v>92</v>
       </c>
       <c r="O36" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="P36" s="6" t="s">
         <v>26</v>
@@ -3811,18 +3811,18 @@
         <v>46199</v>
       </c>
       <c r="S36" s="12" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="T36" s="6">
         <v>0</v>
       </c>
       <c r="U36" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" s="8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B37" s="9">
         <v>46149.16891136574</v>
@@ -3838,10 +3838,10 @@
         <v>26</v>
       </c>
       <c r="G37" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H37" s="10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I37" s="9">
         <v>46189</v>
@@ -3859,13 +3859,13 @@
         <v>26</v>
       </c>
       <c r="N37" s="10" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="O37" s="10" t="s">
         <v>83</v>
       </c>
       <c r="P37" s="10" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="Q37" s="10"/>
       <c r="R37" s="10"/>
@@ -3875,7 +3875,7 @@
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B38" s="5">
         <v>46149.168917256946</v>
@@ -3885,16 +3885,16 @@
         <v>46199.16976444444</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F38" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I38" s="5">
         <v>46191</v>
@@ -3912,13 +3912,13 @@
         <v>26</v>
       </c>
       <c r="N38" s="6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="O38" s="6" t="s">
         <v>84</v>
       </c>
       <c r="P38" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="Q38" s="6"/>
       <c r="R38" s="6"/>
@@ -3928,7 +3928,7 @@
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" s="8" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B39" s="9">
         <v>46149.16892260416</v>
@@ -3938,16 +3938,16 @@
         <v>46169.859801203704</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F39" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G39" s="10" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H39" s="10" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I39" s="9">
         <v>46189</v>
@@ -3968,7 +3968,7 @@
         <v>92</v>
       </c>
       <c r="O39" s="10" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="P39" s="10" t="s">
         <v>26</v>
@@ -3980,18 +3980,18 @@
         <v>46230</v>
       </c>
       <c r="S39" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T39" s="10">
         <v>0</v>
       </c>
       <c r="U39" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B40" s="5">
         <v>46149.168932870365</v>
@@ -4007,10 +4007,10 @@
         <v>26</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H40" s="6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I40" s="5">
         <v>46189</v>
@@ -4028,13 +4028,13 @@
         <v>26</v>
       </c>
       <c r="N40" s="6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="O40" s="6" t="s">
         <v>89</v>
       </c>
       <c r="P40" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="Q40" s="6"/>
       <c r="R40" s="6"/>
@@ -4044,7 +4044,7 @@
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B41" s="9">
         <v>46149.16893796297</v>
@@ -4054,16 +4054,16 @@
         <v>46169.859942118055</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F41" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G41" s="10" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H41" s="10" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I41" s="9">
         <v>46198</v>
@@ -4081,13 +4081,13 @@
         <v>26</v>
       </c>
       <c r="N41" s="10" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="O41" s="10" t="s">
         <v>90</v>
       </c>
       <c r="P41" s="10" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="Q41" s="10"/>
       <c r="R41" s="10"/>
@@ -4097,7 +4097,7 @@
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B42" s="5">
         <v>46149.16894290509</v>
@@ -4107,16 +4107,16 @@
         <v>46169.859966018514</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F42" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I42" s="5">
         <v>46227</v>
@@ -4134,10 +4134,10 @@
         <v>26</v>
       </c>
       <c r="N42" s="6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="O42" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="P42" s="6" t="s">
         <v>26</v>
@@ -4150,7 +4150,7 @@
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="8" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B43" s="9">
         <v>46149.16894577546</v>
@@ -4160,16 +4160,16 @@
         <v>46169.85983048611</v>
       </c>
       <c r="E43" s="10" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F43" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G43" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H43" s="10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I43" s="9">
         <v>46189</v>
@@ -4190,7 +4190,7 @@
         <v>92</v>
       </c>
       <c r="O43" s="10" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="P43" s="10" t="s">
         <v>26</v>
@@ -4202,18 +4202,18 @@
         <v>46210</v>
       </c>
       <c r="S43" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T43" s="10">
         <v>0</v>
       </c>
       <c r="U43" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B44" s="5">
         <v>46149.16894971065</v>
@@ -4229,10 +4229,10 @@
         <v>26</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I44" s="5">
         <v>46189</v>
@@ -4250,13 +4250,13 @@
         <v>26</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="O44" s="6" t="s">
         <v>86</v>
       </c>
       <c r="P44" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="Q44" s="6"/>
       <c r="R44" s="6"/>
@@ -4266,7 +4266,7 @@
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" s="8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B45" s="9">
         <v>46149.1689542824</v>
@@ -4276,16 +4276,16 @@
         <v>46191.68560096065</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F45" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G45" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H45" s="10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I45" s="9">
         <v>46191</v>
@@ -4303,13 +4303,13 @@
         <v>26</v>
       </c>
       <c r="N45" s="10" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="O45" s="10" t="s">
         <v>87</v>
       </c>
       <c r="P45" s="10" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="Q45" s="10"/>
       <c r="R45" s="10"/>
@@ -4319,17 +4319,17 @@
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B46" s="5">
         <v>46149.16868141203</v>
       </c>
       <c r="C46" s="6"/>
       <c r="D46" s="5">
-        <v>46184.514930833335</v>
+        <v>46199.77902613426</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F46" s="6" t="s">
         <v>25</v>
@@ -4353,7 +4353,7 @@
         <v>26</v>
       </c>
       <c r="O46" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="P46" s="6" t="s">
         <v>26</v>
@@ -4362,11 +4362,13 @@
       <c r="R46" s="6"/>
       <c r="S46" s="6"/>
       <c r="T46" s="6"/>
-      <c r="U46" s="6"/>
+      <c r="U46" s="12" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" s="8" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B47" s="9">
         <v>46149.16895986111</v>
@@ -4378,16 +4380,16 @@
         <v>46197.71368634259</v>
       </c>
       <c r="E47" s="10" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F47" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G47" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H47" s="10" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="I47" s="9">
         <v>46162</v>
@@ -4405,13 +4407,13 @@
         <v>26</v>
       </c>
       <c r="N47" s="10" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="O47" s="10" t="s">
         <v>60</v>
       </c>
       <c r="P47" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="Q47" s="9">
         <v>46162</v>
@@ -4431,26 +4433,28 @@
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B48" s="5">
         <v>46149.16896564815</v>
       </c>
-      <c r="C48" s="6"/>
+      <c r="C48" s="5">
+        <v>46199.779006689816</v>
+      </c>
       <c r="D48" s="5">
-        <v>46199.752894212965</v>
+        <v>46199.779022372684</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F48" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="I48" s="5">
         <v>46177</v>
@@ -4468,13 +4472,13 @@
         <v>26</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="O48" s="6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="P48" s="6" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="Q48" s="5">
         <v>46146</v>
@@ -4486,10 +4490,10 @@
         <v>33</v>
       </c>
       <c r="T48" s="6">
-        <v>0</v>
-      </c>
-      <c r="U48" s="12" t="s">
-        <v>181</v>
+        <v>1</v>
+      </c>
+      <c r="U48" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
@@ -4499,9 +4503,11 @@
       <c r="B49" s="9">
         <v>46149.16897216435</v>
       </c>
-      <c r="C49" s="10"/>
+      <c r="C49" s="9">
+        <v>46199.779062685186</v>
+      </c>
       <c r="D49" s="9">
-        <v>46184.168774861115</v>
+        <v>46199.77907827546</v>
       </c>
       <c r="E49" s="10" t="s">
         <v>79</v>
@@ -4529,10 +4535,10 @@
         <v>26</v>
       </c>
       <c r="N49" s="10" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="O49" s="10" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="P49" s="10" t="s">
         <v>185</v>
@@ -4544,13 +4550,13 @@
         <v>46153</v>
       </c>
       <c r="S49" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T49" s="10">
-        <v>0</v>
-      </c>
-      <c r="U49" s="11" t="s">
-        <v>81</v>
+        <v>1</v>
+      </c>
+      <c r="U49" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
@@ -4592,7 +4598,7 @@
         <v>26</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="O50" s="6" t="s">
         <v>190</v>
@@ -4607,13 +4613,13 @@
         <v>46241</v>
       </c>
       <c r="S50" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T50" s="6">
         <v>0</v>
       </c>
       <c r="U50" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
@@ -4909,7 +4915,7 @@
         <v>198</v>
       </c>
       <c r="O56" s="6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="P56" s="6" t="s">
         <v>204</v>
@@ -4921,13 +4927,13 @@
         <v>46203</v>
       </c>
       <c r="S56" s="12" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="T56" s="6">
         <v>0</v>
       </c>
       <c r="U56" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
@@ -4948,10 +4954,10 @@
         <v>26</v>
       </c>
       <c r="G57" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H57" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I57" s="9">
         <v>46204</v>
@@ -4990,7 +4996,7 @@
         <v>0</v>
       </c>
       <c r="U57" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
@@ -5035,7 +5041,7 @@
         <v>198</v>
       </c>
       <c r="O58" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="P58" s="6" t="s">
         <v>211</v>
@@ -5047,13 +5053,13 @@
         <v>46203</v>
       </c>
       <c r="S58" s="12" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="T58" s="6">
         <v>0</v>
       </c>
       <c r="U58" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
@@ -5074,10 +5080,10 @@
         <v>26</v>
       </c>
       <c r="G59" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H59" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I59" s="9">
         <v>46204</v>
@@ -5116,7 +5122,7 @@
         <v>0</v>
       </c>
       <c r="U59" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
@@ -5161,7 +5167,7 @@
         <v>198</v>
       </c>
       <c r="O60" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="P60" s="6" t="s">
         <v>217</v>
@@ -5173,13 +5179,13 @@
         <v>46212</v>
       </c>
       <c r="S60" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T60" s="6">
         <v>0</v>
       </c>
       <c r="U60" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
@@ -5200,10 +5206,10 @@
         <v>26</v>
       </c>
       <c r="G61" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H61" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I61" s="9">
         <v>46213</v>
@@ -5236,13 +5242,13 @@
         <v>46216</v>
       </c>
       <c r="S61" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T61" s="10">
         <v>0</v>
       </c>
       <c r="U61" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
@@ -5346,13 +5352,13 @@
         <v>46219</v>
       </c>
       <c r="S63" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T63" s="10">
         <v>0</v>
       </c>
       <c r="U63" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
@@ -5621,13 +5627,13 @@
         <v>46226</v>
       </c>
       <c r="S68" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T68" s="6">
         <v>0</v>
       </c>
       <c r="U68" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
@@ -5639,7 +5645,7 @@
       </c>
       <c r="C69" s="10"/>
       <c r="D69" s="9">
-        <v>46155.59950737268</v>
+        <v>46199.779078356485</v>
       </c>
       <c r="E69" s="10" t="s">
         <v>192</v>
@@ -5692,7 +5698,7 @@
       </c>
       <c r="C70" s="6"/>
       <c r="D70" s="5">
-        <v>46155.59950449074</v>
+        <v>46199.77907907407</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>192</v>
@@ -5745,7 +5751,7 @@
       </c>
       <c r="C71" s="10"/>
       <c r="D71" s="9">
-        <v>46155.5995016088</v>
+        <v>46199.77908222222</v>
       </c>
       <c r="E71" s="10" t="s">
         <v>192</v>
@@ -5798,7 +5804,7 @@
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46155.59949699074</v>
+        <v>46199.7790828588</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>192</v>
@@ -5860,10 +5866,10 @@
         <v>26</v>
       </c>
       <c r="G73" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H73" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I73" s="9">
         <v>46227</v>
@@ -5896,13 +5902,13 @@
         <v>46227</v>
       </c>
       <c r="S73" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T73" s="10">
         <v>0</v>
       </c>
       <c r="U73" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
@@ -5914,7 +5920,7 @@
       </c>
       <c r="C74" s="6"/>
       <c r="D74" s="5">
-        <v>46155.59963545139</v>
+        <v>46199.77907962963</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>192</v>
@@ -5923,10 +5929,10 @@
         <v>26</v>
       </c>
       <c r="G74" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H74" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I74" s="5">
         <v>46227</v>
@@ -5967,7 +5973,7 @@
       </c>
       <c r="C75" s="10"/>
       <c r="D75" s="9">
-        <v>46155.59963275463</v>
+        <v>46199.77908010417</v>
       </c>
       <c r="E75" s="10" t="s">
         <v>192</v>
@@ -5976,10 +5982,10 @@
         <v>26</v>
       </c>
       <c r="G75" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H75" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I75" s="9">
         <v>46227</v>
@@ -6020,7 +6026,7 @@
       </c>
       <c r="C76" s="6"/>
       <c r="D76" s="5">
-        <v>46155.59962995371</v>
+        <v>46199.779083437505</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>192</v>
@@ -6029,10 +6035,10 @@
         <v>26</v>
       </c>
       <c r="G76" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I76" s="5">
         <v>46227</v>
@@ -6073,7 +6079,7 @@
       </c>
       <c r="C77" s="10"/>
       <c r="D77" s="9">
-        <v>46155.599625891206</v>
+        <v>46199.779083877314</v>
       </c>
       <c r="E77" s="10" t="s">
         <v>192</v>
@@ -6082,10 +6088,10 @@
         <v>26</v>
       </c>
       <c r="G77" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H77" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I77" s="9">
         <v>46227</v>
@@ -6204,7 +6210,7 @@
         <v>198</v>
       </c>
       <c r="O79" s="10" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="P79" s="10" t="s">
         <v>256</v>
@@ -6222,7 +6228,7 @@
         <v>0</v>
       </c>
       <c r="U79" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
@@ -6267,7 +6273,7 @@
         <v>198</v>
       </c>
       <c r="O80" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="P80" s="6" t="s">
         <v>259</v>
@@ -6285,7 +6291,7 @@
         <v>0</v>
       </c>
       <c r="U80" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
@@ -6330,7 +6336,7 @@
         <v>198</v>
       </c>
       <c r="O81" s="10" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="P81" s="10" t="s">
         <v>259</v>
@@ -6348,7 +6354,7 @@
         <v>0</v>
       </c>
       <c r="U81" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
@@ -6393,7 +6399,7 @@
         <v>198</v>
       </c>
       <c r="O82" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="P82" s="6" t="s">
         <v>264</v>
@@ -6405,13 +6411,13 @@
         <v>46231</v>
       </c>
       <c r="S82" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T82" s="6">
         <v>0</v>
       </c>
       <c r="U82" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">
@@ -6515,13 +6521,13 @@
         <v>46234</v>
       </c>
       <c r="S84" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T84" s="6">
         <v>0</v>
       </c>
       <c r="U84" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="85" spans="1:21" x14ac:dyDescent="0.25">
@@ -6790,13 +6796,13 @@
         <v>46237</v>
       </c>
       <c r="S89" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T89" s="10">
         <v>0</v>
       </c>
       <c r="U89" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="90" spans="1:21" x14ac:dyDescent="0.25">
@@ -6808,7 +6814,7 @@
       </c>
       <c r="C90" s="6"/>
       <c r="D90" s="5">
-        <v>46155.600606238426</v>
+        <v>46199.77908100694</v>
       </c>
       <c r="E90" s="6" t="s">
         <v>192</v>
@@ -6859,7 +6865,7 @@
       </c>
       <c r="C91" s="10"/>
       <c r="D91" s="9">
-        <v>46155.60060333333</v>
+        <v>46199.77908144676</v>
       </c>
       <c r="E91" s="10" t="s">
         <v>192</v>
@@ -6910,7 +6916,7 @@
       </c>
       <c r="C92" s="6"/>
       <c r="D92" s="5">
-        <v>46155.600600254635</v>
+        <v>46199.77908483797</v>
       </c>
       <c r="E92" s="6" t="s">
         <v>192</v>
@@ -6961,7 +6967,7 @@
       </c>
       <c r="C93" s="10"/>
       <c r="D93" s="9">
-        <v>46155.60059528935</v>
+        <v>46199.779085277776</v>
       </c>
       <c r="E93" s="10" t="s">
         <v>192</v>
@@ -7057,13 +7063,13 @@
         <v>46238</v>
       </c>
       <c r="S94" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T94" s="6">
         <v>0</v>
       </c>
       <c r="U94" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="95" spans="1:21" x14ac:dyDescent="0.25">
@@ -7075,7 +7081,7 @@
       </c>
       <c r="C95" s="10"/>
       <c r="D95" s="9">
-        <v>46155.600763483795</v>
+        <v>46199.779080567125</v>
       </c>
       <c r="E95" s="10" t="s">
         <v>192</v>
@@ -7126,7 +7132,7 @@
       </c>
       <c r="C96" s="6"/>
       <c r="D96" s="5">
-        <v>46155.60076056713</v>
+        <v>46199.779077430554</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>192</v>
@@ -7177,7 +7183,7 @@
       </c>
       <c r="C97" s="10"/>
       <c r="D97" s="9">
-        <v>46155.60075752315</v>
+        <v>46199.779084340276</v>
       </c>
       <c r="E97" s="10" t="s">
         <v>192</v>
@@ -7228,7 +7234,7 @@
       </c>
       <c r="C98" s="6"/>
       <c r="D98" s="5">
-        <v>46155.600753645835</v>
+        <v>46199.779085752314</v>
       </c>
       <c r="E98" s="6" t="s">
         <v>192</v>
@@ -7324,13 +7330,13 @@
         <v>46239</v>
       </c>
       <c r="S99" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T99" s="10">
         <v>0</v>
       </c>
       <c r="U99" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="100" spans="1:21" x14ac:dyDescent="0.25">
@@ -7342,7 +7348,7 @@
       </c>
       <c r="C100" s="6"/>
       <c r="D100" s="5">
-        <v>46155.600918067124</v>
+        <v>46199.779077858795</v>
       </c>
       <c r="E100" s="6" t="s">
         <v>192</v>
@@ -7393,7 +7399,7 @@
       </c>
       <c r="C101" s="10"/>
       <c r="D101" s="9">
-        <v>46155.60091518519</v>
+        <v>46199.77908177083</v>
       </c>
       <c r="E101" s="10" t="s">
         <v>192</v>
@@ -7444,7 +7450,7 @@
       </c>
       <c r="C102" s="6"/>
       <c r="D102" s="5">
-        <v>46155.60091216435</v>
+        <v>46199.77908608796</v>
       </c>
       <c r="E102" s="6" t="s">
         <v>192</v>
@@ -7495,7 +7501,7 @@
       </c>
       <c r="C103" s="10"/>
       <c r="D103" s="9">
-        <v>46155.60090780092</v>
+        <v>46199.77908645834</v>
       </c>
       <c r="E103" s="10" t="s">
         <v>192</v>
@@ -7591,13 +7597,13 @@
         <v>46240</v>
       </c>
       <c r="S104" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T104" s="6">
         <v>0</v>
       </c>
       <c r="U104" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="105" spans="1:21" x14ac:dyDescent="0.25">
@@ -7866,13 +7872,13 @@
         <v>46244</v>
       </c>
       <c r="S109" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T109" s="10">
         <v>0</v>
       </c>
       <c r="U109" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="110" spans="1:21" x14ac:dyDescent="0.25">
@@ -8178,13 +8184,13 @@
         <v>46245</v>
       </c>
       <c r="S115" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T115" s="10">
         <v>0</v>
       </c>
       <c r="U115" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="116" spans="1:21" x14ac:dyDescent="0.25">
@@ -8445,13 +8451,13 @@
         <v>46246</v>
       </c>
       <c r="S120" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T120" s="6">
         <v>0</v>
       </c>
       <c r="U120" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="121" spans="1:21" x14ac:dyDescent="0.25">
@@ -8720,13 +8726,13 @@
         <v>46247</v>
       </c>
       <c r="S125" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T125" s="10">
         <v>0</v>
       </c>
       <c r="U125" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="126" spans="1:21" x14ac:dyDescent="0.25">
@@ -8987,13 +8993,13 @@
         <v>46248</v>
       </c>
       <c r="S130" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T130" s="6">
         <v>0</v>
       </c>
       <c r="U130" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="131" spans="1:21" x14ac:dyDescent="0.25">
@@ -9301,13 +9307,13 @@
         <v>46255</v>
       </c>
       <c r="S136" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T136" s="6">
         <v>0</v>
       </c>
       <c r="U136" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="137" spans="1:21" x14ac:dyDescent="0.25">
@@ -9364,13 +9370,13 @@
         <v>46255</v>
       </c>
       <c r="S137" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="T137" s="10">
         <v>0</v>
       </c>
       <c r="U137" s="11" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-01 22:10 UTC
</commit_message>
<xml_diff>
--- a/data/50001545 - XEMORTIZ MINERA FRISCO.xlsx
+++ b/data/50001545 - XEMORTIZ MINERA FRISCO.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1609" uniqueCount="374">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1610" uniqueCount="374">
   <si>
     <t>50001545 - XEMORTIZ MINERA FRISCO</t>
   </si>
@@ -315,280 +315,280 @@
     <t>Propuesta compras:,Generación OC materiales corte Laser OT 4315</t>
   </si>
   <si>
+    <t>1214596725443928</t>
+  </si>
+  <si>
+    <t>Propuesta Corte plasma  OT 4315</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generación OC Corte Plasma OT 4315 </t>
+  </si>
+  <si>
+    <t>1214596725443938</t>
+  </si>
+  <si>
+    <t>Propuesta Mecanizado OT 4315</t>
+  </si>
+  <si>
+    <t>Generación OC Mecanizado OT 4315</t>
+  </si>
+  <si>
+    <t>1214596734036201</t>
+  </si>
+  <si>
+    <t>Propuesta Fabricación externa  OT 4315</t>
+  </si>
+  <si>
+    <t>Generacion OC Fabricación Externa OT 4315</t>
+  </si>
+  <si>
+    <t>1214563704105176</t>
+  </si>
+  <si>
+    <t>Compras:</t>
+  </si>
+  <si>
+    <t>Motor OT 4315,Alabe OT 4315,rodete OT 4315,Materiales corte Laser OT 4315</t>
+  </si>
+  <si>
+    <t>1214596734036211</t>
+  </si>
+  <si>
+    <t>Alabe OT 4315</t>
+  </si>
+  <si>
+    <t>Eliana</t>
+  </si>
+  <si>
+    <t>ecarico@zitron.com</t>
+  </si>
+  <si>
+    <t>Generación OC Alabe OT 4315,Fabricación Alabe OT 4315</t>
+  </si>
+  <si>
+    <t>Tarea sin iniciar</t>
+  </si>
+  <si>
+    <t>1214596734036226</t>
+  </si>
+  <si>
+    <t>Generación OC Alabe OT 4315</t>
+  </si>
+  <si>
+    <t>Alabe OT 4315,Fabricación Alabe OT 4315</t>
+  </si>
+  <si>
+    <t>Baja</t>
+  </si>
+  <si>
+    <t>1214596725445208</t>
+  </si>
+  <si>
+    <t>Fabricación Alabe OT 4315</t>
+  </si>
+  <si>
+    <t>Alabe OT 4315,Recepcion Alabe</t>
+  </si>
+  <si>
+    <t>1214596725445226</t>
+  </si>
+  <si>
+    <t>rodete OT 4315</t>
+  </si>
+  <si>
+    <t>Fabricación Rodete OT 4315,Generación OC Rodete OT 4315</t>
+  </si>
+  <si>
+    <t>1214596772319023</t>
+  </si>
+  <si>
+    <t>Generación OC Rodete OT 4315</t>
+  </si>
+  <si>
+    <t>Fabricación Rodete OT 4315,rodete OT 4315</t>
+  </si>
+  <si>
+    <t>1214596725454716</t>
+  </si>
+  <si>
+    <t>Fabricación Rodete OT 4315</t>
+  </si>
+  <si>
+    <t>rodete OT 4315,Recepcion Rodete</t>
+  </si>
+  <si>
+    <t>1214596725454734</t>
+  </si>
+  <si>
+    <t>Motor OT 4315</t>
+  </si>
+  <si>
+    <t>Generación OC motor OT 4315,Fabricación motor OT 4315,Planos motor proveedor OT 4315</t>
+  </si>
+  <si>
+    <t>1214596772320275</t>
+  </si>
+  <si>
+    <t>Generación OC motor OT 4315</t>
+  </si>
+  <si>
+    <t>Motor OT 4315,Fabricación motor OT 4315,Planos motor proveedor OT 4315</t>
+  </si>
+  <si>
+    <t>1214596772320293</t>
+  </si>
+  <si>
+    <t>Fabricación motor OT 4315</t>
+  </si>
+  <si>
+    <t>Recepcion motor,Motor OT 4315</t>
+  </si>
+  <si>
+    <t>1214596772322550</t>
+  </si>
+  <si>
+    <t>Planos motor proveedor OT 4315</t>
+  </si>
+  <si>
+    <t>Planos definitivos,Motor OT 4315</t>
+  </si>
+  <si>
+    <t>1214596772322568</t>
+  </si>
+  <si>
+    <t>Materiales corte Laser OT 4315</t>
+  </si>
+  <si>
+    <t>Yerlia Ayleen Castillo Diaz</t>
+  </si>
+  <si>
+    <t>yerlia.castillo@zitron.com</t>
+  </si>
+  <si>
+    <t>Generación OC materiales corte Laser OT 4315,Fabricacion Corte Laser  OT 4315</t>
+  </si>
+  <si>
+    <t>1214596969807197</t>
+  </si>
+  <si>
+    <t>Generación OC materiales corte Laser OT 4315</t>
+  </si>
+  <si>
+    <t>Materiales corte Laser OT 4315,Fabricacion Corte Laser  OT 4315</t>
+  </si>
+  <si>
+    <t>1214596969807215</t>
+  </si>
+  <si>
+    <t>Fabricacion Corte Laser  OT 4315</t>
+  </si>
+  <si>
+    <t>Recepcion materiales corte laser,Materiales corte Laser OT 4315</t>
+  </si>
+  <si>
+    <t>1214596969814573</t>
+  </si>
+  <si>
+    <t>Materiales Corte Plasma  OT 4315</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fabricación Corte Plasma OT 4315 ,Generación OC Corte Plasma OT 4315 </t>
+  </si>
+  <si>
+    <t>1214596969796648</t>
+  </si>
+  <si>
+    <t>Fabricación Corte Plasma OT 4315 ,Materiales Corte Plasma  OT 4315</t>
+  </si>
+  <si>
+    <t>1214596772340020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fabricación Corte Plasma OT 4315 </t>
+  </si>
+  <si>
+    <t>Recepcion Materiales corte plasma,Materiales Corte Plasma  OT 4315</t>
+  </si>
+  <si>
+    <t>1214596772340035</t>
+  </si>
+  <si>
+    <t>Fabricación Externa OT 4315</t>
+  </si>
+  <si>
+    <t>Rosemary Singh</t>
+  </si>
+  <si>
+    <t>rosemary.singh@zitron.com</t>
+  </si>
+  <si>
+    <t>Generacion OC Fabricación Externa OT 4315,Fabricación estructura proveedor externo OT 4315</t>
+  </si>
+  <si>
+    <t>1214596772340045</t>
+  </si>
+  <si>
+    <t>Fabricación Externa OT 4315,Fabricación estructura proveedor externo OT 4315</t>
+  </si>
+  <si>
+    <t>1214596725472897</t>
+  </si>
+  <si>
+    <t>Fabricación estructura proveedor externo OT 4315</t>
+  </si>
+  <si>
+    <t>Recepcion fabricación externa ,Fabricación Externa OT 4315,Control de calidad fabricación externa  OT 4315</t>
+  </si>
+  <si>
+    <t>1214596725472912</t>
+  </si>
+  <si>
+    <t>Control de calidad fabricación externa  OT 4315</t>
+  </si>
+  <si>
+    <t>Nicolás López</t>
+  </si>
+  <si>
+    <t>nicolas.lopez@zitron.com</t>
+  </si>
+  <si>
+    <t>1214596725472956</t>
+  </si>
+  <si>
+    <t>Mecanizado OT 4315</t>
+  </si>
+  <si>
+    <t>Fabricación Mecanizado OT 4315,Generación OC Mecanizado OT 4315</t>
+  </si>
+  <si>
+    <t>Media</t>
+  </si>
+  <si>
+    <t>1214596725472966</t>
+  </si>
+  <si>
+    <t>Fabricación Mecanizado OT 4315,Mecanizado OT 4315</t>
+  </si>
+  <si>
+    <t>1214596725472981</t>
+  </si>
+  <si>
+    <t>Fabricación Mecanizado OT 4315</t>
+  </si>
+  <si>
+    <t>Mecanizado OT 4315,Recepcion mecanizado</t>
+  </si>
+  <si>
+    <t>1214563704105178</t>
+  </si>
+  <si>
+    <t>Ingenieria y diseñoo:</t>
+  </si>
+  <si>
+    <t>Planos preliminar,Planos definitivos</t>
+  </si>
+  <si>
     <t>Tarea en curso</t>
-  </si>
-  <si>
-    <t>1214596725443928</t>
-  </si>
-  <si>
-    <t>Propuesta Corte plasma  OT 4315</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generación OC Corte Plasma OT 4315 </t>
-  </si>
-  <si>
-    <t>1214596725443938</t>
-  </si>
-  <si>
-    <t>Propuesta Mecanizado OT 4315</t>
-  </si>
-  <si>
-    <t>Generación OC Mecanizado OT 4315</t>
-  </si>
-  <si>
-    <t>1214596734036201</t>
-  </si>
-  <si>
-    <t>Propuesta Fabricación externa  OT 4315</t>
-  </si>
-  <si>
-    <t>Generacion OC Fabricación Externa OT 4315</t>
-  </si>
-  <si>
-    <t>1214563704105176</t>
-  </si>
-  <si>
-    <t>Compras:</t>
-  </si>
-  <si>
-    <t>Motor OT 4315,Alabe OT 4315,rodete OT 4315,Materiales corte Laser OT 4315</t>
-  </si>
-  <si>
-    <t>1214596734036211</t>
-  </si>
-  <si>
-    <t>Alabe OT 4315</t>
-  </si>
-  <si>
-    <t>Eliana</t>
-  </si>
-  <si>
-    <t>ecarico@zitron.com</t>
-  </si>
-  <si>
-    <t>Generación OC Alabe OT 4315,Fabricación Alabe OT 4315</t>
-  </si>
-  <si>
-    <t>Tarea sin iniciar</t>
-  </si>
-  <si>
-    <t>1214596734036226</t>
-  </si>
-  <si>
-    <t>Generación OC Alabe OT 4315</t>
-  </si>
-  <si>
-    <t>Alabe OT 4315,Fabricación Alabe OT 4315</t>
-  </si>
-  <si>
-    <t>Baja</t>
-  </si>
-  <si>
-    <t>1214596725445208</t>
-  </si>
-  <si>
-    <t>Fabricación Alabe OT 4315</t>
-  </si>
-  <si>
-    <t>Alabe OT 4315,Recepcion Alabe</t>
-  </si>
-  <si>
-    <t>1214596725445226</t>
-  </si>
-  <si>
-    <t>rodete OT 4315</t>
-  </si>
-  <si>
-    <t>Fabricación Rodete OT 4315,Generación OC Rodete OT 4315</t>
-  </si>
-  <si>
-    <t>1214596772319023</t>
-  </si>
-  <si>
-    <t>Generación OC Rodete OT 4315</t>
-  </si>
-  <si>
-    <t>Fabricación Rodete OT 4315,rodete OT 4315</t>
-  </si>
-  <si>
-    <t>1214596725454716</t>
-  </si>
-  <si>
-    <t>Fabricación Rodete OT 4315</t>
-  </si>
-  <si>
-    <t>rodete OT 4315,Recepcion Rodete</t>
-  </si>
-  <si>
-    <t>1214596725454734</t>
-  </si>
-  <si>
-    <t>Motor OT 4315</t>
-  </si>
-  <si>
-    <t>Generación OC motor OT 4315,Fabricación motor OT 4315,Planos motor proveedor OT 4315</t>
-  </si>
-  <si>
-    <t>1214596772320275</t>
-  </si>
-  <si>
-    <t>Generación OC motor OT 4315</t>
-  </si>
-  <si>
-    <t>Motor OT 4315,Fabricación motor OT 4315,Planos motor proveedor OT 4315</t>
-  </si>
-  <si>
-    <t>1214596772320293</t>
-  </si>
-  <si>
-    <t>Fabricación motor OT 4315</t>
-  </si>
-  <si>
-    <t>Recepcion motor,Motor OT 4315</t>
-  </si>
-  <si>
-    <t>1214596772322550</t>
-  </si>
-  <si>
-    <t>Planos motor proveedor OT 4315</t>
-  </si>
-  <si>
-    <t>Planos definitivos,Motor OT 4315</t>
-  </si>
-  <si>
-    <t>1214596772322568</t>
-  </si>
-  <si>
-    <t>Materiales corte Laser OT 4315</t>
-  </si>
-  <si>
-    <t>Yerlia Ayleen Castillo Diaz</t>
-  </si>
-  <si>
-    <t>yerlia.castillo@zitron.com</t>
-  </si>
-  <si>
-    <t>Generación OC materiales corte Laser OT 4315,Fabricacion Corte Laser  OT 4315</t>
-  </si>
-  <si>
-    <t>1214596969807197</t>
-  </si>
-  <si>
-    <t>Generación OC materiales corte Laser OT 4315</t>
-  </si>
-  <si>
-    <t>Materiales corte Laser OT 4315,Fabricacion Corte Laser  OT 4315</t>
-  </si>
-  <si>
-    <t>1214596969807215</t>
-  </si>
-  <si>
-    <t>Fabricacion Corte Laser  OT 4315</t>
-  </si>
-  <si>
-    <t>Recepcion materiales corte laser,Materiales corte Laser OT 4315</t>
-  </si>
-  <si>
-    <t>1214596969814573</t>
-  </si>
-  <si>
-    <t>Materiales Corte Plasma  OT 4315</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fabricación Corte Plasma OT 4315 ,Generación OC Corte Plasma OT 4315 </t>
-  </si>
-  <si>
-    <t>1214596969796648</t>
-  </si>
-  <si>
-    <t>Fabricación Corte Plasma OT 4315 ,Materiales Corte Plasma  OT 4315</t>
-  </si>
-  <si>
-    <t>1214596772340020</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fabricación Corte Plasma OT 4315 </t>
-  </si>
-  <si>
-    <t>Recepcion Materiales corte plasma,Materiales Corte Plasma  OT 4315</t>
-  </si>
-  <si>
-    <t>1214596772340035</t>
-  </si>
-  <si>
-    <t>Fabricación Externa OT 4315</t>
-  </si>
-  <si>
-    <t>Rosemary Singh</t>
-  </si>
-  <si>
-    <t>rosemary.singh@zitron.com</t>
-  </si>
-  <si>
-    <t>Generacion OC Fabricación Externa OT 4315,Fabricación estructura proveedor externo OT 4315</t>
-  </si>
-  <si>
-    <t>1214596772340045</t>
-  </si>
-  <si>
-    <t>Fabricación Externa OT 4315,Fabricación estructura proveedor externo OT 4315</t>
-  </si>
-  <si>
-    <t>1214596725472897</t>
-  </si>
-  <si>
-    <t>Fabricación estructura proveedor externo OT 4315</t>
-  </si>
-  <si>
-    <t>Recepcion fabricación externa ,Fabricación Externa OT 4315,Control de calidad fabricación externa  OT 4315</t>
-  </si>
-  <si>
-    <t>1214596725472912</t>
-  </si>
-  <si>
-    <t>Control de calidad fabricación externa  OT 4315</t>
-  </si>
-  <si>
-    <t>Nicolás López</t>
-  </si>
-  <si>
-    <t>nicolas.lopez@zitron.com</t>
-  </si>
-  <si>
-    <t>1214596725472956</t>
-  </si>
-  <si>
-    <t>Mecanizado OT 4315</t>
-  </si>
-  <si>
-    <t>Fabricación Mecanizado OT 4315,Generación OC Mecanizado OT 4315</t>
-  </si>
-  <si>
-    <t>Media</t>
-  </si>
-  <si>
-    <t>1214596725472966</t>
-  </si>
-  <si>
-    <t>Fabricación Mecanizado OT 4315,Mecanizado OT 4315</t>
-  </si>
-  <si>
-    <t>1214596725472981</t>
-  </si>
-  <si>
-    <t>Fabricación Mecanizado OT 4315</t>
-  </si>
-  <si>
-    <t>Mecanizado OT 4315,Recepcion mecanizado</t>
-  </si>
-  <si>
-    <t>1214563704105178</t>
-  </si>
-  <si>
-    <t>Ingenieria y diseñoo:</t>
-  </si>
-  <si>
-    <t>Planos preliminar,Planos definitivos</t>
   </si>
   <si>
     <t>1214596624002438</t>
@@ -2436,9 +2436,11 @@
       <c r="B14" s="5">
         <v>46149.16867222222</v>
       </c>
-      <c r="C14" s="6"/>
+      <c r="C14" s="5">
+        <v>46204.91290795139</v>
+      </c>
       <c r="D14" s="5">
-        <v>46197.5026965625</v>
+        <v>46204.912918587965</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>63</v>
@@ -2473,8 +2475,12 @@
       <c r="Q14" s="6"/>
       <c r="R14" s="6"/>
       <c r="S14" s="6"/>
-      <c r="T14" s="6"/>
-      <c r="U14" s="6"/>
+      <c r="T14" s="6">
+        <v>1</v>
+      </c>
+      <c r="U14" s="7" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
@@ -2678,9 +2684,11 @@
       <c r="B18" s="5">
         <v>46149.168784837966</v>
       </c>
-      <c r="C18" s="6"/>
+      <c r="C18" s="5">
+        <v>46204.91285559028</v>
+      </c>
       <c r="D18" s="5">
-        <v>46199.77909486111</v>
+        <v>46204.91287212963</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>76</v>
@@ -2728,25 +2736,27 @@
         <v>33</v>
       </c>
       <c r="T18" s="6">
-        <v>0</v>
-      </c>
-      <c r="U18" s="12" t="s">
-        <v>81</v>
+        <v>1</v>
+      </c>
+      <c r="U18" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B19" s="9">
         <v>46149.168789351854</v>
       </c>
-      <c r="C19" s="10"/>
+      <c r="C19" s="9">
+        <v>46204.91289165509</v>
+      </c>
       <c r="D19" s="9">
-        <v>46199.779095300924</v>
+        <v>46204.91290902778</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F19" s="10" t="s">
         <v>26</v>
@@ -2779,7 +2789,7 @@
         <v>79</v>
       </c>
       <c r="P19" s="10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="Q19" s="9">
         <v>46185</v>
@@ -2791,25 +2801,27 @@
         <v>33</v>
       </c>
       <c r="T19" s="10">
-        <v>0</v>
-      </c>
-      <c r="U19" s="12" t="s">
-        <v>81</v>
+        <v>1</v>
+      </c>
+      <c r="U19" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B20" s="5">
         <v>46149.16879285879</v>
       </c>
-      <c r="C20" s="6"/>
+      <c r="C20" s="5">
+        <v>46204.91205277778</v>
+      </c>
       <c r="D20" s="5">
-        <v>46199.77909486111</v>
+        <v>46204.91223577547</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>26</v>
@@ -2842,7 +2854,7 @@
         <v>79</v>
       </c>
       <c r="P20" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="Q20" s="5">
         <v>46185</v>
@@ -2854,25 +2866,27 @@
         <v>33</v>
       </c>
       <c r="T20" s="6">
-        <v>0</v>
-      </c>
-      <c r="U20" s="12" t="s">
-        <v>81</v>
+        <v>1</v>
+      </c>
+      <c r="U20" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B21" s="9">
         <v>46149.16879642361</v>
       </c>
-      <c r="C21" s="10"/>
+      <c r="C21" s="9">
+        <v>46204.911869143514</v>
+      </c>
       <c r="D21" s="9">
-        <v>46199.77909490741</v>
+        <v>46204.91200600694</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F21" s="10" t="s">
         <v>26</v>
@@ -2905,7 +2919,7 @@
         <v>79</v>
       </c>
       <c r="P21" s="10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="Q21" s="9">
         <v>46185</v>
@@ -2917,15 +2931,15 @@
         <v>33</v>
       </c>
       <c r="T21" s="10">
-        <v>0</v>
-      </c>
-      <c r="U21" s="12" t="s">
-        <v>81</v>
+        <v>1</v>
+      </c>
+      <c r="U21" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B22" s="5">
         <v>46149.168676875</v>
@@ -2935,7 +2949,7 @@
         <v>46155.55343407407</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>25</v>
@@ -2959,7 +2973,7 @@
         <v>26</v>
       </c>
       <c r="O22" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="P22" s="6" t="s">
         <v>26</v>
@@ -2972,7 +2986,7 @@
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B23" s="9">
         <v>46149.168800127314</v>
@@ -2982,16 +2996,16 @@
         <v>46169.85973167824</v>
       </c>
       <c r="E23" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="F23" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G23" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="F23" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G23" s="10" t="s">
+      <c r="H23" s="10" t="s">
         <v>96</v>
-      </c>
-      <c r="H23" s="10" t="s">
-        <v>97</v>
       </c>
       <c r="I23" s="9">
         <v>46157</v>
@@ -3009,13 +3023,13 @@
         <v>26</v>
       </c>
       <c r="N23" s="10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="O23" s="10" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="P23" s="10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="Q23" s="9">
         <v>46157</v>
@@ -3030,12 +3044,12 @@
         <v>0</v>
       </c>
       <c r="U23" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B24" s="5">
         <v>46149.168804155095</v>
@@ -3045,16 +3059,16 @@
         <v>46196.87158508102</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G24" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="H24" s="6" t="s">
         <v>96</v>
-      </c>
-      <c r="H24" s="6" t="s">
-        <v>97</v>
       </c>
       <c r="I24" s="5">
         <v>46157</v>
@@ -3072,29 +3086,29 @@
         <v>26</v>
       </c>
       <c r="N24" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="O24" s="6" t="s">
         <v>69</v>
       </c>
       <c r="P24" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="Q24" s="6"/>
       <c r="R24" s="6"/>
       <c r="S24" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T24" s="6">
         <v>0</v>
       </c>
       <c r="U24" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B25" s="9">
         <v>46149.16880861111</v>
@@ -3104,16 +3118,16 @@
         <v>46169.86022740741</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F25" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G25" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="H25" s="10" t="s">
         <v>96</v>
-      </c>
-      <c r="H25" s="10" t="s">
-        <v>97</v>
       </c>
       <c r="I25" s="9">
         <v>46161</v>
@@ -3131,29 +3145,29 @@
         <v>26</v>
       </c>
       <c r="N25" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="O25" s="10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P25" s="10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="Q25" s="10"/>
       <c r="R25" s="10"/>
       <c r="S25" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T25" s="10">
         <v>0</v>
       </c>
       <c r="U25" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B26" s="5">
         <v>46149.16881337963</v>
@@ -3163,16 +3177,16 @@
         <v>46179.17667454861</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G26" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="H26" s="6" t="s">
         <v>96</v>
-      </c>
-      <c r="H26" s="6" t="s">
-        <v>97</v>
       </c>
       <c r="I26" s="5">
         <v>46157</v>
@@ -3190,13 +3204,13 @@
         <v>26</v>
       </c>
       <c r="N26" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="O26" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="P26" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="Q26" s="5">
         <v>46157</v>
@@ -3211,12 +3225,12 @@
         <v>0</v>
       </c>
       <c r="U26" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B27" s="9">
         <v>46149.16881752315</v>
@@ -3226,16 +3240,16 @@
         <v>46197.50269849537</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F27" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G27" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="H27" s="10" t="s">
         <v>96</v>
-      </c>
-      <c r="H27" s="10" t="s">
-        <v>97</v>
       </c>
       <c r="I27" s="9">
         <v>46157</v>
@@ -3253,29 +3267,29 @@
         <v>26</v>
       </c>
       <c r="N27" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="O27" s="10" t="s">
         <v>72</v>
       </c>
       <c r="P27" s="10" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="Q27" s="10"/>
       <c r="R27" s="10"/>
       <c r="S27" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T27" s="10">
         <v>0</v>
       </c>
       <c r="U27" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B28" s="5">
         <v>46149.168821851854</v>
@@ -3285,16 +3299,16 @@
         <v>46178.170599363424</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F28" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G28" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="H28" s="6" t="s">
         <v>96</v>
-      </c>
-      <c r="H28" s="6" t="s">
-        <v>97</v>
       </c>
       <c r="I28" s="5">
         <v>46161</v>
@@ -3312,29 +3326,29 @@
         <v>26</v>
       </c>
       <c r="N28" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="O28" s="6" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="P28" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="Q28" s="6"/>
       <c r="R28" s="6"/>
       <c r="S28" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T28" s="6">
         <v>0</v>
       </c>
       <c r="U28" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B29" s="9">
         <v>46149.1688262963</v>
@@ -3344,16 +3358,16 @@
         <v>46199.75288726852</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F29" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G29" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="H29" s="10" t="s">
         <v>96</v>
-      </c>
-      <c r="H29" s="10" t="s">
-        <v>97</v>
       </c>
       <c r="I29" s="9">
         <v>46157</v>
@@ -3371,13 +3385,13 @@
         <v>26</v>
       </c>
       <c r="N29" s="10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="O29" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="P29" s="10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="Q29" s="9">
         <v>46157</v>
@@ -3392,12 +3406,12 @@
         <v>0</v>
       </c>
       <c r="U29" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B30" s="5">
         <v>46149.168830532406</v>
@@ -3409,16 +3423,16 @@
         <v>46199.75283171296</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F30" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G30" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="H30" s="6" t="s">
         <v>96</v>
-      </c>
-      <c r="H30" s="6" t="s">
-        <v>97</v>
       </c>
       <c r="I30" s="5">
         <v>46157</v>
@@ -3436,29 +3450,29 @@
         <v>26</v>
       </c>
       <c r="N30" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="O30" s="6" t="s">
         <v>66</v>
       </c>
       <c r="P30" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="Q30" s="6"/>
       <c r="R30" s="6"/>
       <c r="S30" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T30" s="6">
         <v>0</v>
       </c>
       <c r="U30" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B31" s="9">
         <v>46149.1688349537</v>
@@ -3468,16 +3482,16 @@
         <v>46199.752836423606</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F31" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G31" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="H31" s="10" t="s">
         <v>96</v>
-      </c>
-      <c r="H31" s="10" t="s">
-        <v>97</v>
       </c>
       <c r="I31" s="9">
         <v>46168</v>
@@ -3495,29 +3509,29 @@
         <v>26</v>
       </c>
       <c r="N31" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="O31" s="10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="P31" s="10" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="Q31" s="10"/>
       <c r="R31" s="10"/>
       <c r="S31" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T31" s="10">
         <v>0</v>
       </c>
       <c r="U31" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B32" s="5">
         <v>46149.16884</v>
@@ -3529,16 +3543,16 @@
         <v>46199.752879155094</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F32" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G32" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="H32" s="6" t="s">
         <v>96</v>
-      </c>
-      <c r="H32" s="6" t="s">
-        <v>97</v>
       </c>
       <c r="I32" s="5">
         <v>46168</v>
@@ -3556,29 +3570,29 @@
         <v>26</v>
       </c>
       <c r="N32" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="O32" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="P32" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Q32" s="6"/>
       <c r="R32" s="6"/>
       <c r="S32" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T32" s="6">
         <v>0</v>
       </c>
       <c r="U32" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B33" s="9">
         <v>46149.168844375</v>
@@ -3588,16 +3602,16 @@
         <v>46200.194168518516</v>
       </c>
       <c r="E33" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="F33" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G33" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="F33" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G33" s="10" t="s">
+      <c r="H33" s="10" t="s">
         <v>130</v>
-      </c>
-      <c r="H33" s="10" t="s">
-        <v>131</v>
       </c>
       <c r="I33" s="9">
         <v>46189</v>
@@ -3615,13 +3629,13 @@
         <v>26</v>
       </c>
       <c r="N33" s="10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="O33" s="10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="P33" s="10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="Q33" s="9">
         <v>46189</v>
@@ -3636,31 +3650,31 @@
         <v>0</v>
       </c>
       <c r="U33" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B34" s="5">
         <v>46149.16884893518</v>
       </c>
       <c r="C34" s="6"/>
       <c r="D34" s="5">
-        <v>46190.16888383102</v>
+        <v>46204.91286611111</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F34" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G34" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="H34" s="6" t="s">
         <v>130</v>
-      </c>
-      <c r="H34" s="6" t="s">
-        <v>131</v>
       </c>
       <c r="I34" s="5">
         <v>46189</v>
@@ -3678,29 +3692,29 @@
         <v>26</v>
       </c>
       <c r="N34" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="O34" s="6" t="s">
         <v>76</v>
       </c>
       <c r="P34" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="Q34" s="6"/>
       <c r="R34" s="6"/>
       <c r="S34" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T34" s="6">
         <v>0</v>
       </c>
       <c r="U34" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B35" s="9">
         <v>46149.16885364584</v>
@@ -3710,16 +3724,16 @@
         <v>46199.16976567129</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F35" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G35" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="H35" s="10" t="s">
         <v>130</v>
-      </c>
-      <c r="H35" s="10" t="s">
-        <v>131</v>
       </c>
       <c r="I35" s="9">
         <v>46191</v>
@@ -3737,29 +3751,29 @@
         <v>26</v>
       </c>
       <c r="N35" s="10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="O35" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="P35" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="Q35" s="10"/>
       <c r="R35" s="10"/>
       <c r="S35" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T35" s="10">
         <v>0</v>
       </c>
       <c r="U35" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B36" s="5">
         <v>46149.1688584375</v>
@@ -3769,16 +3783,16 @@
         <v>46200.194168437505</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F36" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G36" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="H36" s="6" t="s">
         <v>130</v>
-      </c>
-      <c r="H36" s="6" t="s">
-        <v>131</v>
       </c>
       <c r="I36" s="5">
         <v>46189</v>
@@ -3796,10 +3810,10 @@
         <v>26</v>
       </c>
       <c r="N36" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="O36" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P36" s="6" t="s">
         <v>26</v>
@@ -3817,31 +3831,31 @@
         <v>0</v>
       </c>
       <c r="U36" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" s="8" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B37" s="9">
         <v>46149.16891136574</v>
       </c>
       <c r="C37" s="10"/>
       <c r="D37" s="9">
-        <v>46190.16888201389</v>
+        <v>46204.91289927083</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F37" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G37" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="H37" s="10" t="s">
         <v>130</v>
-      </c>
-      <c r="H37" s="10" t="s">
-        <v>131</v>
       </c>
       <c r="I37" s="9">
         <v>46189</v>
@@ -3859,13 +3873,13 @@
         <v>26</v>
       </c>
       <c r="N37" s="10" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="O37" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="P37" s="10" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="Q37" s="10"/>
       <c r="R37" s="10"/>
@@ -3875,7 +3889,7 @@
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B38" s="5">
         <v>46149.168917256946</v>
@@ -3885,16 +3899,16 @@
         <v>46199.16976444444</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F38" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G38" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="H38" s="6" t="s">
         <v>130</v>
-      </c>
-      <c r="H38" s="6" t="s">
-        <v>131</v>
       </c>
       <c r="I38" s="5">
         <v>46191</v>
@@ -3912,13 +3926,13 @@
         <v>26</v>
       </c>
       <c r="N38" s="6" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="O38" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P38" s="6" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="Q38" s="6"/>
       <c r="R38" s="6"/>
@@ -3928,7 +3942,7 @@
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" s="8" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B39" s="9">
         <v>46149.16892260416</v>
@@ -3938,16 +3952,16 @@
         <v>46169.859801203704</v>
       </c>
       <c r="E39" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="F39" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G39" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="F39" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G39" s="10" t="s">
+      <c r="H39" s="10" t="s">
         <v>149</v>
-      </c>
-      <c r="H39" s="10" t="s">
-        <v>150</v>
       </c>
       <c r="I39" s="9">
         <v>46189</v>
@@ -3965,10 +3979,10 @@
         <v>26</v>
       </c>
       <c r="N39" s="10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="O39" s="10" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="P39" s="10" t="s">
         <v>26</v>
@@ -3980,37 +3994,37 @@
         <v>46230</v>
       </c>
       <c r="S39" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T39" s="10">
         <v>0</v>
       </c>
       <c r="U39" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B40" s="5">
         <v>46149.168932870365</v>
       </c>
       <c r="C40" s="6"/>
       <c r="D40" s="5">
-        <v>46197.16885377315</v>
+        <v>46204.91187768518</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F40" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G40" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="H40" s="6" t="s">
         <v>149</v>
-      </c>
-      <c r="H40" s="6" t="s">
-        <v>150</v>
       </c>
       <c r="I40" s="5">
         <v>46189</v>
@@ -4028,13 +4042,13 @@
         <v>26</v>
       </c>
       <c r="N40" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="O40" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="P40" s="6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="Q40" s="6"/>
       <c r="R40" s="6"/>
@@ -4044,7 +4058,7 @@
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B41" s="9">
         <v>46149.16893796297</v>
@@ -4054,16 +4068,16 @@
         <v>46169.859942118055</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F41" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G41" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="H41" s="10" t="s">
         <v>149</v>
-      </c>
-      <c r="H41" s="10" t="s">
-        <v>150</v>
       </c>
       <c r="I41" s="9">
         <v>46198</v>
@@ -4081,13 +4095,13 @@
         <v>26</v>
       </c>
       <c r="N41" s="10" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="O41" s="10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="P41" s="10" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="Q41" s="10"/>
       <c r="R41" s="10"/>
@@ -4097,7 +4111,7 @@
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B42" s="5">
         <v>46149.16894290509</v>
@@ -4107,16 +4121,16 @@
         <v>46169.859966018514</v>
       </c>
       <c r="E42" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="F42" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G42" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="F42" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G42" s="6" t="s">
+      <c r="H42" s="6" t="s">
         <v>159</v>
-      </c>
-      <c r="H42" s="6" t="s">
-        <v>160</v>
       </c>
       <c r="I42" s="5">
         <v>46227</v>
@@ -4134,10 +4148,10 @@
         <v>26</v>
       </c>
       <c r="N42" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="O42" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="P42" s="6" t="s">
         <v>26</v>
@@ -4150,7 +4164,7 @@
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="8" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B43" s="9">
         <v>46149.16894577546</v>
@@ -4160,16 +4174,16 @@
         <v>46203.185002569444</v>
       </c>
       <c r="E43" s="10" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F43" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G43" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="H43" s="10" t="s">
         <v>130</v>
-      </c>
-      <c r="H43" s="10" t="s">
-        <v>131</v>
       </c>
       <c r="I43" s="9">
         <v>46189</v>
@@ -4187,10 +4201,10 @@
         <v>26</v>
       </c>
       <c r="N43" s="10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="O43" s="10" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="P43" s="10" t="s">
         <v>26</v>
@@ -4202,37 +4216,37 @@
         <v>46210</v>
       </c>
       <c r="S43" s="12" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="T43" s="10">
         <v>0</v>
       </c>
       <c r="U43" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B44" s="5">
         <v>46149.16894971065</v>
       </c>
       <c r="C44" s="6"/>
       <c r="D44" s="5">
-        <v>46191.68554611111</v>
+        <v>46204.91205900463</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F44" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G44" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="H44" s="6" t="s">
         <v>130</v>
-      </c>
-      <c r="H44" s="6" t="s">
-        <v>131</v>
       </c>
       <c r="I44" s="5">
         <v>46189</v>
@@ -4250,13 +4264,13 @@
         <v>26</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="O44" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="P44" s="6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="Q44" s="6"/>
       <c r="R44" s="6"/>
@@ -4266,7 +4280,7 @@
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B45" s="9">
         <v>46149.1689542824</v>
@@ -4276,16 +4290,16 @@
         <v>46191.68560096065</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F45" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G45" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="H45" s="10" t="s">
         <v>130</v>
-      </c>
-      <c r="H45" s="10" t="s">
-        <v>131</v>
       </c>
       <c r="I45" s="9">
         <v>46191</v>
@@ -4303,13 +4317,13 @@
         <v>26</v>
       </c>
       <c r="N45" s="10" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="O45" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="P45" s="10" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="Q45" s="10"/>
       <c r="R45" s="10"/>
@@ -4319,7 +4333,7 @@
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B46" s="5">
         <v>46149.16868141203</v>
@@ -4329,7 +4343,7 @@
         <v>46199.77902613426</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F46" s="6" t="s">
         <v>25</v>
@@ -4353,7 +4367,7 @@
         <v>26</v>
       </c>
       <c r="O46" s="6" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="P46" s="6" t="s">
         <v>26</v>
@@ -4363,7 +4377,7 @@
       <c r="S46" s="6"/>
       <c r="T46" s="6"/>
       <c r="U46" s="12" t="s">
-        <v>81</v>
+        <v>172</v>
       </c>
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
@@ -4407,7 +4421,7 @@
         <v>26</v>
       </c>
       <c r="N47" s="10" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="O47" s="10" t="s">
         <v>60</v>
@@ -4472,7 +4486,7 @@
         <v>26</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="O48" s="6" t="s">
         <v>180</v>
@@ -4535,7 +4549,7 @@
         <v>26</v>
       </c>
       <c r="N49" s="10" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="O49" s="10" t="s">
         <v>179</v>
@@ -4550,7 +4564,7 @@
         <v>46153</v>
       </c>
       <c r="S49" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T49" s="10">
         <v>1</v>
@@ -4598,7 +4612,7 @@
         <v>26</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="O50" s="6" t="s">
         <v>190</v>
@@ -4613,13 +4627,13 @@
         <v>46241</v>
       </c>
       <c r="S50" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T50" s="6">
         <v>0</v>
       </c>
       <c r="U50" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
@@ -4915,7 +4929,7 @@
         <v>198</v>
       </c>
       <c r="O56" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="P56" s="6" t="s">
         <v>204</v>
@@ -4933,7 +4947,7 @@
         <v>0</v>
       </c>
       <c r="U56" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
@@ -4954,10 +4968,10 @@
         <v>26</v>
       </c>
       <c r="G57" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="H57" s="10" t="s">
         <v>159</v>
-      </c>
-      <c r="H57" s="10" t="s">
-        <v>160</v>
       </c>
       <c r="I57" s="9">
         <v>46204</v>
@@ -4996,7 +5010,7 @@
         <v>0</v>
       </c>
       <c r="U57" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
@@ -5041,7 +5055,7 @@
         <v>198</v>
       </c>
       <c r="O58" s="6" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="P58" s="6" t="s">
         <v>211</v>
@@ -5059,7 +5073,7 @@
         <v>0</v>
       </c>
       <c r="U58" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
@@ -5080,10 +5094,10 @@
         <v>26</v>
       </c>
       <c r="G59" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="H59" s="10" t="s">
         <v>159</v>
-      </c>
-      <c r="H59" s="10" t="s">
-        <v>160</v>
       </c>
       <c r="I59" s="9">
         <v>46204</v>
@@ -5122,7 +5136,7 @@
         <v>0</v>
       </c>
       <c r="U59" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
@@ -5167,7 +5181,7 @@
         <v>198</v>
       </c>
       <c r="O60" s="6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="P60" s="6" t="s">
         <v>217</v>
@@ -5179,13 +5193,13 @@
         <v>46212</v>
       </c>
       <c r="S60" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T60" s="6">
         <v>0</v>
       </c>
       <c r="U60" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
@@ -5206,10 +5220,10 @@
         <v>26</v>
       </c>
       <c r="G61" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="H61" s="10" t="s">
         <v>159</v>
-      </c>
-      <c r="H61" s="10" t="s">
-        <v>160</v>
       </c>
       <c r="I61" s="9">
         <v>46213</v>
@@ -5242,13 +5256,13 @@
         <v>46216</v>
       </c>
       <c r="S61" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T61" s="10">
         <v>0</v>
       </c>
       <c r="U61" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
@@ -5352,13 +5366,13 @@
         <v>46219</v>
       </c>
       <c r="S63" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T63" s="10">
         <v>0</v>
       </c>
       <c r="U63" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
@@ -5627,13 +5641,13 @@
         <v>46226</v>
       </c>
       <c r="S68" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T68" s="6">
         <v>0</v>
       </c>
       <c r="U68" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
@@ -5866,10 +5880,10 @@
         <v>26</v>
       </c>
       <c r="G73" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="H73" s="10" t="s">
         <v>159</v>
-      </c>
-      <c r="H73" s="10" t="s">
-        <v>160</v>
       </c>
       <c r="I73" s="9">
         <v>46227</v>
@@ -5902,13 +5916,13 @@
         <v>46227</v>
       </c>
       <c r="S73" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T73" s="10">
         <v>0</v>
       </c>
       <c r="U73" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
@@ -5929,10 +5943,10 @@
         <v>26</v>
       </c>
       <c r="G74" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="H74" s="6" t="s">
         <v>159</v>
-      </c>
-      <c r="H74" s="6" t="s">
-        <v>160</v>
       </c>
       <c r="I74" s="5">
         <v>46227</v>
@@ -5982,10 +5996,10 @@
         <v>26</v>
       </c>
       <c r="G75" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="H75" s="10" t="s">
         <v>159</v>
-      </c>
-      <c r="H75" s="10" t="s">
-        <v>160</v>
       </c>
       <c r="I75" s="9">
         <v>46227</v>
@@ -6035,10 +6049,10 @@
         <v>26</v>
       </c>
       <c r="G76" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="H76" s="6" t="s">
         <v>159</v>
-      </c>
-      <c r="H76" s="6" t="s">
-        <v>160</v>
       </c>
       <c r="I76" s="5">
         <v>46227</v>
@@ -6088,10 +6102,10 @@
         <v>26</v>
       </c>
       <c r="G77" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="H77" s="10" t="s">
         <v>159</v>
-      </c>
-      <c r="H77" s="10" t="s">
-        <v>160</v>
       </c>
       <c r="I77" s="9">
         <v>46227</v>
@@ -6210,7 +6224,7 @@
         <v>198</v>
       </c>
       <c r="O79" s="10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="P79" s="10" t="s">
         <v>256</v>
@@ -6228,7 +6242,7 @@
         <v>0</v>
       </c>
       <c r="U79" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
@@ -6273,7 +6287,7 @@
         <v>198</v>
       </c>
       <c r="O80" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="P80" s="6" t="s">
         <v>259</v>
@@ -6291,7 +6305,7 @@
         <v>0</v>
       </c>
       <c r="U80" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
@@ -6336,7 +6350,7 @@
         <v>198</v>
       </c>
       <c r="O81" s="10" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="P81" s="10" t="s">
         <v>259</v>
@@ -6354,7 +6368,7 @@
         <v>0</v>
       </c>
       <c r="U81" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
@@ -6399,7 +6413,7 @@
         <v>198</v>
       </c>
       <c r="O82" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="P82" s="6" t="s">
         <v>264</v>
@@ -6411,13 +6425,13 @@
         <v>46231</v>
       </c>
       <c r="S82" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T82" s="6">
         <v>0</v>
       </c>
       <c r="U82" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">
@@ -6521,13 +6535,13 @@
         <v>46234</v>
       </c>
       <c r="S84" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T84" s="6">
         <v>0</v>
       </c>
       <c r="U84" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="85" spans="1:21" x14ac:dyDescent="0.25">
@@ -6796,13 +6810,13 @@
         <v>46237</v>
       </c>
       <c r="S89" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T89" s="10">
         <v>0</v>
       </c>
       <c r="U89" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="90" spans="1:21" x14ac:dyDescent="0.25">
@@ -7063,13 +7077,13 @@
         <v>46238</v>
       </c>
       <c r="S94" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T94" s="6">
         <v>0</v>
       </c>
       <c r="U94" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="95" spans="1:21" x14ac:dyDescent="0.25">
@@ -7330,13 +7344,13 @@
         <v>46239</v>
       </c>
       <c r="S99" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T99" s="10">
         <v>0</v>
       </c>
       <c r="U99" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="100" spans="1:21" x14ac:dyDescent="0.25">
@@ -7597,13 +7611,13 @@
         <v>46240</v>
       </c>
       <c r="S104" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T104" s="6">
         <v>0</v>
       </c>
       <c r="U104" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="105" spans="1:21" x14ac:dyDescent="0.25">
@@ -7872,13 +7886,13 @@
         <v>46244</v>
       </c>
       <c r="S109" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T109" s="10">
         <v>0</v>
       </c>
       <c r="U109" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="110" spans="1:21" x14ac:dyDescent="0.25">
@@ -8184,13 +8198,13 @@
         <v>46245</v>
       </c>
       <c r="S115" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T115" s="10">
         <v>0</v>
       </c>
       <c r="U115" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="116" spans="1:21" x14ac:dyDescent="0.25">
@@ -8451,13 +8465,13 @@
         <v>46246</v>
       </c>
       <c r="S120" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T120" s="6">
         <v>0</v>
       </c>
       <c r="U120" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="121" spans="1:21" x14ac:dyDescent="0.25">
@@ -8726,13 +8740,13 @@
         <v>46247</v>
       </c>
       <c r="S125" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T125" s="10">
         <v>0</v>
       </c>
       <c r="U125" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="126" spans="1:21" x14ac:dyDescent="0.25">
@@ -8993,13 +9007,13 @@
         <v>46248</v>
       </c>
       <c r="S130" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T130" s="6">
         <v>0</v>
       </c>
       <c r="U130" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="131" spans="1:21" x14ac:dyDescent="0.25">
@@ -9307,13 +9321,13 @@
         <v>46255</v>
       </c>
       <c r="S136" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T136" s="6">
         <v>0</v>
       </c>
       <c r="U136" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="137" spans="1:21" x14ac:dyDescent="0.25">
@@ -9370,13 +9384,13 @@
         <v>46255</v>
       </c>
       <c r="S137" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="T137" s="10">
         <v>0</v>
       </c>
       <c r="U137" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-07-02 21:07 UTC
</commit_message>
<xml_diff>
--- a/data/50001545 - XEMORTIZ MINERA FRISCO.xlsx
+++ b/data/50001545 - XEMORTIZ MINERA FRISCO.xlsx
@@ -3959,9 +3959,11 @@
       <c r="B39" s="9">
         <v>46149.16892260416</v>
       </c>
-      <c r="C39" s="10"/>
+      <c r="C39" s="9">
+        <v>46205.843624166664</v>
+      </c>
       <c r="D39" s="9">
-        <v>46169.859801203704</v>
+        <v>46205.84364175926</v>
       </c>
       <c r="E39" s="10" t="s">
         <v>147</v>
@@ -4009,10 +4011,10 @@
         <v>102</v>
       </c>
       <c r="T39" s="10">
-        <v>0</v>
-      </c>
-      <c r="U39" s="11" t="s">
-        <v>98</v>
+        <v>1</v>
+      </c>
+      <c r="U39" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
@@ -4022,9 +4024,11 @@
       <c r="B40" s="5">
         <v>46149.168932870365</v>
       </c>
-      <c r="C40" s="6"/>
+      <c r="C40" s="5">
+        <v>46205.8435071412</v>
+      </c>
       <c r="D40" s="5">
-        <v>46204.91187768518</v>
+        <v>46205.843509259255</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>89</v>
@@ -4075,9 +4079,11 @@
       <c r="B41" s="9">
         <v>46149.16893796297</v>
       </c>
-      <c r="C41" s="10"/>
+      <c r="C41" s="9">
+        <v>46205.84357833333</v>
+      </c>
       <c r="D41" s="9">
-        <v>46169.859942118055</v>
+        <v>46205.84357975694</v>
       </c>
       <c r="E41" s="10" t="s">
         <v>154</v>
@@ -4130,7 +4136,7 @@
       </c>
       <c r="C42" s="6"/>
       <c r="D42" s="5">
-        <v>46169.859966018514</v>
+        <v>46205.843587766205</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>157</v>
@@ -6398,7 +6404,7 @@
       </c>
       <c r="C82" s="6"/>
       <c r="D82" s="5">
-        <v>46155.59985006944</v>
+        <v>46205.84359559028</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>263</v>
@@ -6448,8 +6454,8 @@
       <c r="T82" s="6">
         <v>0</v>
       </c>
-      <c r="U82" s="11" t="s">
-        <v>98</v>
+      <c r="U82" s="12" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
KPI actualizado 2026-07-09 16:35 UTC
</commit_message>
<xml_diff>
--- a/data/50001545 - XEMORTIZ MINERA FRISCO.xlsx
+++ b/data/50001545 - XEMORTIZ MINERA FRISCO.xlsx
@@ -366,19 +366,19 @@
     <t>Generación OC Alabe OT 4315,Fabricación Alabe OT 4315</t>
   </si>
   <si>
+    <t>1214596734036226</t>
+  </si>
+  <si>
+    <t>Generación OC Alabe OT 4315</t>
+  </si>
+  <si>
+    <t>Alabe OT 4315,Fabricación Alabe OT 4315</t>
+  </si>
+  <si>
+    <t>Baja</t>
+  </si>
+  <si>
     <t>Tarea sin iniciar</t>
-  </si>
-  <si>
-    <t>1214596734036226</t>
-  </si>
-  <si>
-    <t>Generación OC Alabe OT 4315</t>
-  </si>
-  <si>
-    <t>Alabe OT 4315,Fabricación Alabe OT 4315</t>
-  </si>
-  <si>
-    <t>Baja</t>
   </si>
   <si>
     <t>1214596725445208</t>
@@ -2946,7 +2946,7 @@
       </c>
       <c r="C22" s="6"/>
       <c r="D22" s="5">
-        <v>46205.60770953704</v>
+        <v>46212.66494016204</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>91</v>
@@ -2991,9 +2991,11 @@
       <c r="B23" s="9">
         <v>46149.168800127314</v>
       </c>
-      <c r="C23" s="10"/>
+      <c r="C23" s="9">
+        <v>46212.664802025465</v>
+      </c>
       <c r="D23" s="9">
-        <v>46169.85973167824</v>
+        <v>46212.66481476852</v>
       </c>
       <c r="E23" s="10" t="s">
         <v>94</v>
@@ -3041,25 +3043,27 @@
         <v>33</v>
       </c>
       <c r="T23" s="10">
-        <v>0</v>
-      </c>
-      <c r="U23" s="11" t="s">
-        <v>98</v>
+        <v>1</v>
+      </c>
+      <c r="U23" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B24" s="5">
         <v>46149.168804155095</v>
       </c>
-      <c r="C24" s="6"/>
+      <c r="C24" s="5">
+        <v>46212.664752557874</v>
+      </c>
       <c r="D24" s="5">
-        <v>46196.87158508102</v>
+        <v>46212.66475459491</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>26</v>
@@ -3092,18 +3096,18 @@
         <v>69</v>
       </c>
       <c r="P24" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="Q24" s="6"/>
       <c r="R24" s="6"/>
       <c r="S24" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T24" s="6">
         <v>0</v>
       </c>
       <c r="U24" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
@@ -3113,9 +3117,11 @@
       <c r="B25" s="9">
         <v>46149.16880861111</v>
       </c>
-      <c r="C25" s="10"/>
+      <c r="C25" s="9">
+        <v>46212.66478641204</v>
+      </c>
       <c r="D25" s="9">
-        <v>46169.86022740741</v>
+        <v>46212.66478789352</v>
       </c>
       <c r="E25" s="10" t="s">
         <v>104</v>
@@ -3148,7 +3154,7 @@
         <v>94</v>
       </c>
       <c r="O25" s="10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="P25" s="10" t="s">
         <v>105</v>
@@ -3156,13 +3162,13 @@
       <c r="Q25" s="10"/>
       <c r="R25" s="10"/>
       <c r="S25" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T25" s="10">
         <v>0</v>
       </c>
       <c r="U25" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
@@ -3172,9 +3178,11 @@
       <c r="B26" s="5">
         <v>46149.16881337963</v>
       </c>
-      <c r="C26" s="6"/>
+      <c r="C26" s="5">
+        <v>46212.664931990745</v>
+      </c>
       <c r="D26" s="5">
-        <v>46179.17667454861</v>
+        <v>46212.66494965278</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>107</v>
@@ -3222,10 +3230,10 @@
         <v>33</v>
       </c>
       <c r="T26" s="6">
-        <v>0</v>
-      </c>
-      <c r="U26" s="11" t="s">
-        <v>98</v>
+        <v>1</v>
+      </c>
+      <c r="U26" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
@@ -3235,9 +3243,11 @@
       <c r="B27" s="9">
         <v>46149.16881752315</v>
       </c>
-      <c r="C27" s="10"/>
+      <c r="C27" s="9">
+        <v>46212.66487011574</v>
+      </c>
       <c r="D27" s="9">
-        <v>46197.50269849537</v>
+        <v>46212.664871597226</v>
       </c>
       <c r="E27" s="10" t="s">
         <v>110</v>
@@ -3278,13 +3288,13 @@
       <c r="Q27" s="10"/>
       <c r="R27" s="10"/>
       <c r="S27" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T27" s="10">
         <v>0</v>
       </c>
       <c r="U27" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
@@ -3294,9 +3304,11 @@
       <c r="B28" s="5">
         <v>46149.168821851854</v>
       </c>
-      <c r="C28" s="6"/>
+      <c r="C28" s="5">
+        <v>46212.66491304398</v>
+      </c>
       <c r="D28" s="5">
-        <v>46178.170599363424</v>
+        <v>46212.664914918976</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>113</v>
@@ -3337,13 +3349,13 @@
       <c r="Q28" s="6"/>
       <c r="R28" s="6"/>
       <c r="S28" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T28" s="6">
         <v>0</v>
       </c>
       <c r="U28" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
@@ -3406,7 +3418,7 @@
         <v>0</v>
       </c>
       <c r="U29" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
@@ -3461,13 +3473,13 @@
       <c r="Q30" s="6"/>
       <c r="R30" s="6"/>
       <c r="S30" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T30" s="6">
         <v>0</v>
       </c>
       <c r="U30" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
@@ -3520,13 +3532,13 @@
       <c r="Q31" s="10"/>
       <c r="R31" s="10"/>
       <c r="S31" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T31" s="10">
         <v>0</v>
       </c>
       <c r="U31" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
@@ -3581,13 +3593,13 @@
       <c r="Q32" s="6"/>
       <c r="R32" s="6"/>
       <c r="S32" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T32" s="6">
         <v>0</v>
       </c>
       <c r="U32" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
@@ -3707,13 +3719,13 @@
       <c r="Q34" s="6"/>
       <c r="R34" s="6"/>
       <c r="S34" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T34" s="6">
         <v>0</v>
       </c>
       <c r="U34" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
@@ -3768,13 +3780,13 @@
       <c r="Q35" s="10"/>
       <c r="R35" s="10"/>
       <c r="S35" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T35" s="10">
         <v>0</v>
       </c>
       <c r="U35" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
@@ -4008,7 +4020,7 @@
         <v>46230</v>
       </c>
       <c r="S39" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T39" s="10">
         <v>1</v>
@@ -4588,7 +4600,7 @@
         <v>46153</v>
       </c>
       <c r="S49" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T49" s="10">
         <v>1</v>
@@ -4651,13 +4663,13 @@
         <v>46241</v>
       </c>
       <c r="S50" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T50" s="6">
         <v>0</v>
       </c>
       <c r="U50" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
@@ -5034,7 +5046,7 @@
         <v>0</v>
       </c>
       <c r="U57" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
@@ -5160,7 +5172,7 @@
         <v>0</v>
       </c>
       <c r="U59" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
@@ -5286,7 +5298,7 @@
         <v>0</v>
       </c>
       <c r="U61" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
@@ -5396,7 +5408,7 @@
         <v>0</v>
       </c>
       <c r="U63" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
@@ -5665,13 +5677,13 @@
         <v>46226</v>
       </c>
       <c r="S68" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T68" s="6">
         <v>0</v>
       </c>
       <c r="U68" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
@@ -5940,13 +5952,13 @@
         <v>46227</v>
       </c>
       <c r="S73" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T73" s="10">
         <v>0</v>
       </c>
       <c r="U73" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
@@ -6170,7 +6182,7 @@
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46155.57120092593</v>
+        <v>46212.66505685185</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>197</v>
@@ -6215,9 +6227,11 @@
       <c r="B79" s="9">
         <v>46149.16913708333</v>
       </c>
-      <c r="C79" s="10"/>
+      <c r="C79" s="9">
+        <v>46212.66504260417</v>
+      </c>
       <c r="D79" s="9">
-        <v>46182.17098876157</v>
+        <v>46212.66505976852</v>
       </c>
       <c r="E79" s="10" t="s">
         <v>255</v>
@@ -6263,10 +6277,10 @@
         <v>33</v>
       </c>
       <c r="T79" s="10">
-        <v>0</v>
-      </c>
-      <c r="U79" s="11" t="s">
-        <v>98</v>
+        <v>1</v>
+      </c>
+      <c r="U79" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
@@ -6276,9 +6290,11 @@
       <c r="B80" s="5">
         <v>46149.16914224537</v>
       </c>
-      <c r="C80" s="6"/>
+      <c r="C80" s="5">
+        <v>46212.665051261574</v>
+      </c>
       <c r="D80" s="5">
-        <v>46165.180999432865</v>
+        <v>46212.66506702546</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>258</v>
@@ -6326,10 +6342,10 @@
         <v>33</v>
       </c>
       <c r="T80" s="6">
-        <v>0</v>
-      </c>
-      <c r="U80" s="11" t="s">
-        <v>98</v>
+        <v>1</v>
+      </c>
+      <c r="U80" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
@@ -6392,7 +6408,7 @@
         <v>0</v>
       </c>
       <c r="U81" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
@@ -6449,7 +6465,7 @@
         <v>46231</v>
       </c>
       <c r="S82" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T82" s="6">
         <v>0</v>
@@ -6559,13 +6575,13 @@
         <v>46234</v>
       </c>
       <c r="S84" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T84" s="6">
         <v>0</v>
       </c>
       <c r="U84" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="85" spans="1:21" x14ac:dyDescent="0.25">
@@ -6834,13 +6850,13 @@
         <v>46237</v>
       </c>
       <c r="S89" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T89" s="10">
         <v>0</v>
       </c>
       <c r="U89" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="90" spans="1:21" x14ac:dyDescent="0.25">
@@ -6852,7 +6868,7 @@
       </c>
       <c r="C90" s="6"/>
       <c r="D90" s="5">
-        <v>46199.77908100694</v>
+        <v>46212.6650581713</v>
       </c>
       <c r="E90" s="6" t="s">
         <v>191</v>
@@ -6903,7 +6919,7 @@
       </c>
       <c r="C91" s="10"/>
       <c r="D91" s="9">
-        <v>46199.77908144676</v>
+        <v>46212.665059328705</v>
       </c>
       <c r="E91" s="10" t="s">
         <v>191</v>
@@ -6954,7 +6970,7 @@
       </c>
       <c r="C92" s="6"/>
       <c r="D92" s="5">
-        <v>46199.77908483797</v>
+        <v>46212.66505967593</v>
       </c>
       <c r="E92" s="6" t="s">
         <v>191</v>
@@ -7005,7 +7021,7 @@
       </c>
       <c r="C93" s="10"/>
       <c r="D93" s="9">
-        <v>46199.779085277776</v>
+        <v>46212.66506008102</v>
       </c>
       <c r="E93" s="10" t="s">
         <v>191</v>
@@ -7101,13 +7117,13 @@
         <v>46238</v>
       </c>
       <c r="S94" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T94" s="6">
         <v>0</v>
       </c>
       <c r="U94" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="95" spans="1:21" x14ac:dyDescent="0.25">
@@ -7119,7 +7135,7 @@
       </c>
       <c r="C95" s="10"/>
       <c r="D95" s="9">
-        <v>46199.779080567125</v>
+        <v>46212.665048483796</v>
       </c>
       <c r="E95" s="10" t="s">
         <v>191</v>
@@ -7170,7 +7186,7 @@
       </c>
       <c r="C96" s="6"/>
       <c r="D96" s="5">
-        <v>46199.779077430554</v>
+        <v>46212.66504763889</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>191</v>
@@ -7221,7 +7237,7 @@
       </c>
       <c r="C97" s="10"/>
       <c r="D97" s="9">
-        <v>46199.779084340276</v>
+        <v>46212.665048993054</v>
       </c>
       <c r="E97" s="10" t="s">
         <v>191</v>
@@ -7272,7 +7288,7 @@
       </c>
       <c r="C98" s="6"/>
       <c r="D98" s="5">
-        <v>46199.779085752314</v>
+        <v>46212.665049456016</v>
       </c>
       <c r="E98" s="6" t="s">
         <v>191</v>
@@ -7368,13 +7384,13 @@
         <v>46239</v>
       </c>
       <c r="S99" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T99" s="10">
         <v>0</v>
       </c>
       <c r="U99" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="100" spans="1:21" x14ac:dyDescent="0.25">
@@ -7635,13 +7651,13 @@
         <v>46240</v>
       </c>
       <c r="S104" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T104" s="6">
         <v>0</v>
       </c>
       <c r="U104" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="105" spans="1:21" x14ac:dyDescent="0.25">
@@ -7910,13 +7926,13 @@
         <v>46244</v>
       </c>
       <c r="S109" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T109" s="10">
         <v>0</v>
       </c>
       <c r="U109" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="110" spans="1:21" x14ac:dyDescent="0.25">
@@ -8222,13 +8238,13 @@
         <v>46245</v>
       </c>
       <c r="S115" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T115" s="10">
         <v>0</v>
       </c>
       <c r="U115" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="116" spans="1:21" x14ac:dyDescent="0.25">
@@ -8489,13 +8505,13 @@
         <v>46246</v>
       </c>
       <c r="S120" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T120" s="6">
         <v>0</v>
       </c>
       <c r="U120" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="121" spans="1:21" x14ac:dyDescent="0.25">
@@ -8764,13 +8780,13 @@
         <v>46247</v>
       </c>
       <c r="S125" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T125" s="10">
         <v>0</v>
       </c>
       <c r="U125" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="126" spans="1:21" x14ac:dyDescent="0.25">
@@ -9031,13 +9047,13 @@
         <v>46248</v>
       </c>
       <c r="S130" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T130" s="6">
         <v>0</v>
       </c>
       <c r="U130" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="131" spans="1:21" x14ac:dyDescent="0.25">
@@ -9345,13 +9361,13 @@
         <v>46255</v>
       </c>
       <c r="S136" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T136" s="6">
         <v>0</v>
       </c>
       <c r="U136" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="137" spans="1:21" x14ac:dyDescent="0.25">
@@ -9408,13 +9424,13 @@
         <v>46255</v>
       </c>
       <c r="S137" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T137" s="10">
         <v>0</v>
       </c>
       <c r="U137" s="11" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Curva S actualizada 2026-07-13 16:38 Chile
</commit_message>
<xml_diff>
--- a/data/50001545 - XEMORTIZ MINERA FRISCO.xlsx
+++ b/data/50001545 - XEMORTIZ MINERA FRISCO.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1610" uniqueCount="374">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1611" uniqueCount="374">
   <si>
     <t>50001545 - XEMORTIZ MINERA FRISCO</t>
   </si>
@@ -4883,9 +4883,11 @@
       <c r="B55" s="9">
         <v>46149.1690050926</v>
       </c>
-      <c r="C55" s="10"/>
+      <c r="C55" s="9">
+        <v>46216.83961519676</v>
+      </c>
       <c r="D55" s="9">
-        <v>46155.55893427083</v>
+        <v>46216.8396287963</v>
       </c>
       <c r="E55" s="10" t="s">
         <v>197</v>
@@ -4920,8 +4922,12 @@
       <c r="Q55" s="10"/>
       <c r="R55" s="10"/>
       <c r="S55" s="10"/>
-      <c r="T55" s="10"/>
-      <c r="U55" s="10"/>
+      <c r="T55" s="10">
+        <v>1</v>
+      </c>
+      <c r="U55" s="7" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
@@ -4930,9 +4936,11 @@
       <c r="B56" s="5">
         <v>46149.16900940972</v>
       </c>
-      <c r="C56" s="6"/>
+      <c r="C56" s="5">
+        <v>46216.839534756946</v>
+      </c>
       <c r="D56" s="5">
-        <v>46205.60769931713</v>
+        <v>46216.83970709491</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>200</v>
@@ -4980,10 +4988,10 @@
         <v>33</v>
       </c>
       <c r="T56" s="6">
-        <v>0</v>
-      </c>
-      <c r="U56" s="12" t="s">
-        <v>171</v>
+        <v>1</v>
+      </c>
+      <c r="U56" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
@@ -4993,9 +5001,11 @@
       <c r="B57" s="9">
         <v>46149.16901516204</v>
       </c>
-      <c r="C57" s="10"/>
+      <c r="C57" s="9">
+        <v>46216.83958197916</v>
+      </c>
       <c r="D57" s="9">
-        <v>46205.16832303241</v>
+        <v>46216.83978594907</v>
       </c>
       <c r="E57" s="10" t="s">
         <v>205</v>
@@ -5043,10 +5053,10 @@
         <v>33</v>
       </c>
       <c r="T57" s="10">
-        <v>0</v>
-      </c>
-      <c r="U57" s="11" t="s">
-        <v>102</v>
+        <v>1</v>
+      </c>
+      <c r="U57" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
@@ -5056,9 +5066,11 @@
       <c r="B58" s="5">
         <v>46149.16902107639</v>
       </c>
-      <c r="C58" s="6"/>
+      <c r="C58" s="5">
+        <v>46216.839544409726</v>
+      </c>
       <c r="D58" s="5">
-        <v>46205.60894056713</v>
+        <v>46216.83981521991</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>209</v>
@@ -5106,10 +5118,10 @@
         <v>33</v>
       </c>
       <c r="T58" s="6">
-        <v>0</v>
-      </c>
-      <c r="U58" s="12" t="s">
-        <v>171</v>
+        <v>1</v>
+      </c>
+      <c r="U58" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
@@ -5119,9 +5131,11 @@
       <c r="B59" s="9">
         <v>46149.16902621528</v>
       </c>
-      <c r="C59" s="10"/>
+      <c r="C59" s="9">
+        <v>46216.83958944444</v>
+      </c>
       <c r="D59" s="9">
-        <v>46205.16831765046</v>
+        <v>46216.83984586806</v>
       </c>
       <c r="E59" s="10" t="s">
         <v>212</v>
@@ -5169,10 +5183,10 @@
         <v>33</v>
       </c>
       <c r="T59" s="10">
-        <v>0</v>
-      </c>
-      <c r="U59" s="11" t="s">
-        <v>102</v>
+        <v>1</v>
+      </c>
+      <c r="U59" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
@@ -5182,9 +5196,11 @@
       <c r="B60" s="5">
         <v>46149.1690303588</v>
       </c>
-      <c r="C60" s="6"/>
+      <c r="C60" s="5">
+        <v>46216.839551620375</v>
+      </c>
       <c r="D60" s="5">
-        <v>46213.20552466435</v>
+        <v>46216.83987789352</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>215</v>
@@ -5232,10 +5248,10 @@
         <v>33</v>
       </c>
       <c r="T60" s="6">
-        <v>0</v>
-      </c>
-      <c r="U60" s="12" t="s">
-        <v>171</v>
+        <v>1</v>
+      </c>
+      <c r="U60" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
@@ -5245,9 +5261,11 @@
       <c r="B61" s="9">
         <v>46149.16903488426</v>
       </c>
-      <c r="C61" s="10"/>
+      <c r="C61" s="9">
+        <v>46216.83960126157</v>
+      </c>
       <c r="D61" s="9">
-        <v>46216.16866572917</v>
+        <v>46216.83990553241</v>
       </c>
       <c r="E61" s="10" t="s">
         <v>216</v>
@@ -5295,10 +5313,10 @@
         <v>218</v>
       </c>
       <c r="T61" s="10">
-        <v>0</v>
-      </c>
-      <c r="U61" s="11" t="s">
-        <v>102</v>
+        <v>1</v>
+      </c>
+      <c r="U61" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
@@ -5420,7 +5438,7 @@
       </c>
       <c r="C64" s="6"/>
       <c r="D64" s="5">
-        <v>46155.59925321759</v>
+        <v>46216.83960648148</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>191</v>
@@ -5473,7 +5491,7 @@
       </c>
       <c r="C65" s="10"/>
       <c r="D65" s="9">
-        <v>46155.59924960649</v>
+        <v>46216.839607754635</v>
       </c>
       <c r="E65" s="10" t="s">
         <v>191</v>
@@ -5526,7 +5544,7 @@
       </c>
       <c r="C66" s="6"/>
       <c r="D66" s="5">
-        <v>46155.59924675926</v>
+        <v>46216.83960883102</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>191</v>
@@ -5579,7 +5597,7 @@
       </c>
       <c r="C67" s="10"/>
       <c r="D67" s="9">
-        <v>46155.59924362268</v>
+        <v>46216.83960983796</v>
       </c>
       <c r="E67" s="10" t="s">
         <v>191</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-13 21:10 UTC
</commit_message>
<xml_diff>
--- a/data/50001545 - XEMORTIZ MINERA FRISCO.xlsx
+++ b/data/50001545 - XEMORTIZ MINERA FRISCO.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1611" uniqueCount="374">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1613" uniqueCount="374">
   <si>
     <t>50001545 - XEMORTIZ MINERA FRISCO</t>
   </si>
@@ -351,6 +351,9 @@
     <t>Motor OT 4315,Alabe OT 4315,rodete OT 4315,Materiales corte Laser OT 4315</t>
   </si>
   <si>
+    <t>Tarea en curso</t>
+  </si>
+  <si>
     <t>1214596734036211</t>
   </si>
   <si>
@@ -583,9 +586,6 @@
   </si>
   <si>
     <t>Planos preliminar,Planos definitivos</t>
-  </si>
-  <si>
-    <t>Tarea en curso</t>
   </si>
   <si>
     <t>1214596624002438</t>
@@ -2946,7 +2946,7 @@
       </c>
       <c r="C22" s="6"/>
       <c r="D22" s="5">
-        <v>46212.66494016204</v>
+        <v>46216.87167356482</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>91</v>
@@ -2982,11 +2982,13 @@
       <c r="R22" s="6"/>
       <c r="S22" s="6"/>
       <c r="T22" s="6"/>
-      <c r="U22" s="6"/>
+      <c r="U22" s="12" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B23" s="9">
         <v>46149.168800127314</v>
@@ -2998,16 +3000,16 @@
         <v>46212.66481476852</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F23" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G23" s="10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H23" s="10" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="I23" s="9">
         <v>46157</v>
@@ -3028,7 +3030,7 @@
         <v>91</v>
       </c>
       <c r="O23" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="P23" s="10" t="s">
         <v>91</v>
@@ -3051,7 +3053,7 @@
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B24" s="5">
         <v>46149.168804155095</v>
@@ -3063,16 +3065,16 @@
         <v>46212.66475459491</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="I24" s="5">
         <v>46157</v>
@@ -3090,29 +3092,29 @@
         <v>26</v>
       </c>
       <c r="N24" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="O24" s="6" t="s">
         <v>69</v>
       </c>
       <c r="P24" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="Q24" s="6"/>
       <c r="R24" s="6"/>
       <c r="S24" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="T24" s="6">
         <v>0</v>
       </c>
       <c r="U24" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B25" s="9">
         <v>46149.16880861111</v>
@@ -3124,16 +3126,16 @@
         <v>46212.66478789352</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F25" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G25" s="10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H25" s="10" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="I25" s="9">
         <v>46161</v>
@@ -3151,29 +3153,29 @@
         <v>26</v>
       </c>
       <c r="N25" s="10" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="O25" s="10" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="P25" s="10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Q25" s="10"/>
       <c r="R25" s="10"/>
       <c r="S25" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="T25" s="10">
         <v>0</v>
       </c>
       <c r="U25" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B26" s="5">
         <v>46149.16881337963</v>
@@ -3185,16 +3187,16 @@
         <v>46212.66494965278</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="I26" s="5">
         <v>46157</v>
@@ -3215,7 +3217,7 @@
         <v>91</v>
       </c>
       <c r="O26" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="P26" s="6" t="s">
         <v>91</v>
@@ -3238,7 +3240,7 @@
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B27" s="9">
         <v>46149.16881752315</v>
@@ -3250,16 +3252,16 @@
         <v>46212.664871597226</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F27" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G27" s="10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H27" s="10" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="I27" s="9">
         <v>46157</v>
@@ -3277,29 +3279,29 @@
         <v>26</v>
       </c>
       <c r="N27" s="10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="O27" s="10" t="s">
         <v>72</v>
       </c>
       <c r="P27" s="10" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="Q27" s="10"/>
       <c r="R27" s="10"/>
       <c r="S27" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="T27" s="10">
         <v>0</v>
       </c>
       <c r="U27" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B28" s="5">
         <v>46149.168821851854</v>
@@ -3311,16 +3313,16 @@
         <v>46212.664914918976</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F28" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="I28" s="5">
         <v>46161</v>
@@ -3338,48 +3340,50 @@
         <v>26</v>
       </c>
       <c r="N28" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="O28" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="P28" s="6" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Q28" s="6"/>
       <c r="R28" s="6"/>
       <c r="S28" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="T28" s="6">
         <v>0</v>
       </c>
       <c r="U28" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B29" s="9">
         <v>46149.1688262963</v>
       </c>
-      <c r="C29" s="10"/>
+      <c r="C29" s="9">
+        <v>46216.871654560186</v>
+      </c>
       <c r="D29" s="9">
-        <v>46199.75288726852</v>
+        <v>46216.87176959491</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F29" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G29" s="10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H29" s="10" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="I29" s="9">
         <v>46157</v>
@@ -3400,7 +3404,7 @@
         <v>91</v>
       </c>
       <c r="O29" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="P29" s="10" t="s">
         <v>91</v>
@@ -3415,15 +3419,15 @@
         <v>33</v>
       </c>
       <c r="T29" s="10">
-        <v>0</v>
-      </c>
-      <c r="U29" s="11" t="s">
-        <v>102</v>
+        <v>1</v>
+      </c>
+      <c r="U29" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B30" s="5">
         <v>46149.168830532406</v>
@@ -3435,16 +3439,16 @@
         <v>46199.75283171296</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F30" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="I30" s="5">
         <v>46157</v>
@@ -3462,48 +3466,50 @@
         <v>26</v>
       </c>
       <c r="N30" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="O30" s="6" t="s">
         <v>66</v>
       </c>
       <c r="P30" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Q30" s="6"/>
       <c r="R30" s="6"/>
       <c r="S30" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="T30" s="6">
         <v>0</v>
       </c>
       <c r="U30" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B31" s="9">
         <v>46149.1688349537</v>
       </c>
-      <c r="C31" s="10"/>
+      <c r="C31" s="9">
+        <v>46216.87163922454</v>
+      </c>
       <c r="D31" s="9">
-        <v>46199.752836423606</v>
+        <v>46216.87164077546</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F31" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G31" s="10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H31" s="10" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="I31" s="9">
         <v>46168</v>
@@ -3521,29 +3527,29 @@
         <v>26</v>
       </c>
       <c r="N31" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="O31" s="10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="P31" s="10" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="Q31" s="10"/>
       <c r="R31" s="10"/>
       <c r="S31" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="T31" s="10">
         <v>0</v>
       </c>
       <c r="U31" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B32" s="5">
         <v>46149.16884</v>
@@ -3555,16 +3561,16 @@
         <v>46199.752879155094</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F32" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="I32" s="5">
         <v>46168</v>
@@ -3582,29 +3588,29 @@
         <v>26</v>
       </c>
       <c r="N32" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="O32" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="P32" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Q32" s="6"/>
       <c r="R32" s="6"/>
       <c r="S32" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="T32" s="6">
         <v>0</v>
       </c>
       <c r="U32" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B33" s="9">
         <v>46149.168844375</v>
@@ -3616,16 +3622,16 @@
         <v>46205.60771266204</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F33" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G33" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H33" s="10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I33" s="9">
         <v>46189</v>
@@ -3646,7 +3652,7 @@
         <v>91</v>
       </c>
       <c r="O33" s="10" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="P33" s="10" t="s">
         <v>91</v>
@@ -3669,7 +3675,7 @@
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B34" s="5">
         <v>46149.16884893518</v>
@@ -3681,16 +3687,16 @@
         <v>46205.60762148148</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F34" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I34" s="5">
         <v>46189</v>
@@ -3708,29 +3714,29 @@
         <v>26</v>
       </c>
       <c r="N34" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="O34" s="6" t="s">
         <v>76</v>
       </c>
       <c r="P34" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q34" s="6"/>
       <c r="R34" s="6"/>
       <c r="S34" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="T34" s="6">
         <v>0</v>
       </c>
       <c r="U34" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B35" s="9">
         <v>46149.16885364584</v>
@@ -3742,16 +3748,16 @@
         <v>46205.60768407407</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F35" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G35" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H35" s="10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I35" s="9">
         <v>46191</v>
@@ -3769,29 +3775,29 @@
         <v>26</v>
       </c>
       <c r="N35" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="O35" s="10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="P35" s="10" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="Q35" s="10"/>
       <c r="R35" s="10"/>
       <c r="S35" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="T35" s="10">
         <v>0</v>
       </c>
       <c r="U35" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B36" s="5">
         <v>46149.1688584375</v>
@@ -3803,16 +3809,16 @@
         <v>46205.608947719906</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F36" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I36" s="5">
         <v>46189</v>
@@ -3833,7 +3839,7 @@
         <v>91</v>
       </c>
       <c r="O36" s="6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="P36" s="6" t="s">
         <v>26</v>
@@ -3856,7 +3862,7 @@
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" s="8" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B37" s="9">
         <v>46149.16891136574</v>
@@ -3874,10 +3880,10 @@
         <v>26</v>
       </c>
       <c r="G37" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H37" s="10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I37" s="9">
         <v>46189</v>
@@ -3895,13 +3901,13 @@
         <v>26</v>
       </c>
       <c r="N37" s="10" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O37" s="10" t="s">
         <v>82</v>
       </c>
       <c r="P37" s="10" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="Q37" s="10"/>
       <c r="R37" s="10"/>
@@ -3911,7 +3917,7 @@
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B38" s="5">
         <v>46149.168917256946</v>
@@ -3923,16 +3929,16 @@
         <v>46205.60892006944</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F38" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I38" s="5">
         <v>46191</v>
@@ -3950,13 +3956,13 @@
         <v>26</v>
       </c>
       <c r="N38" s="6" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O38" s="6" t="s">
         <v>83</v>
       </c>
       <c r="P38" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="Q38" s="6"/>
       <c r="R38" s="6"/>
@@ -3966,7 +3972,7 @@
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" s="8" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B39" s="9">
         <v>46149.16892260416</v>
@@ -3978,16 +3984,16 @@
         <v>46205.84364175926</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F39" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G39" s="10" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H39" s="10" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I39" s="9">
         <v>46189</v>
@@ -4008,7 +4014,7 @@
         <v>91</v>
       </c>
       <c r="O39" s="10" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="P39" s="10" t="s">
         <v>26</v>
@@ -4020,7 +4026,7 @@
         <v>46230</v>
       </c>
       <c r="S39" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="T39" s="10">
         <v>1</v>
@@ -4031,7 +4037,7 @@
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B40" s="5">
         <v>46149.168932870365</v>
@@ -4049,10 +4055,10 @@
         <v>26</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H40" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I40" s="5">
         <v>46189</v>
@@ -4070,13 +4076,13 @@
         <v>26</v>
       </c>
       <c r="N40" s="6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="O40" s="6" t="s">
         <v>88</v>
       </c>
       <c r="P40" s="6" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="Q40" s="6"/>
       <c r="R40" s="6"/>
@@ -4086,7 +4092,7 @@
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B41" s="9">
         <v>46149.16893796297</v>
@@ -4098,16 +4104,16 @@
         <v>46205.84357975694</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F41" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G41" s="10" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H41" s="10" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I41" s="9">
         <v>46198</v>
@@ -4125,13 +4131,13 @@
         <v>26</v>
       </c>
       <c r="N41" s="10" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="O41" s="10" t="s">
         <v>89</v>
       </c>
       <c r="P41" s="10" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="Q41" s="10"/>
       <c r="R41" s="10"/>
@@ -4141,7 +4147,7 @@
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B42" s="5">
         <v>46149.16894290509</v>
@@ -4151,16 +4157,16 @@
         <v>46205.843587766205</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F42" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="I42" s="5">
         <v>46227</v>
@@ -4178,10 +4184,10 @@
         <v>26</v>
       </c>
       <c r="N42" s="6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="O42" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="P42" s="6" t="s">
         <v>26</v>
@@ -4194,7 +4200,7 @@
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="8" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B43" s="9">
         <v>46149.16894577546</v>
@@ -4206,16 +4212,16 @@
         <v>46211.19248402778</v>
       </c>
       <c r="E43" s="10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F43" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G43" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H43" s="10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I43" s="9">
         <v>46189</v>
@@ -4236,7 +4242,7 @@
         <v>91</v>
       </c>
       <c r="O43" s="10" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="P43" s="10" t="s">
         <v>26</v>
@@ -4259,7 +4265,7 @@
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B44" s="5">
         <v>46149.16894971065</v>
@@ -4277,10 +4283,10 @@
         <v>26</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I44" s="5">
         <v>46189</v>
@@ -4298,13 +4304,13 @@
         <v>26</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="O44" s="6" t="s">
         <v>85</v>
       </c>
       <c r="P44" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="Q44" s="6"/>
       <c r="R44" s="6"/>
@@ -4314,7 +4320,7 @@
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" s="8" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B45" s="9">
         <v>46149.1689542824</v>
@@ -4326,16 +4332,16 @@
         <v>46205.61326564815</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F45" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G45" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H45" s="10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I45" s="9">
         <v>46191</v>
@@ -4353,13 +4359,13 @@
         <v>26</v>
       </c>
       <c r="N45" s="10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="O45" s="10" t="s">
         <v>86</v>
       </c>
       <c r="P45" s="10" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="Q45" s="10"/>
       <c r="R45" s="10"/>
@@ -4369,7 +4375,7 @@
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B46" s="5">
         <v>46149.16868141203</v>
@@ -4379,7 +4385,7 @@
         <v>46199.77902613426</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F46" s="6" t="s">
         <v>25</v>
@@ -4403,7 +4409,7 @@
         <v>26</v>
       </c>
       <c r="O46" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P46" s="6" t="s">
         <v>26</v>
@@ -4413,7 +4419,7 @@
       <c r="S46" s="6"/>
       <c r="T46" s="6"/>
       <c r="U46" s="12" t="s">
-        <v>171</v>
+        <v>93</v>
       </c>
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
@@ -4457,7 +4463,7 @@
         <v>26</v>
       </c>
       <c r="N47" s="10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="O47" s="10" t="s">
         <v>60</v>
@@ -4522,7 +4528,7 @@
         <v>26</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="O48" s="6" t="s">
         <v>179</v>
@@ -4585,7 +4591,7 @@
         <v>26</v>
       </c>
       <c r="N49" s="10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="O49" s="10" t="s">
         <v>178</v>
@@ -4600,7 +4606,7 @@
         <v>46153</v>
       </c>
       <c r="S49" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="T49" s="10">
         <v>1</v>
@@ -4648,7 +4654,7 @@
         <v>26</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="O50" s="6" t="s">
         <v>189</v>
@@ -4663,13 +4669,13 @@
         <v>46241</v>
       </c>
       <c r="S50" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="T50" s="6">
         <v>0</v>
       </c>
       <c r="U50" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
@@ -4973,7 +4979,7 @@
         <v>197</v>
       </c>
       <c r="O56" s="6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="P56" s="6" t="s">
         <v>203</v>
@@ -5014,10 +5020,10 @@
         <v>26</v>
       </c>
       <c r="G57" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H57" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="I57" s="9">
         <v>46204</v>
@@ -5103,7 +5109,7 @@
         <v>197</v>
       </c>
       <c r="O58" s="6" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="P58" s="6" t="s">
         <v>210</v>
@@ -5144,10 +5150,10 @@
         <v>26</v>
       </c>
       <c r="G59" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H59" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="I59" s="9">
         <v>46204</v>
@@ -5233,7 +5239,7 @@
         <v>197</v>
       </c>
       <c r="O60" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="P60" s="6" t="s">
         <v>216</v>
@@ -5274,10 +5280,10 @@
         <v>26</v>
       </c>
       <c r="G61" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H61" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="I61" s="9">
         <v>46213</v>
@@ -5426,7 +5432,7 @@
         <v>0</v>
       </c>
       <c r="U63" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
@@ -5695,13 +5701,13 @@
         <v>46226</v>
       </c>
       <c r="S68" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="T68" s="6">
         <v>0</v>
       </c>
       <c r="U68" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
@@ -5934,10 +5940,10 @@
         <v>26</v>
       </c>
       <c r="G73" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H73" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="I73" s="9">
         <v>46227</v>
@@ -5970,13 +5976,13 @@
         <v>46227</v>
       </c>
       <c r="S73" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="T73" s="10">
         <v>0</v>
       </c>
       <c r="U73" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
@@ -5997,10 +6003,10 @@
         <v>26</v>
       </c>
       <c r="G74" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H74" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="I74" s="5">
         <v>46227</v>
@@ -6050,10 +6056,10 @@
         <v>26</v>
       </c>
       <c r="G75" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H75" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="I75" s="9">
         <v>46227</v>
@@ -6103,10 +6109,10 @@
         <v>26</v>
       </c>
       <c r="G76" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="I76" s="5">
         <v>46227</v>
@@ -6156,10 +6162,10 @@
         <v>26</v>
       </c>
       <c r="G77" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H77" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="I77" s="9">
         <v>46227</v>
@@ -6200,7 +6206,7 @@
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46212.66505685185</v>
+        <v>46216.87183908565</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>197</v>
@@ -6236,7 +6242,9 @@
       <c r="R78" s="6"/>
       <c r="S78" s="6"/>
       <c r="T78" s="6"/>
-      <c r="U78" s="6"/>
+      <c r="U78" s="12" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" s="8" t="s">
@@ -6280,7 +6288,7 @@
         <v>197</v>
       </c>
       <c r="O79" s="10" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="P79" s="10" t="s">
         <v>256</v>
@@ -6345,7 +6353,7 @@
         <v>197</v>
       </c>
       <c r="O80" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="P80" s="6" t="s">
         <v>259</v>
@@ -6373,9 +6381,11 @@
       <c r="B81" s="9">
         <v>46149.16914733796</v>
       </c>
-      <c r="C81" s="10"/>
+      <c r="C81" s="9">
+        <v>46216.871819039356</v>
+      </c>
       <c r="D81" s="9">
-        <v>46198.171336064814</v>
+        <v>46216.8718724537</v>
       </c>
       <c r="E81" s="10" t="s">
         <v>261</v>
@@ -6408,7 +6418,7 @@
         <v>197</v>
       </c>
       <c r="O81" s="10" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="P81" s="10" t="s">
         <v>259</v>
@@ -6423,10 +6433,10 @@
         <v>33</v>
       </c>
       <c r="T81" s="10">
-        <v>0</v>
-      </c>
-      <c r="U81" s="11" t="s">
-        <v>102</v>
+        <v>1</v>
+      </c>
+      <c r="U81" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
@@ -6471,7 +6481,7 @@
         <v>197</v>
       </c>
       <c r="O82" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="P82" s="6" t="s">
         <v>264</v>
@@ -6483,13 +6493,13 @@
         <v>46231</v>
       </c>
       <c r="S82" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="T82" s="6">
         <v>0</v>
       </c>
       <c r="U82" s="12" t="s">
-        <v>171</v>
+        <v>93</v>
       </c>
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">
@@ -6593,13 +6603,13 @@
         <v>46234</v>
       </c>
       <c r="S84" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="T84" s="6">
         <v>0</v>
       </c>
       <c r="U84" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="85" spans="1:21" x14ac:dyDescent="0.25">
@@ -6868,13 +6878,13 @@
         <v>46237</v>
       </c>
       <c r="S89" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="T89" s="10">
         <v>0</v>
       </c>
       <c r="U89" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="90" spans="1:21" x14ac:dyDescent="0.25">
@@ -7139,13 +7149,13 @@
         <v>46238</v>
       </c>
       <c r="S94" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="T94" s="6">
         <v>0</v>
       </c>
       <c r="U94" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="95" spans="1:21" x14ac:dyDescent="0.25">
@@ -7410,13 +7420,13 @@
         <v>46239</v>
       </c>
       <c r="S99" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="T99" s="10">
         <v>0</v>
       </c>
       <c r="U99" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="100" spans="1:21" x14ac:dyDescent="0.25">
@@ -7428,7 +7438,7 @@
       </c>
       <c r="C100" s="6"/>
       <c r="D100" s="5">
-        <v>46199.779077858795</v>
+        <v>46216.87182809028</v>
       </c>
       <c r="E100" s="6" t="s">
         <v>191</v>
@@ -7479,7 +7489,7 @@
       </c>
       <c r="C101" s="10"/>
       <c r="D101" s="9">
-        <v>46199.77908177083</v>
+        <v>46216.87182944444</v>
       </c>
       <c r="E101" s="10" t="s">
         <v>191</v>
@@ -7530,7 +7540,7 @@
       </c>
       <c r="C102" s="6"/>
       <c r="D102" s="5">
-        <v>46199.77908608796</v>
+        <v>46216.87183001157</v>
       </c>
       <c r="E102" s="6" t="s">
         <v>191</v>
@@ -7581,7 +7591,7 @@
       </c>
       <c r="C103" s="10"/>
       <c r="D103" s="9">
-        <v>46199.77908645834</v>
+        <v>46216.871830648146</v>
       </c>
       <c r="E103" s="10" t="s">
         <v>191</v>
@@ -7677,13 +7687,13 @@
         <v>46240</v>
       </c>
       <c r="S104" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="T104" s="6">
         <v>0</v>
       </c>
       <c r="U104" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="105" spans="1:21" x14ac:dyDescent="0.25">
@@ -7952,13 +7962,13 @@
         <v>46244</v>
       </c>
       <c r="S109" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="T109" s="10">
         <v>0</v>
       </c>
       <c r="U109" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="110" spans="1:21" x14ac:dyDescent="0.25">
@@ -8264,13 +8274,13 @@
         <v>46245</v>
       </c>
       <c r="S115" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="T115" s="10">
         <v>0</v>
       </c>
       <c r="U115" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="116" spans="1:21" x14ac:dyDescent="0.25">
@@ -8531,13 +8541,13 @@
         <v>46246</v>
       </c>
       <c r="S120" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="T120" s="6">
         <v>0</v>
       </c>
       <c r="U120" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="121" spans="1:21" x14ac:dyDescent="0.25">
@@ -8806,13 +8816,13 @@
         <v>46247</v>
       </c>
       <c r="S125" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="T125" s="10">
         <v>0</v>
       </c>
       <c r="U125" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="126" spans="1:21" x14ac:dyDescent="0.25">
@@ -9073,13 +9083,13 @@
         <v>46248</v>
       </c>
       <c r="S130" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="T130" s="6">
         <v>0</v>
       </c>
       <c r="U130" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="131" spans="1:21" x14ac:dyDescent="0.25">
@@ -9387,13 +9397,13 @@
         <v>46255</v>
       </c>
       <c r="S136" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="T136" s="6">
         <v>0</v>
       </c>
       <c r="U136" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="137" spans="1:21" x14ac:dyDescent="0.25">
@@ -9450,13 +9460,13 @@
         <v>46255</v>
       </c>
       <c r="S137" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="T137" s="10">
         <v>0</v>
       </c>
       <c r="U137" s="11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Curva S actualizada 2026-08-08 09:58 Chile
</commit_message>
<xml_diff>
--- a/data/50001545 - XEMORTIZ MINERA FRISCO.xlsx
+++ b/data/50001545 - XEMORTIZ MINERA FRISCO.xlsx
@@ -639,388 +639,388 @@
     <t>OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2</t>
   </si>
   <si>
+    <t>1214596734105084</t>
+  </si>
+  <si>
+    <t>OT 4315 ZVN 1-9-63/2</t>
+  </si>
+  <si>
+    <t>check pruebas FAT,OT 4315 ZVN 1-9-63/2</t>
+  </si>
+  <si>
+    <t>1214596734105094</t>
+  </si>
+  <si>
+    <t>1214739697907509</t>
+  </si>
+  <si>
+    <t>1214739697907510</t>
+  </si>
+  <si>
+    <t>1214596734105104</t>
+  </si>
+  <si>
+    <t>Bodega:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recepcion materiales corte laser,Control de calidad corte laser </t>
+  </si>
+  <si>
+    <t>1214596734112602</t>
+  </si>
+  <si>
+    <t>Recepcion materiales corte laser</t>
+  </si>
+  <si>
+    <t>Victor Muñoz</t>
+  </si>
+  <si>
+    <t>victor.munoz@zitron.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bodega:,Control de calidad corte laser </t>
+  </si>
+  <si>
+    <t>1214596734112622</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Control de calidad corte laser </t>
+  </si>
+  <si>
+    <t>Recepcion materiales corte laser,Recepcion Materiales corte plasma</t>
+  </si>
+  <si>
+    <t>OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2,Bodega:,OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2</t>
+  </si>
+  <si>
+    <t>1214596734114879</t>
+  </si>
+  <si>
+    <t>Recepcion Materiales corte plasma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Control de calidad Corte plasma,Control de calidad corte laser </t>
+  </si>
+  <si>
+    <t>1214596624027372</t>
+  </si>
+  <si>
+    <t>Control de calidad Corte plasma</t>
+  </si>
+  <si>
+    <t>OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2</t>
+  </si>
+  <si>
+    <t>1214596624027387</t>
+  </si>
+  <si>
+    <t>Recepcion mecanizado</t>
+  </si>
+  <si>
+    <t>Control de calidad Mecanizado</t>
+  </si>
+  <si>
+    <t>1214596624027530</t>
+  </si>
+  <si>
+    <t>1214596624027545</t>
+  </si>
+  <si>
+    <t>Caldereria:</t>
+  </si>
+  <si>
+    <t>Preparación Materiales,Armado,Control de calidad Armado</t>
+  </si>
+  <si>
+    <t>1214596624027555</t>
+  </si>
+  <si>
+    <t>Preparación Materiales</t>
+  </si>
+  <si>
+    <t>Nicolás Mol</t>
+  </si>
+  <si>
+    <t>nicolas.mol@zitron.com</t>
+  </si>
+  <si>
+    <t>OT2 4307 ZVN 1-9-86/2 ,OT 4315 ZVN 1-9-63/2,OT 4375 - ZVN 1-9-86/2 + TOB + REJ + TIPO A,OT 4376 -ZVN 1-9-63/2 + TOB + REJ + TIPO A,OT 4377-ZVN 1-9-86/2 + TOB + REJ + TPA,OT4378-ZVN 1-9-63/2 + TOB + REJ + 2FAR + TIPO A ,OT 4381 -ZVN 1-9-63/2 + TOB + REJ + TIPO A,ot  4382 -ZVN 1-9-86/2 + TOB+ REJ + TIPO A ,ot  4385 -VENTILADORES 45KCFMx4"CA - ZVN 1-12-37/4,ot  4385 -VENTILADORES 45KCFMx4"CA - ZVN 1-12-37/4,OT 4394 -ZVN 1-9-86/2 + TOB + REJ,OT 4395 -ZVN 1-16-315/4 + TOB + REJ + 2FAR160/200</t>
+  </si>
+  <si>
+    <t>1214596725492919</t>
+  </si>
+  <si>
+    <t>Control de calidad corte laser ,Control de calidad Mecanizado,Control de calidad Corte plasma</t>
+  </si>
+  <si>
+    <t>Preparación Materiales,OT 4315 ZVN 1-9-63/2</t>
+  </si>
+  <si>
+    <t>1214596725514576</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Control de calidad Corte plasma,Control de calidad Mecanizado,Control de calidad corte laser </t>
+  </si>
+  <si>
+    <t>1214739697907430</t>
+  </si>
+  <si>
+    <t>Control de calidad Mecanizado,Control de calidad corte laser ,Control de calidad Corte plasma</t>
+  </si>
+  <si>
+    <t>1214739697907431</t>
+  </si>
+  <si>
+    <t>1214596734023783</t>
+  </si>
+  <si>
+    <t>Armado</t>
+  </si>
+  <si>
+    <t>1214596772418926</t>
+  </si>
+  <si>
+    <t>OT 4315 ZVN 1-9-63/2,check planos</t>
+  </si>
+  <si>
+    <t>Armado,OT 4315 ZVN 1-9-63/2</t>
+  </si>
+  <si>
+    <t>1214596772419042</t>
+  </si>
+  <si>
+    <t>1214739697907432</t>
+  </si>
+  <si>
+    <t>1214739697907433</t>
+  </si>
+  <si>
+    <t>1214596772419062</t>
+  </si>
+  <si>
+    <t>Control de calidad Armado</t>
+  </si>
+  <si>
+    <t>1214596772420232</t>
+  </si>
+  <si>
+    <t>OT 4315 ZVN 1-9-63/2,Control de calidad Armado,Revestimiento</t>
+  </si>
+  <si>
+    <t>1214596772420252</t>
+  </si>
+  <si>
+    <t>1214739697907434</t>
+  </si>
+  <si>
+    <t>OT3 4315 ZVN 1-9-63/2</t>
+  </si>
+  <si>
+    <t>1214739697907435</t>
+  </si>
+  <si>
+    <t>OT4 4315 ZVN 1-9-63/2</t>
+  </si>
+  <si>
+    <t>1214596772422416</t>
+  </si>
+  <si>
+    <t>Recepcion motor,Recepcion Rodete,Recepcion Alabe</t>
+  </si>
+  <si>
+    <t>1214596772422426</t>
+  </si>
+  <si>
+    <t>Recepcion Rodete</t>
+  </si>
+  <si>
+    <t>OT 4315 ZVN 1-9-63/2,Bodega:,OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2</t>
+  </si>
+  <si>
+    <t>1214596772422581</t>
+  </si>
+  <si>
+    <t>Recepcion Alabe</t>
+  </si>
+  <si>
+    <t>Bodega:,OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2</t>
+  </si>
+  <si>
+    <t>1214596772422601</t>
+  </si>
+  <si>
+    <t>Recepcion motor</t>
+  </si>
+  <si>
+    <t>1214596624060758</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recepcion fabricación externa </t>
+  </si>
+  <si>
+    <t>OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2,Revestimiento</t>
+  </si>
+  <si>
+    <t>1214596772424812</t>
+  </si>
+  <si>
+    <t>Montaje:</t>
+  </si>
+  <si>
+    <t>Revestimiento,Montaje motor,Montaje Rodete,RE-PINTADO,Montaje Alabe,Pruebas FAT</t>
+  </si>
+  <si>
+    <t>1214596772424822</t>
+  </si>
+  <si>
+    <t>Revestimiento</t>
+  </si>
+  <si>
+    <t>OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2,Recepcion fabricación externa ,OT3 4315 ZVN 1-9-63/2,OT4 4315 ZVN 1-9-63/2</t>
+  </si>
+  <si>
+    <t>1214596725524470</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OT 4315 ZVN 1-9-63/2,Recepcion fabricación externa </t>
+  </si>
+  <si>
+    <t>1214596725524485</t>
+  </si>
+  <si>
+    <t>1214739697907436</t>
+  </si>
+  <si>
+    <t>OT 4315 ZVN 1-9-63/2,Revestimiento</t>
+  </si>
+  <si>
+    <t>1214739697907437</t>
+  </si>
+  <si>
+    <t>1214596969874290</t>
+  </si>
+  <si>
+    <t>Montaje Alabe</t>
+  </si>
+  <si>
+    <t>1214596969874305</t>
+  </si>
+  <si>
+    <t>Recepcion Alabe,check planos</t>
+  </si>
+  <si>
+    <t>OT 4315 ZVN 1-9-63/2,Montaje Alabe</t>
+  </si>
+  <si>
+    <t>1214596969874389</t>
+  </si>
+  <si>
+    <t>1214739697907438</t>
+  </si>
+  <si>
+    <t>Recepcion Alabe,OT3 4315 ZVN 1-9-63/2,check planos</t>
+  </si>
+  <si>
+    <t>1214739697907439</t>
+  </si>
+  <si>
+    <t>Recepcion Alabe,OT4 4315 ZVN 1-9-63/2,check planos</t>
+  </si>
+  <si>
+    <t>1214596969874409</t>
+  </si>
+  <si>
+    <t>Montaje Rodete</t>
+  </si>
+  <si>
+    <t>1214596772441701</t>
+  </si>
+  <si>
+    <t>OT 4315 ZVN 1-9-63/2,Recepcion Rodete,check planos</t>
+  </si>
+  <si>
+    <t>1214596734152702</t>
+  </si>
+  <si>
+    <t>1214739697907440</t>
+  </si>
+  <si>
+    <t>OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2,Montaje Rodete</t>
+  </si>
+  <si>
+    <t>1214739697907441</t>
+  </si>
+  <si>
+    <t>OT 4315 ZVN 1-9-63/2,check planos,Recepcion Rodete</t>
+  </si>
+  <si>
+    <t>1214596734152727</t>
+  </si>
+  <si>
+    <t>Montaje motor</t>
+  </si>
+  <si>
+    <t>1214596734154011</t>
+  </si>
+  <si>
+    <t>Recepcion motor,check planos</t>
+  </si>
+  <si>
+    <t>OT 4315 ZVN 1-9-63/2,Montaje motor</t>
+  </si>
+  <si>
+    <t>1214596969875021</t>
+  </si>
+  <si>
+    <t>check planos,Recepcion motor</t>
+  </si>
+  <si>
+    <t>1214739697907442</t>
+  </si>
+  <si>
+    <t>OT 4315 ZVN 1-9-63/2,check planos,Recepcion motor</t>
+  </si>
+  <si>
+    <t>1214739697907443</t>
+  </si>
+  <si>
+    <t>OT 4315 ZVN 1-9-63/2,Recepcion motor,check planos</t>
+  </si>
+  <si>
+    <t>1214596969875041</t>
+  </si>
+  <si>
+    <t>Pruebas FAT</t>
+  </si>
+  <si>
+    <t>1214596624084258</t>
+  </si>
+  <si>
+    <t>Pruebas FAT,OT 4315 ZVN 1-9-63/2</t>
+  </si>
+  <si>
+    <t>1214596624084278</t>
+  </si>
+  <si>
+    <t>1214739697907445</t>
+  </si>
+  <si>
+    <t>OT 4315 ZVN 1-9-63/2,Pruebas FAT</t>
+  </si>
+  <si>
+    <t>1214739697907444</t>
+  </si>
+  <si>
+    <t>1214596624029751</t>
+  </si>
+  <si>
+    <t>RE-PINTADO</t>
+  </si>
+  <si>
+    <t>Coordinacion Entrega con Cliente,Montaje:</t>
+  </si>
+  <si>
     <t>Media</t>
-  </si>
-  <si>
-    <t>1214596734105084</t>
-  </si>
-  <si>
-    <t>OT 4315 ZVN 1-9-63/2</t>
-  </si>
-  <si>
-    <t>check pruebas FAT,OT 4315 ZVN 1-9-63/2</t>
-  </si>
-  <si>
-    <t>1214596734105094</t>
-  </si>
-  <si>
-    <t>1214739697907509</t>
-  </si>
-  <si>
-    <t>1214739697907510</t>
-  </si>
-  <si>
-    <t>1214596734105104</t>
-  </si>
-  <si>
-    <t>Bodega:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Recepcion materiales corte laser,Control de calidad corte laser </t>
-  </si>
-  <si>
-    <t>1214596734112602</t>
-  </si>
-  <si>
-    <t>Recepcion materiales corte laser</t>
-  </si>
-  <si>
-    <t>Victor Muñoz</t>
-  </si>
-  <si>
-    <t>victor.munoz@zitron.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bodega:,Control de calidad corte laser </t>
-  </si>
-  <si>
-    <t>1214596734112622</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Control de calidad corte laser </t>
-  </si>
-  <si>
-    <t>Recepcion materiales corte laser,Recepcion Materiales corte plasma</t>
-  </si>
-  <si>
-    <t>OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2,Bodega:,OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2</t>
-  </si>
-  <si>
-    <t>1214596734114879</t>
-  </si>
-  <si>
-    <t>Recepcion Materiales corte plasma</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Control de calidad Corte plasma,Control de calidad corte laser </t>
-  </si>
-  <si>
-    <t>1214596624027372</t>
-  </si>
-  <si>
-    <t>Control de calidad Corte plasma</t>
-  </si>
-  <si>
-    <t>OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2</t>
-  </si>
-  <si>
-    <t>1214596624027387</t>
-  </si>
-  <si>
-    <t>Recepcion mecanizado</t>
-  </si>
-  <si>
-    <t>Control de calidad Mecanizado</t>
-  </si>
-  <si>
-    <t>1214596624027530</t>
-  </si>
-  <si>
-    <t>1214596624027545</t>
-  </si>
-  <si>
-    <t>Caldereria:</t>
-  </si>
-  <si>
-    <t>Preparación Materiales,Armado,Control de calidad Armado</t>
-  </si>
-  <si>
-    <t>1214596624027555</t>
-  </si>
-  <si>
-    <t>Preparación Materiales</t>
-  </si>
-  <si>
-    <t>Nicolás Mol</t>
-  </si>
-  <si>
-    <t>nicolas.mol@zitron.com</t>
-  </si>
-  <si>
-    <t>OT2 4307 ZVN 1-9-86/2 ,OT 4315 ZVN 1-9-63/2,OT 4375 - ZVN 1-9-86/2 + TOB + REJ + TIPO A,OT 4376 -ZVN 1-9-63/2 + TOB + REJ + TIPO A,OT 4377-ZVN 1-9-86/2 + TOB + REJ + TPA,OT4378-ZVN 1-9-63/2 + TOB + REJ + 2FAR + TIPO A ,OT 4381 -ZVN 1-9-63/2 + TOB + REJ + TIPO A,ot  4382 -ZVN 1-9-86/2 + TOB+ REJ + TIPO A ,ot  4385 -VENTILADORES 45KCFMx4"CA - ZVN 1-12-37/4,ot  4385 -VENTILADORES 45KCFMx4"CA - ZVN 1-12-37/4,OT 4394 -ZVN 1-9-86/2 + TOB + REJ,OT 4395 -ZVN 1-16-315/4 + TOB + REJ + 2FAR160/200</t>
-  </si>
-  <si>
-    <t>1214596725492919</t>
-  </si>
-  <si>
-    <t>Control de calidad corte laser ,Control de calidad Mecanizado,Control de calidad Corte plasma</t>
-  </si>
-  <si>
-    <t>Preparación Materiales,OT 4315 ZVN 1-9-63/2</t>
-  </si>
-  <si>
-    <t>1214596725514576</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Control de calidad Corte plasma,Control de calidad Mecanizado,Control de calidad corte laser </t>
-  </si>
-  <si>
-    <t>1214739697907430</t>
-  </si>
-  <si>
-    <t>Control de calidad Mecanizado,Control de calidad corte laser ,Control de calidad Corte plasma</t>
-  </si>
-  <si>
-    <t>1214739697907431</t>
-  </si>
-  <si>
-    <t>1214596734023783</t>
-  </si>
-  <si>
-    <t>Armado</t>
-  </si>
-  <si>
-    <t>1214596772418926</t>
-  </si>
-  <si>
-    <t>OT 4315 ZVN 1-9-63/2,check planos</t>
-  </si>
-  <si>
-    <t>Armado,OT 4315 ZVN 1-9-63/2</t>
-  </si>
-  <si>
-    <t>1214596772419042</t>
-  </si>
-  <si>
-    <t>1214739697907432</t>
-  </si>
-  <si>
-    <t>1214739697907433</t>
-  </si>
-  <si>
-    <t>1214596772419062</t>
-  </si>
-  <si>
-    <t>Control de calidad Armado</t>
-  </si>
-  <si>
-    <t>1214596772420232</t>
-  </si>
-  <si>
-    <t>OT 4315 ZVN 1-9-63/2,Control de calidad Armado,Revestimiento</t>
-  </si>
-  <si>
-    <t>1214596772420252</t>
-  </si>
-  <si>
-    <t>1214739697907434</t>
-  </si>
-  <si>
-    <t>OT3 4315 ZVN 1-9-63/2</t>
-  </si>
-  <si>
-    <t>1214739697907435</t>
-  </si>
-  <si>
-    <t>OT4 4315 ZVN 1-9-63/2</t>
-  </si>
-  <si>
-    <t>1214596772422416</t>
-  </si>
-  <si>
-    <t>Recepcion motor,Recepcion Rodete,Recepcion Alabe</t>
-  </si>
-  <si>
-    <t>1214596772422426</t>
-  </si>
-  <si>
-    <t>Recepcion Rodete</t>
-  </si>
-  <si>
-    <t>OT 4315 ZVN 1-9-63/2,Bodega:,OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2</t>
-  </si>
-  <si>
-    <t>1214596772422581</t>
-  </si>
-  <si>
-    <t>Recepcion Alabe</t>
-  </si>
-  <si>
-    <t>Bodega:,OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2</t>
-  </si>
-  <si>
-    <t>1214596772422601</t>
-  </si>
-  <si>
-    <t>Recepcion motor</t>
-  </si>
-  <si>
-    <t>1214596624060758</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Recepcion fabricación externa </t>
-  </si>
-  <si>
-    <t>OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2,Revestimiento</t>
-  </si>
-  <si>
-    <t>1214596772424812</t>
-  </si>
-  <si>
-    <t>Montaje:</t>
-  </si>
-  <si>
-    <t>Revestimiento,Montaje motor,Montaje Rodete,RE-PINTADO,Montaje Alabe,Pruebas FAT</t>
-  </si>
-  <si>
-    <t>1214596772424822</t>
-  </si>
-  <si>
-    <t>Revestimiento</t>
-  </si>
-  <si>
-    <t>OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2,Recepcion fabricación externa ,OT3 4315 ZVN 1-9-63/2,OT4 4315 ZVN 1-9-63/2</t>
-  </si>
-  <si>
-    <t>1214596725524470</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OT 4315 ZVN 1-9-63/2,Recepcion fabricación externa </t>
-  </si>
-  <si>
-    <t>1214596725524485</t>
-  </si>
-  <si>
-    <t>1214739697907436</t>
-  </si>
-  <si>
-    <t>OT 4315 ZVN 1-9-63/2,Revestimiento</t>
-  </si>
-  <si>
-    <t>1214739697907437</t>
-  </si>
-  <si>
-    <t>1214596969874290</t>
-  </si>
-  <si>
-    <t>Montaje Alabe</t>
-  </si>
-  <si>
-    <t>1214596969874305</t>
-  </si>
-  <si>
-    <t>Recepcion Alabe,check planos</t>
-  </si>
-  <si>
-    <t>OT 4315 ZVN 1-9-63/2,Montaje Alabe</t>
-  </si>
-  <si>
-    <t>1214596969874389</t>
-  </si>
-  <si>
-    <t>1214739697907438</t>
-  </si>
-  <si>
-    <t>Recepcion Alabe,OT3 4315 ZVN 1-9-63/2,check planos</t>
-  </si>
-  <si>
-    <t>1214739697907439</t>
-  </si>
-  <si>
-    <t>Recepcion Alabe,OT4 4315 ZVN 1-9-63/2,check planos</t>
-  </si>
-  <si>
-    <t>1214596969874409</t>
-  </si>
-  <si>
-    <t>Montaje Rodete</t>
-  </si>
-  <si>
-    <t>1214596772441701</t>
-  </si>
-  <si>
-    <t>OT 4315 ZVN 1-9-63/2,Recepcion Rodete,check planos</t>
-  </si>
-  <si>
-    <t>1214596734152702</t>
-  </si>
-  <si>
-    <t>1214739697907440</t>
-  </si>
-  <si>
-    <t>OT 4315 ZVN 1-9-63/2,OT 4315 ZVN 1-9-63/2,Montaje Rodete</t>
-  </si>
-  <si>
-    <t>1214739697907441</t>
-  </si>
-  <si>
-    <t>OT 4315 ZVN 1-9-63/2,check planos,Recepcion Rodete</t>
-  </si>
-  <si>
-    <t>1214596734152727</t>
-  </si>
-  <si>
-    <t>Montaje motor</t>
-  </si>
-  <si>
-    <t>1214596734154011</t>
-  </si>
-  <si>
-    <t>Recepcion motor,check planos</t>
-  </si>
-  <si>
-    <t>OT 4315 ZVN 1-9-63/2,Montaje motor</t>
-  </si>
-  <si>
-    <t>1214596969875021</t>
-  </si>
-  <si>
-    <t>check planos,Recepcion motor</t>
-  </si>
-  <si>
-    <t>1214739697907442</t>
-  </si>
-  <si>
-    <t>OT 4315 ZVN 1-9-63/2,check planos,Recepcion motor</t>
-  </si>
-  <si>
-    <t>1214739697907443</t>
-  </si>
-  <si>
-    <t>OT 4315 ZVN 1-9-63/2,Recepcion motor,check planos</t>
-  </si>
-  <si>
-    <t>1214596969875041</t>
-  </si>
-  <si>
-    <t>Pruebas FAT</t>
-  </si>
-  <si>
-    <t>1214596624084258</t>
-  </si>
-  <si>
-    <t>Pruebas FAT,OT 4315 ZVN 1-9-63/2</t>
-  </si>
-  <si>
-    <t>1214596624084278</t>
-  </si>
-  <si>
-    <t>1214739697907445</t>
-  </si>
-  <si>
-    <t>OT 4315 ZVN 1-9-63/2,Pruebas FAT</t>
-  </si>
-  <si>
-    <t>1214739697907444</t>
-  </si>
-  <si>
-    <t>1214596624029751</t>
-  </si>
-  <si>
-    <t>RE-PINTADO</t>
-  </si>
-  <si>
-    <t>Coordinacion Entrega con Cliente,Montaje:</t>
   </si>
   <si>
     <t>1214596772470213</t>
@@ -4621,7 +4621,7 @@
       </c>
       <c r="C50" s="6"/>
       <c r="D50" s="5">
-        <v>46241.168307569445</v>
+        <v>46242.18436197916</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>185</v>
@@ -4665,8 +4665,8 @@
       <c r="R50" s="5">
         <v>46241</v>
       </c>
-      <c r="S50" s="12" t="s">
-        <v>189</v>
+      <c r="S50" s="11" t="s">
+        <v>33</v>
       </c>
       <c r="T50" s="6">
         <v>0</v>
@@ -4677,7 +4677,7 @@
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" s="8" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B51" s="9">
         <v>46149.168991412036</v>
@@ -4687,7 +4687,7 @@
         <v>46241.16831026621</v>
       </c>
       <c r="E51" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F51" s="10" t="s">
         <v>26</v>
@@ -4715,10 +4715,10 @@
         <v>185</v>
       </c>
       <c r="O51" s="10" t="s">
+        <v>190</v>
+      </c>
+      <c r="P51" s="10" t="s">
         <v>191</v>
-      </c>
-      <c r="P51" s="10" t="s">
-        <v>192</v>
       </c>
       <c r="Q51" s="10"/>
       <c r="R51" s="10"/>
@@ -4728,7 +4728,7 @@
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B52" s="5">
         <v>46149.16900017361</v>
@@ -4738,7 +4738,7 @@
         <v>46241.16831137732</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F52" s="6" t="s">
         <v>26</v>
@@ -4766,10 +4766,10 @@
         <v>185</v>
       </c>
       <c r="O52" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="P52" s="6" t="s">
         <v>191</v>
-      </c>
-      <c r="P52" s="6" t="s">
-        <v>192</v>
       </c>
       <c r="Q52" s="6"/>
       <c r="R52" s="6"/>
@@ -4779,7 +4779,7 @@
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B53" s="9">
         <v>46155.577817384255</v>
@@ -4789,7 +4789,7 @@
         <v>46241.1683981713</v>
       </c>
       <c r="E53" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F53" s="10" t="s">
         <v>26</v>
@@ -4817,10 +4817,10 @@
         <v>185</v>
       </c>
       <c r="O53" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P53" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="Q53" s="10"/>
       <c r="R53" s="10"/>
@@ -4830,7 +4830,7 @@
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B54" s="5">
         <v>46155.577829050926</v>
@@ -4840,7 +4840,7 @@
         <v>46241.1684000463</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F54" s="6" t="s">
         <v>26</v>
@@ -4868,10 +4868,10 @@
         <v>185</v>
       </c>
       <c r="O54" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P54" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="Q54" s="6"/>
       <c r="R54" s="6"/>
@@ -4881,7 +4881,7 @@
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" s="8" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B55" s="9">
         <v>46149.1690050926</v>
@@ -4893,7 +4893,7 @@
         <v>46216.8396287963</v>
       </c>
       <c r="E55" s="10" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F55" s="10" t="s">
         <v>25</v>
@@ -4917,7 +4917,7 @@
         <v>26</v>
       </c>
       <c r="O55" s="10" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="P55" s="10" t="s">
         <v>26</v>
@@ -4934,7 +4934,7 @@
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B56" s="5">
         <v>46149.16900940972</v>
@@ -4946,16 +4946,16 @@
         <v>46216.83970709491</v>
       </c>
       <c r="E56" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="F56" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G56" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="F56" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G56" s="6" t="s">
+      <c r="H56" s="6" t="s">
         <v>201</v>
-      </c>
-      <c r="H56" s="6" t="s">
-        <v>202</v>
       </c>
       <c r="I56" s="5">
         <v>46202</v>
@@ -4973,13 +4973,13 @@
         <v>26</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="O56" s="6" t="s">
         <v>136</v>
       </c>
       <c r="P56" s="6" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="Q56" s="5">
         <v>46202</v>
@@ -4999,7 +4999,7 @@
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A57" s="8" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B57" s="9">
         <v>46149.16901516204</v>
@@ -5011,7 +5011,7 @@
         <v>46216.83978594907</v>
       </c>
       <c r="E57" s="10" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F57" s="10" t="s">
         <v>26</v>
@@ -5038,13 +5038,13 @@
         <v>26</v>
       </c>
       <c r="N57" s="10" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="O57" s="10" t="s">
+        <v>205</v>
+      </c>
+      <c r="P57" s="10" t="s">
         <v>206</v>
-      </c>
-      <c r="P57" s="10" t="s">
-        <v>207</v>
       </c>
       <c r="Q57" s="9">
         <v>46174</v>
@@ -5064,7 +5064,7 @@
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B58" s="5">
         <v>46149.16902107639</v>
@@ -5076,16 +5076,16 @@
         <v>46216.83981521991</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G58" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="H58" s="6" t="s">
         <v>201</v>
-      </c>
-      <c r="H58" s="6" t="s">
-        <v>202</v>
       </c>
       <c r="I58" s="5">
         <v>46202</v>
@@ -5103,13 +5103,13 @@
         <v>26</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="O58" s="6" t="s">
         <v>144</v>
       </c>
       <c r="P58" s="6" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="Q58" s="5">
         <v>46202</v>
@@ -5129,7 +5129,7 @@
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A59" s="8" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B59" s="9">
         <v>46149.16902621528</v>
@@ -5141,7 +5141,7 @@
         <v>46216.83984586806</v>
       </c>
       <c r="E59" s="10" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F59" s="10" t="s">
         <v>26</v>
@@ -5168,13 +5168,13 @@
         <v>26</v>
       </c>
       <c r="N59" s="10" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="O59" s="10" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="P59" s="10" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="Q59" s="9">
         <v>46174</v>
@@ -5194,7 +5194,7 @@
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B60" s="5">
         <v>46149.1690303588</v>
@@ -5206,16 +5206,16 @@
         <v>46216.83987789352</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F60" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G60" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="H60" s="6" t="s">
         <v>201</v>
-      </c>
-      <c r="H60" s="6" t="s">
-        <v>202</v>
       </c>
       <c r="I60" s="5">
         <v>46211</v>
@@ -5233,13 +5233,13 @@
         <v>26</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="O60" s="6" t="s">
         <v>166</v>
       </c>
       <c r="P60" s="6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="Q60" s="5">
         <v>46211</v>
@@ -5259,7 +5259,7 @@
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A61" s="8" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B61" s="9">
         <v>46149.16903488426</v>
@@ -5271,7 +5271,7 @@
         <v>46217.188729456015</v>
       </c>
       <c r="E61" s="10" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F61" s="10" t="s">
         <v>26</v>
@@ -5298,13 +5298,13 @@
         <v>26</v>
       </c>
       <c r="N61" s="10" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="O61" s="10" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P61" s="10" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="Q61" s="9">
         <v>46213</v>
@@ -5324,7 +5324,7 @@
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B62" s="5">
         <v>46149.1690391088</v>
@@ -5334,7 +5334,7 @@
         <v>46224.67388769676</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F62" s="6" t="s">
         <v>25</v>
@@ -5358,7 +5358,7 @@
         <v>26</v>
       </c>
       <c r="O62" s="6" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="P62" s="6" t="s">
         <v>26</v>
@@ -5371,7 +5371,7 @@
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A63" s="8" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B63" s="9">
         <v>46149.169042442125</v>
@@ -5383,16 +5383,16 @@
         <v>46240.582704201384</v>
       </c>
       <c r="E63" s="10" t="s">
+        <v>221</v>
+      </c>
+      <c r="F63" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G63" s="10" t="s">
         <v>222</v>
       </c>
-      <c r="F63" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G63" s="10" t="s">
+      <c r="H63" s="10" t="s">
         <v>223</v>
-      </c>
-      <c r="H63" s="10" t="s">
-        <v>224</v>
       </c>
       <c r="I63" s="9">
         <v>46217</v>
@@ -5410,13 +5410,13 @@
         <v>26</v>
       </c>
       <c r="N63" s="10" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="O63" s="10" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="P63" s="10" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="Q63" s="9">
         <v>46217</v>
@@ -5436,7 +5436,7 @@
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B64" s="5">
         <v>46149.169049375</v>
@@ -5448,16 +5448,16 @@
         <v>46224.673700625004</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F64" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G64" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="H64" s="6" t="s">
         <v>223</v>
-      </c>
-      <c r="H64" s="6" t="s">
-        <v>224</v>
       </c>
       <c r="I64" s="5">
         <v>46217</v>
@@ -5475,13 +5475,13 @@
         <v>26</v>
       </c>
       <c r="N64" s="6" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="O64" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="P64" s="6" t="s">
         <v>227</v>
-      </c>
-      <c r="P64" s="6" t="s">
-        <v>228</v>
       </c>
       <c r="Q64" s="6"/>
       <c r="R64" s="6"/>
@@ -5491,7 +5491,7 @@
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A65" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B65" s="9">
         <v>46149.16905616898</v>
@@ -5503,16 +5503,16 @@
         <v>46224.67370611111</v>
       </c>
       <c r="E65" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F65" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G65" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="H65" s="10" t="s">
         <v>223</v>
-      </c>
-      <c r="H65" s="10" t="s">
-        <v>224</v>
       </c>
       <c r="I65" s="9">
         <v>46217</v>
@@ -5530,13 +5530,13 @@
         <v>26</v>
       </c>
       <c r="N65" s="10" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="O65" s="10" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="P65" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="Q65" s="10"/>
       <c r="R65" s="10"/>
@@ -5546,7 +5546,7 @@
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B66" s="5">
         <v>46155.562074166664</v>
@@ -5558,16 +5558,16 @@
         <v>46224.67371170138</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F66" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G66" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="H66" s="6" t="s">
         <v>223</v>
-      </c>
-      <c r="H66" s="6" t="s">
-        <v>224</v>
       </c>
       <c r="I66" s="5">
         <v>46217</v>
@@ -5585,13 +5585,13 @@
         <v>26</v>
       </c>
       <c r="N66" s="6" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="O66" s="6" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="P66" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="Q66" s="6"/>
       <c r="R66" s="6"/>
@@ -5601,7 +5601,7 @@
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A67" s="8" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B67" s="9">
         <v>46155.562095416666</v>
@@ -5613,16 +5613,16 @@
         <v>46224.67371741898</v>
       </c>
       <c r="E67" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F67" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G67" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="H67" s="10" t="s">
         <v>223</v>
-      </c>
-      <c r="H67" s="10" t="s">
-        <v>224</v>
       </c>
       <c r="I67" s="9">
         <v>46217</v>
@@ -5640,13 +5640,13 @@
         <v>26</v>
       </c>
       <c r="N67" s="10" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="O67" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="P67" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="Q67" s="10"/>
       <c r="R67" s="10"/>
@@ -5656,7 +5656,7 @@
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B68" s="5">
         <v>46149.169104699075</v>
@@ -5668,16 +5668,16 @@
         <v>46227.16954216435</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F68" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G68" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="H68" s="6" t="s">
         <v>223</v>
-      </c>
-      <c r="H68" s="6" t="s">
-        <v>224</v>
       </c>
       <c r="I68" s="5">
         <v>46220</v>
@@ -5695,13 +5695,13 @@
         <v>26</v>
       </c>
       <c r="N68" s="6" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="O68" s="6" t="s">
         <v>188</v>
       </c>
       <c r="P68" s="6" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="Q68" s="5">
         <v>46220</v>
@@ -5721,7 +5721,7 @@
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A69" s="8" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B69" s="9">
         <v>46149.1691096412</v>
@@ -5733,16 +5733,16 @@
         <v>46224.67384578704</v>
       </c>
       <c r="E69" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F69" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G69" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="H69" s="10" t="s">
         <v>223</v>
-      </c>
-      <c r="H69" s="10" t="s">
-        <v>224</v>
       </c>
       <c r="I69" s="9">
         <v>46220</v>
@@ -5760,13 +5760,13 @@
         <v>26</v>
       </c>
       <c r="N69" s="10" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="O69" s="10" t="s">
+        <v>236</v>
+      </c>
+      <c r="P69" s="10" t="s">
         <v>237</v>
-      </c>
-      <c r="P69" s="10" t="s">
-        <v>238</v>
       </c>
       <c r="Q69" s="10"/>
       <c r="R69" s="10"/>
@@ -5776,7 +5776,7 @@
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B70" s="5">
         <v>46149.16911491899</v>
@@ -5788,16 +5788,16 @@
         <v>46224.67385033565</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F70" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G70" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="H70" s="6" t="s">
         <v>223</v>
-      </c>
-      <c r="H70" s="6" t="s">
-        <v>224</v>
       </c>
       <c r="I70" s="5">
         <v>46220</v>
@@ -5815,13 +5815,13 @@
         <v>26</v>
       </c>
       <c r="N70" s="6" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="O70" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="P70" s="6" t="s">
         <v>237</v>
-      </c>
-      <c r="P70" s="6" t="s">
-        <v>238</v>
       </c>
       <c r="Q70" s="6"/>
       <c r="R70" s="6"/>
@@ -5831,7 +5831,7 @@
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71" s="8" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B71" s="9">
         <v>46155.562225625</v>
@@ -5843,16 +5843,16 @@
         <v>46224.67385497685</v>
       </c>
       <c r="E71" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F71" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G71" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="H71" s="10" t="s">
         <v>223</v>
-      </c>
-      <c r="H71" s="10" t="s">
-        <v>224</v>
       </c>
       <c r="I71" s="9">
         <v>46220</v>
@@ -5870,13 +5870,13 @@
         <v>26</v>
       </c>
       <c r="N71" s="10" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="O71" s="10" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="P71" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="Q71" s="10"/>
       <c r="R71" s="10"/>
@@ -5886,7 +5886,7 @@
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B72" s="5">
         <v>46155.56224557871</v>
@@ -5898,16 +5898,16 @@
         <v>46224.67386524305</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F72" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G72" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="H72" s="6" t="s">
         <v>223</v>
-      </c>
-      <c r="H72" s="6" t="s">
-        <v>224</v>
       </c>
       <c r="I72" s="5">
         <v>46220</v>
@@ -5925,13 +5925,13 @@
         <v>26</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="O72" s="6" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="P72" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="Q72" s="6"/>
       <c r="R72" s="6"/>
@@ -5941,7 +5941,7 @@
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A73" s="8" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B73" s="9">
         <v>46149.169119768514</v>
@@ -5951,7 +5951,7 @@
         <v>46228.16710329861</v>
       </c>
       <c r="E73" s="10" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="F73" s="10" t="s">
         <v>26</v>
@@ -5978,13 +5978,13 @@
         <v>26</v>
       </c>
       <c r="N73" s="10" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="O73" s="10" t="s">
         <v>188</v>
       </c>
       <c r="P73" s="10" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="Q73" s="9">
         <v>46227</v>
@@ -6004,7 +6004,7 @@
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B74" s="5">
         <v>46149.16912365741</v>
@@ -6014,7 +6014,7 @@
         <v>46227.16842824074</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F74" s="6" t="s">
         <v>26</v>
@@ -6041,13 +6041,13 @@
         <v>26</v>
       </c>
       <c r="N74" s="6" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="O74" s="6" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="P74" s="6" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="Q74" s="6"/>
       <c r="R74" s="6"/>
@@ -6057,7 +6057,7 @@
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A75" s="8" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B75" s="9">
         <v>46149.16912908565</v>
@@ -6067,7 +6067,7 @@
         <v>46227.16842944444</v>
       </c>
       <c r="E75" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F75" s="10" t="s">
         <v>26</v>
@@ -6094,13 +6094,13 @@
         <v>26</v>
       </c>
       <c r="N75" s="10" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="O75" s="10" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="P75" s="10" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="Q75" s="10"/>
       <c r="R75" s="10"/>
@@ -6110,7 +6110,7 @@
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B76" s="5">
         <v>46155.56233189815</v>
@@ -6120,7 +6120,7 @@
         <v>46227.168525636574</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F76" s="6" t="s">
         <v>26</v>
@@ -6147,13 +6147,13 @@
         <v>26</v>
       </c>
       <c r="N76" s="6" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="O76" s="6" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="P76" s="6" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="Q76" s="6"/>
       <c r="R76" s="6"/>
@@ -6163,7 +6163,7 @@
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77" s="8" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B77" s="9">
         <v>46155.562344351856</v>
@@ -6173,7 +6173,7 @@
         <v>46227.168527118054</v>
       </c>
       <c r="E77" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F77" s="10" t="s">
         <v>26</v>
@@ -6200,13 +6200,13 @@
         <v>26</v>
       </c>
       <c r="N77" s="10" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="O77" s="10" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="P77" s="10" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="Q77" s="10"/>
       <c r="R77" s="10"/>
@@ -6216,7 +6216,7 @@
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B78" s="5">
         <v>46149.16913412037</v>
@@ -6226,7 +6226,7 @@
         <v>46216.87183908565</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F78" s="6" t="s">
         <v>25</v>
@@ -6250,7 +6250,7 @@
         <v>26</v>
       </c>
       <c r="O78" s="6" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="P78" s="6" t="s">
         <v>26</v>
@@ -6265,7 +6265,7 @@
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B79" s="9">
         <v>46149.16913708333</v>
@@ -6277,16 +6277,16 @@
         <v>46212.66505976852</v>
       </c>
       <c r="E79" s="10" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="F79" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G79" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="H79" s="10" t="s">
         <v>201</v>
-      </c>
-      <c r="H79" s="10" t="s">
-        <v>202</v>
       </c>
       <c r="I79" s="10"/>
       <c r="J79" s="9">
@@ -6302,13 +6302,13 @@
         <v>26</v>
       </c>
       <c r="N79" s="10" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="O79" s="10" t="s">
         <v>113</v>
       </c>
       <c r="P79" s="10" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="Q79" s="9">
         <v>46181</v>
@@ -6328,7 +6328,7 @@
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B80" s="5">
         <v>46149.16914224537</v>
@@ -6340,16 +6340,16 @@
         <v>46212.66506702546</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F80" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G80" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="H80" s="6" t="s">
         <v>201</v>
-      </c>
-      <c r="H80" s="6" t="s">
-        <v>202</v>
       </c>
       <c r="I80" s="5">
         <v>46164</v>
@@ -6367,13 +6367,13 @@
         <v>26</v>
       </c>
       <c r="N80" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="O80" s="6" t="s">
         <v>104</v>
       </c>
       <c r="P80" s="6" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="Q80" s="5">
         <v>46164</v>
@@ -6393,7 +6393,7 @@
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81" s="8" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B81" s="9">
         <v>46149.16914733796</v>
@@ -6405,16 +6405,16 @@
         <v>46216.8718724537</v>
       </c>
       <c r="E81" s="10" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F81" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G81" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="H81" s="10" t="s">
         <v>201</v>
-      </c>
-      <c r="H81" s="10" t="s">
-        <v>202</v>
       </c>
       <c r="I81" s="9">
         <v>46197</v>
@@ -6432,13 +6432,13 @@
         <v>26</v>
       </c>
       <c r="N81" s="10" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="O81" s="10" t="s">
         <v>122</v>
       </c>
       <c r="P81" s="10" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="Q81" s="9">
         <v>46197</v>
@@ -6458,7 +6458,7 @@
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B82" s="5">
         <v>46149.16915236111</v>
@@ -6468,16 +6468,16 @@
         <v>46232.203200497686</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F82" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G82" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="H82" s="6" t="s">
         <v>201</v>
-      </c>
-      <c r="H82" s="6" t="s">
-        <v>202</v>
       </c>
       <c r="I82" s="5">
         <v>46231</v>
@@ -6495,13 +6495,13 @@
         <v>26</v>
       </c>
       <c r="N82" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="O82" s="6" t="s">
         <v>154</v>
       </c>
       <c r="P82" s="6" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="Q82" s="5">
         <v>46231</v>
@@ -6521,7 +6521,7 @@
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A83" s="8" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B83" s="9">
         <v>46149.16915732639</v>
@@ -6531,7 +6531,7 @@
         <v>46155.58270766203</v>
       </c>
       <c r="E83" s="10" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="F83" s="10" t="s">
         <v>25</v>
@@ -6555,7 +6555,7 @@
         <v>26</v>
       </c>
       <c r="O83" s="10" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="P83" s="10" t="s">
         <v>26</v>
@@ -6568,7 +6568,7 @@
     </row>
     <row r="84" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A84" s="4" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B84" s="5">
         <v>46149.16916049768</v>
@@ -6578,7 +6578,7 @@
         <v>46237.537617152775</v>
       </c>
       <c r="E84" s="6" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="F84" s="6" t="s">
         <v>26</v>
@@ -6605,13 +6605,13 @@
         <v>26</v>
       </c>
       <c r="N84" s="6" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="O84" s="6" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="P84" s="6" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="Q84" s="5">
         <v>46230</v>
@@ -6631,7 +6631,7 @@
     </row>
     <row r="85" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A85" s="8" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B85" s="9">
         <v>46149.16916685185</v>
@@ -6641,7 +6641,7 @@
         <v>46234.16939539352</v>
       </c>
       <c r="E85" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F85" s="10" t="s">
         <v>26</v>
@@ -6668,10 +6668,10 @@
         <v>26</v>
       </c>
       <c r="N85" s="10" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="O85" s="10" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="P85" s="10" t="s">
         <v>26</v>
@@ -6684,7 +6684,7 @@
     </row>
     <row r="86" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B86" s="5">
         <v>46149.16917037037</v>
@@ -6694,7 +6694,7 @@
         <v>46234.16939739583</v>
       </c>
       <c r="E86" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F86" s="6" t="s">
         <v>26</v>
@@ -6721,10 +6721,10 @@
         <v>26</v>
       </c>
       <c r="N86" s="6" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="O86" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="P86" s="6" t="s">
         <v>26</v>
@@ -6737,7 +6737,7 @@
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A87" s="8" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B87" s="9">
         <v>46155.5624656713</v>
@@ -6747,7 +6747,7 @@
         <v>46234.16952005787</v>
       </c>
       <c r="E87" s="10" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F87" s="10" t="s">
         <v>26</v>
@@ -6774,13 +6774,13 @@
         <v>26</v>
       </c>
       <c r="N87" s="10" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="O87" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P87" s="10" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="Q87" s="10"/>
       <c r="R87" s="10"/>
@@ -6790,7 +6790,7 @@
     </row>
     <row r="88" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B88" s="5">
         <v>46155.562495266204</v>
@@ -6800,7 +6800,7 @@
         <v>46234.16952178241</v>
       </c>
       <c r="E88" s="6" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F88" s="6" t="s">
         <v>26</v>
@@ -6827,13 +6827,13 @@
         <v>26</v>
       </c>
       <c r="N88" s="6" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="O88" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P88" s="6" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="Q88" s="6"/>
       <c r="R88" s="6"/>
@@ -6843,7 +6843,7 @@
     </row>
     <row r="89" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A89" s="8" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B89" s="9">
         <v>46149.16917405093</v>
@@ -6853,7 +6853,7 @@
         <v>46238.20141277778</v>
       </c>
       <c r="E89" s="10" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F89" s="10" t="s">
         <v>26</v>
@@ -6880,13 +6880,13 @@
         <v>26</v>
       </c>
       <c r="N89" s="10" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="O89" s="10" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="P89" s="10" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="Q89" s="9">
         <v>46237</v>
@@ -6906,7 +6906,7 @@
     </row>
     <row r="90" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A90" s="4" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B90" s="5">
         <v>46149.169178321754</v>
@@ -6918,7 +6918,7 @@
         <v>46223.59174438658</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F90" s="6" t="s">
         <v>26</v>
@@ -6943,13 +6943,13 @@
         <v>26</v>
       </c>
       <c r="N90" s="6" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="O90" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="P90" s="6" t="s">
         <v>279</v>
-      </c>
-      <c r="P90" s="6" t="s">
-        <v>280</v>
       </c>
       <c r="Q90" s="6"/>
       <c r="R90" s="6"/>
@@ -6959,7 +6959,7 @@
     </row>
     <row r="91" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A91" s="8" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B91" s="9">
         <v>46149.169183148144</v>
@@ -6971,7 +6971,7 @@
         <v>46223.591741261574</v>
       </c>
       <c r="E91" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F91" s="10" t="s">
         <v>26</v>
@@ -6996,13 +6996,13 @@
         <v>26</v>
       </c>
       <c r="N91" s="10" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="O91" s="10" t="s">
+        <v>278</v>
+      </c>
+      <c r="P91" s="10" t="s">
         <v>279</v>
-      </c>
-      <c r="P91" s="10" t="s">
-        <v>280</v>
       </c>
       <c r="Q91" s="10"/>
       <c r="R91" s="10"/>
@@ -7012,7 +7012,7 @@
     </row>
     <row r="92" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A92" s="4" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B92" s="5">
         <v>46155.56256662037</v>
@@ -7022,7 +7022,7 @@
         <v>46237.16895704861</v>
       </c>
       <c r="E92" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F92" s="6" t="s">
         <v>26</v>
@@ -7047,13 +7047,13 @@
         <v>26</v>
       </c>
       <c r="N92" s="6" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="O92" s="6" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="P92" s="6" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="Q92" s="6"/>
       <c r="R92" s="6"/>
@@ -7063,7 +7063,7 @@
     </row>
     <row r="93" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A93" s="8" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B93" s="9">
         <v>46155.56257849537</v>
@@ -7073,7 +7073,7 @@
         <v>46237.16895965278</v>
       </c>
       <c r="E93" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F93" s="10" t="s">
         <v>26</v>
@@ -7098,13 +7098,13 @@
         <v>26</v>
       </c>
       <c r="N93" s="10" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="O93" s="10" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="P93" s="10" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="Q93" s="10"/>
       <c r="R93" s="10"/>
@@ -7114,7 +7114,7 @@
     </row>
     <row r="94" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A94" s="4" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B94" s="5">
         <v>46149.169187962965</v>
@@ -7124,7 +7124,7 @@
         <v>46239.170314664356</v>
       </c>
       <c r="E94" s="6" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="F94" s="6" t="s">
         <v>26</v>
@@ -7151,13 +7151,13 @@
         <v>26</v>
       </c>
       <c r="N94" s="6" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="O94" s="6" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="P94" s="6" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="Q94" s="5">
         <v>46238</v>
@@ -7177,7 +7177,7 @@
     </row>
     <row r="95" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A95" s="8" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B95" s="9">
         <v>46149.1691919213</v>
@@ -7189,7 +7189,7 @@
         <v>46223.5918337037</v>
       </c>
       <c r="E95" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F95" s="10" t="s">
         <v>26</v>
@@ -7214,13 +7214,13 @@
         <v>26</v>
       </c>
       <c r="N95" s="10" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="O95" s="10" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="P95" s="10" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="Q95" s="10"/>
       <c r="R95" s="10"/>
@@ -7230,7 +7230,7 @@
     </row>
     <row r="96" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A96" s="4" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B96" s="5">
         <v>46149.16919760416</v>
@@ -7242,7 +7242,7 @@
         <v>46223.591830219906</v>
       </c>
       <c r="E96" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F96" s="6" t="s">
         <v>26</v>
@@ -7267,13 +7267,13 @@
         <v>26</v>
       </c>
       <c r="N96" s="6" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="O96" s="6" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="P96" s="6" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="Q96" s="6"/>
       <c r="R96" s="6"/>
@@ -7283,7 +7283,7 @@
     </row>
     <row r="97" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A97" s="8" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B97" s="9">
         <v>46155.562660428244</v>
@@ -7293,7 +7293,7 @@
         <v>46238.16811421297</v>
       </c>
       <c r="E97" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F97" s="10" t="s">
         <v>26</v>
@@ -7318,13 +7318,13 @@
         <v>26</v>
       </c>
       <c r="N97" s="10" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="O97" s="10" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="P97" s="10" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="Q97" s="10"/>
       <c r="R97" s="10"/>
@@ -7334,7 +7334,7 @@
     </row>
     <row r="98" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A98" s="4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B98" s="5">
         <v>46155.56267193287</v>
@@ -7344,7 +7344,7 @@
         <v>46238.16811594907</v>
       </c>
       <c r="E98" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F98" s="6" t="s">
         <v>26</v>
@@ -7369,13 +7369,13 @@
         <v>26</v>
       </c>
       <c r="N98" s="6" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="O98" s="6" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="P98" s="6" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="Q98" s="6"/>
       <c r="R98" s="6"/>
@@ -7385,7 +7385,7 @@
     </row>
     <row r="99" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A99" s="8" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B99" s="9">
         <v>46149.169203125</v>
@@ -7395,7 +7395,7 @@
         <v>46240.170477685184</v>
       </c>
       <c r="E99" s="10" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="F99" s="10" t="s">
         <v>26</v>
@@ -7422,13 +7422,13 @@
         <v>26</v>
       </c>
       <c r="N99" s="10" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="O99" s="10" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="P99" s="10" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="Q99" s="9">
         <v>46239</v>
@@ -7448,7 +7448,7 @@
     </row>
     <row r="100" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A100" s="4" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B100" s="5">
         <v>46149.16920694444</v>
@@ -7458,7 +7458,7 @@
         <v>46239.16802082176</v>
       </c>
       <c r="E100" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F100" s="6" t="s">
         <v>26</v>
@@ -7483,13 +7483,13 @@
         <v>26</v>
       </c>
       <c r="N100" s="6" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="O100" s="6" t="s">
+        <v>297</v>
+      </c>
+      <c r="P100" s="6" t="s">
         <v>298</v>
-      </c>
-      <c r="P100" s="6" t="s">
-        <v>299</v>
       </c>
       <c r="Q100" s="6"/>
       <c r="R100" s="6"/>
@@ -7499,7 +7499,7 @@
     </row>
     <row r="101" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A101" s="8" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B101" s="9">
         <v>46149.16921202546</v>
@@ -7509,7 +7509,7 @@
         <v>46239.16802197917</v>
       </c>
       <c r="E101" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F101" s="10" t="s">
         <v>26</v>
@@ -7534,13 +7534,13 @@
         <v>26</v>
       </c>
       <c r="N101" s="10" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="O101" s="10" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="P101" s="10" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="Q101" s="10"/>
       <c r="R101" s="10"/>
@@ -7550,7 +7550,7 @@
     </row>
     <row r="102" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A102" s="4" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B102" s="5">
         <v>46155.562741851856</v>
@@ -7560,7 +7560,7 @@
         <v>46239.1680906713</v>
       </c>
       <c r="E102" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F102" s="6" t="s">
         <v>26</v>
@@ -7585,13 +7585,13 @@
         <v>26</v>
       </c>
       <c r="N102" s="6" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="O102" s="6" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="P102" s="6" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="Q102" s="6"/>
       <c r="R102" s="6"/>
@@ -7601,7 +7601,7 @@
     </row>
     <row r="103" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A103" s="8" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B103" s="9">
         <v>46155.562755046296</v>
@@ -7611,7 +7611,7 @@
         <v>46239.16809255787</v>
       </c>
       <c r="E103" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F103" s="10" t="s">
         <v>26</v>
@@ -7636,13 +7636,13 @@
         <v>26</v>
       </c>
       <c r="N103" s="10" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="O103" s="10" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="P103" s="10" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="Q103" s="10"/>
       <c r="R103" s="10"/>
@@ -7652,7 +7652,7 @@
     </row>
     <row r="104" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A104" s="4" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B104" s="5">
         <v>46149.16921689815</v>
@@ -7662,7 +7662,7 @@
         <v>46241.20550412037</v>
       </c>
       <c r="E104" s="6" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="F104" s="6" t="s">
         <v>26</v>
@@ -7689,13 +7689,13 @@
         <v>26</v>
       </c>
       <c r="N104" s="6" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="O104" s="6" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="P104" s="6" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="Q104" s="5">
         <v>46240</v>
@@ -7715,7 +7715,7 @@
     </row>
     <row r="105" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A105" s="8" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B105" s="9">
         <v>46149.169220717595</v>
@@ -7725,7 +7725,7 @@
         <v>46240.16781193287</v>
       </c>
       <c r="E105" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F105" s="10" t="s">
         <v>26</v>
@@ -7752,13 +7752,13 @@
         <v>26</v>
       </c>
       <c r="N105" s="10" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="O105" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P105" s="10" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="Q105" s="10"/>
       <c r="R105" s="10"/>
@@ -7768,7 +7768,7 @@
     </row>
     <row r="106" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A106" s="4" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B106" s="5">
         <v>46149.16922577546</v>
@@ -7778,7 +7778,7 @@
         <v>46240.16781346065</v>
       </c>
       <c r="E106" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F106" s="6" t="s">
         <v>26</v>
@@ -7805,13 +7805,13 @@
         <v>26</v>
       </c>
       <c r="N106" s="6" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="O106" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P106" s="6" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="Q106" s="6"/>
       <c r="R106" s="6"/>
@@ -7821,7 +7821,7 @@
     </row>
     <row r="107" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A107" s="8" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B107" s="9">
         <v>46155.56285743056</v>
@@ -7831,7 +7831,7 @@
         <v>46240.167892337966</v>
       </c>
       <c r="E107" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F107" s="10" t="s">
         <v>26</v>
@@ -7858,13 +7858,13 @@
         <v>26</v>
       </c>
       <c r="N107" s="10" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="O107" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P107" s="10" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="Q107" s="10"/>
       <c r="R107" s="10"/>
@@ -7874,7 +7874,7 @@
     </row>
     <row r="108" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A108" s="4" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B108" s="5">
         <v>46155.56284611111</v>
@@ -7884,7 +7884,7 @@
         <v>46240.16789085648</v>
       </c>
       <c r="E108" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F108" s="6" t="s">
         <v>26</v>
@@ -7911,13 +7911,13 @@
         <v>26</v>
       </c>
       <c r="N108" s="6" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="O108" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P108" s="6" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="Q108" s="6"/>
       <c r="R108" s="6"/>
@@ -7927,7 +7927,7 @@
     </row>
     <row r="109" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A109" s="8" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B109" s="9">
         <v>46149.169270370374</v>
@@ -7937,7 +7937,7 @@
         <v>46237.18984681713</v>
       </c>
       <c r="E109" s="10" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F109" s="10" t="s">
         <v>26</v>
@@ -7964,13 +7964,13 @@
         <v>26</v>
       </c>
       <c r="N109" s="10" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="O109" s="10" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="P109" s="10" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="Q109" s="9">
         <v>46244</v>
@@ -7979,7 +7979,7 @@
         <v>46244</v>
       </c>
       <c r="S109" s="12" t="s">
-        <v>189</v>
+        <v>316</v>
       </c>
       <c r="T109" s="10">
         <v>0</v>
@@ -8000,7 +8000,7 @@
         <v>46223.592111550926</v>
       </c>
       <c r="E110" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F110" s="6" t="s">
         <v>26</v>
@@ -8025,10 +8025,10 @@
         <v>26</v>
       </c>
       <c r="N110" s="6" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="O110" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P110" s="6" t="s">
         <v>318</v>
@@ -8051,7 +8051,7 @@
         <v>46223.59211092592</v>
       </c>
       <c r="E111" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F111" s="10" t="s">
         <v>26</v>
@@ -8076,10 +8076,10 @@
         <v>26</v>
       </c>
       <c r="N111" s="10" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="O111" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P111" s="10" t="s">
         <v>318</v>
@@ -8102,7 +8102,7 @@
         <v>46223.59211032407</v>
       </c>
       <c r="E112" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F112" s="6" t="s">
         <v>26</v>
@@ -8127,10 +8127,10 @@
         <v>26</v>
       </c>
       <c r="N112" s="6" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="O112" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P112" s="6" t="s">
         <v>321</v>
@@ -8153,7 +8153,7 @@
         <v>46223.59210969908</v>
       </c>
       <c r="E113" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F113" s="10" t="s">
         <v>26</v>
@@ -8178,10 +8178,10 @@
         <v>26</v>
       </c>
       <c r="N113" s="10" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="O113" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P113" s="10" t="s">
         <v>321</v>
@@ -8291,7 +8291,7 @@
         <v>46245</v>
       </c>
       <c r="S115" s="12" t="s">
-        <v>189</v>
+        <v>316</v>
       </c>
       <c r="T115" s="10">
         <v>0</v>
@@ -8312,7 +8312,7 @@
         <v>46155.60144278935</v>
       </c>
       <c r="E116" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F116" s="6" t="s">
         <v>26</v>
@@ -8340,7 +8340,7 @@
         <v>327</v>
       </c>
       <c r="O116" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P116" s="6" t="s">
         <v>332</v>
@@ -8363,7 +8363,7 @@
         <v>46155.60143921296</v>
       </c>
       <c r="E117" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F117" s="10" t="s">
         <v>26</v>
@@ -8391,7 +8391,7 @@
         <v>327</v>
       </c>
       <c r="O117" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P117" s="10" t="s">
         <v>334</v>
@@ -8414,7 +8414,7 @@
         <v>46155.601436296296</v>
       </c>
       <c r="E118" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F118" s="6" t="s">
         <v>26</v>
@@ -8442,7 +8442,7 @@
         <v>327</v>
       </c>
       <c r="O118" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P118" s="6" t="s">
         <v>334</v>
@@ -8465,7 +8465,7 @@
         <v>46155.60143193287</v>
       </c>
       <c r="E119" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F119" s="10" t="s">
         <v>26</v>
@@ -8493,7 +8493,7 @@
         <v>327</v>
       </c>
       <c r="O119" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P119" s="10" t="s">
         <v>334</v>
@@ -8546,7 +8546,7 @@
         <v>324</v>
       </c>
       <c r="O120" s="6" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="P120" s="6" t="s">
         <v>324</v>
@@ -8558,7 +8558,7 @@
         <v>46246</v>
       </c>
       <c r="S120" s="12" t="s">
-        <v>189</v>
+        <v>316</v>
       </c>
       <c r="T120" s="6">
         <v>0</v>
@@ -8579,7 +8579,7 @@
         <v>46223.592296180555</v>
       </c>
       <c r="E121" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F121" s="10" t="s">
         <v>26</v>
@@ -8609,7 +8609,7 @@
         <v>338</v>
       </c>
       <c r="O121" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P121" s="10" t="s">
         <v>340</v>
@@ -8632,7 +8632,7 @@
         <v>46223.5922953125</v>
       </c>
       <c r="E122" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F122" s="6" t="s">
         <v>26</v>
@@ -8662,7 +8662,7 @@
         <v>338</v>
       </c>
       <c r="O122" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P122" s="6" t="s">
         <v>340</v>
@@ -8685,7 +8685,7 @@
         <v>46223.592294675924</v>
       </c>
       <c r="E123" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F123" s="10" t="s">
         <v>26</v>
@@ -8715,7 +8715,7 @@
         <v>338</v>
       </c>
       <c r="O123" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P123" s="10" t="s">
         <v>343</v>
@@ -8738,7 +8738,7 @@
         <v>46223.592294050926</v>
       </c>
       <c r="E124" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F124" s="6" t="s">
         <v>26</v>
@@ -8768,7 +8768,7 @@
         <v>338</v>
       </c>
       <c r="O124" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P124" s="6" t="s">
         <v>345</v>
@@ -8797,10 +8797,10 @@
         <v>26</v>
       </c>
       <c r="G125" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="H125" s="10" t="s">
         <v>223</v>
-      </c>
-      <c r="H125" s="10" t="s">
-        <v>224</v>
       </c>
       <c r="I125" s="9">
         <v>46247</v>
@@ -8833,7 +8833,7 @@
         <v>46247</v>
       </c>
       <c r="S125" s="12" t="s">
-        <v>189</v>
+        <v>316</v>
       </c>
       <c r="T125" s="10">
         <v>0</v>
@@ -8854,16 +8854,16 @@
         <v>46155.601853796295</v>
       </c>
       <c r="E126" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F126" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G126" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="H126" s="6" t="s">
         <v>223</v>
-      </c>
-      <c r="H126" s="6" t="s">
-        <v>224</v>
       </c>
       <c r="I126" s="6"/>
       <c r="J126" s="5">
@@ -8882,7 +8882,7 @@
         <v>347</v>
       </c>
       <c r="O126" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P126" s="6" t="s">
         <v>350</v>
@@ -8905,16 +8905,16 @@
         <v>46155.60185450231</v>
       </c>
       <c r="E127" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F127" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G127" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="H127" s="10" t="s">
         <v>223</v>
-      </c>
-      <c r="H127" s="10" t="s">
-        <v>224</v>
       </c>
       <c r="I127" s="10"/>
       <c r="J127" s="9">
@@ -8933,7 +8933,7 @@
         <v>347</v>
       </c>
       <c r="O127" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P127" s="10" t="s">
         <v>352</v>
@@ -8956,16 +8956,16 @@
         <v>46155.60185530093</v>
       </c>
       <c r="E128" s="6" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F128" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G128" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="H128" s="6" t="s">
         <v>223</v>
-      </c>
-      <c r="H128" s="6" t="s">
-        <v>224</v>
       </c>
       <c r="I128" s="6"/>
       <c r="J128" s="5">
@@ -8984,7 +8984,7 @@
         <v>347</v>
       </c>
       <c r="O128" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P128" s="6" t="s">
         <v>354</v>
@@ -9007,16 +9007,16 @@
         <v>46155.60185603009</v>
       </c>
       <c r="E129" s="10" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F129" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G129" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="H129" s="10" t="s">
         <v>223</v>
-      </c>
-      <c r="H129" s="10" t="s">
-        <v>224</v>
       </c>
       <c r="I129" s="10"/>
       <c r="J129" s="9">
@@ -9035,7 +9035,7 @@
         <v>347</v>
       </c>
       <c r="O129" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P129" s="10" t="s">
         <v>356</v>
@@ -9064,10 +9064,10 @@
         <v>26</v>
       </c>
       <c r="G130" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="H130" s="6" t="s">
         <v>223</v>
-      </c>
-      <c r="H130" s="6" t="s">
-        <v>224</v>
       </c>
       <c r="I130" s="5">
         <v>46248</v>
@@ -9100,7 +9100,7 @@
         <v>46248</v>
       </c>
       <c r="S130" s="12" t="s">
-        <v>189</v>
+        <v>316</v>
       </c>
       <c r="T130" s="6">
         <v>0</v>
@@ -9121,16 +9121,16 @@
         <v>46155.602132280095</v>
       </c>
       <c r="E131" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F131" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G131" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="H131" s="10" t="s">
         <v>223</v>
-      </c>
-      <c r="H131" s="10" t="s">
-        <v>224</v>
       </c>
       <c r="I131" s="10"/>
       <c r="J131" s="9">
@@ -9149,7 +9149,7 @@
         <v>358</v>
       </c>
       <c r="O131" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P131" s="10" t="s">
         <v>358</v>
@@ -9172,16 +9172,16 @@
         <v>46155.602128969906</v>
       </c>
       <c r="E132" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F132" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G132" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="H132" s="6" t="s">
         <v>223</v>
-      </c>
-      <c r="H132" s="6" t="s">
-        <v>224</v>
       </c>
       <c r="I132" s="6"/>
       <c r="J132" s="5">
@@ -9200,7 +9200,7 @@
         <v>358</v>
       </c>
       <c r="O132" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P132" s="6" t="s">
         <v>358</v>
@@ -9223,16 +9223,16 @@
         <v>46155.60212502315</v>
       </c>
       <c r="E133" s="10" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F133" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G133" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="H133" s="10" t="s">
         <v>223</v>
-      </c>
-      <c r="H133" s="10" t="s">
-        <v>224</v>
       </c>
       <c r="I133" s="10"/>
       <c r="J133" s="9">
@@ -9251,7 +9251,7 @@
         <v>358</v>
       </c>
       <c r="O133" s="10" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="P133" s="10" t="s">
         <v>358</v>
@@ -9274,16 +9274,16 @@
         <v>46155.602120462965</v>
       </c>
       <c r="E134" s="6" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F134" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G134" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="H134" s="6" t="s">
         <v>223</v>
-      </c>
-      <c r="H134" s="6" t="s">
-        <v>224</v>
       </c>
       <c r="I134" s="6"/>
       <c r="J134" s="5">
@@ -9302,7 +9302,7 @@
         <v>358</v>
       </c>
       <c r="O134" s="6" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="P134" s="6" t="s">
         <v>358</v>

</xml_diff>